<commit_message>
Synchronize Vesperfall 0.12 planning workbook and 76-task roadmap; preserve cross-chat requirements, shipped-vs-draft audit and actual test evidence
</commit_message>
<xml_diff>
--- a/vesperfall/AAA-PRODUCTION.xlsx
+++ b/vesperfall/AAA-PRODUCTION.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="R5422c9ec86e54f0d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="2" r:id="R55a7ea2099fa4869"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Milestones" sheetId="3" r:id="R4b608d0afcc44efb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Device QA" sheetId="4" r:id="R78d077327f794c7e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="5" r:id="R9b625fbc4c40465a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risk Register" sheetId="6" r:id="R0317debfb8b54e62"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="R242c3143bbe74260"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="2" r:id="R59926fb31b304cee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Milestones" sheetId="3" r:id="R006124efab6c4c9c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Device QA" sheetId="4" r:id="R4ba785b8f0b94f51"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="5" r:id="R00e8525b5cfb4e32"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risk Register" sheetId="6" r:id="Re505e8c2936744b2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -22,7 +22,7 @@
     <x:numFmt numFmtId="200" formatCode="0"/>
     <x:numFmt numFmtId="201" formatCode="yyyy-mm-dd"/>
   </x:numFmts>
-  <x:fonts count="8">
+  <x:fonts count="11">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -67,8 +67,24 @@
       <x:color rgb="FF203441"/>
       <x:name val="Calibri"/>
     </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF176B68"/>
+      <x:name val="Calibri"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF243B47"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="5">
+  <x:fills count="8">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -90,6 +106,21 @@
         <x:fgColor rgb="FF176F68"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF176B68"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEFF4F4"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="2">
     <x:border/>
@@ -98,7 +129,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="35">
+  <x:cellXfs count="48">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -195,6 +226,31 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -294,7 +350,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="DeviceMatrix" displayName="DeviceMatrix" ref="A5:J15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="DeviceMatrix" displayName="DeviceMatrix" ref="A5:J17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Device / mode"/>
@@ -328,7 +384,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="ProductionRisks" displayName="ProductionRisks" ref="A5:H15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="ProductionRisks" displayName="ProductionRisks" ref="A5:H17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Risk"/>
@@ -572,7 +628,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="12" t="str">
-        <x:v>v0.11.0 / Rosefire / 2026-09-12. Original gothic shaders extend the existing First Bell game. AAA-level finish remains a quality-gated aspiration, not a hardware certificate.</x:v>
+        <x:v>v0.12.0 / Tidelight / planning audit 2026-09-13. Roadmap, workbook and core diagnostic version labels are synchronized; gameplay mechanics and save formats are unchanged.</x:v>
       </x:c>
       <x:c r="B3" s="12"/>
       <x:c r="C3" s="12"/>
@@ -628,7 +684,7 @@
       <x:c r="B7" s="28"/>
       <x:c r="C7" s="28" t="n">
         <x:f>COUNTIF(Backlog!C6:C81,"Implemented")</x:f>
-        <x:v>35</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="D7" s="28"/>
       <x:c r="E7" s="28" t="n">
@@ -718,7 +774,7 @@
     </x:row>
     <x:row r="15" ht="24" customHeight="1">
       <x:c r="A15" s="6" t="str">
-        <x:v>This release adds ten guided archery lessons and the optional Bellkeeper Oath: three connected encounters, a three-phase boss, recovery beats and saved continuation. V49-V52 and V76 remain Partial until their broader human, hardware and production gates are met.</x:v>
+        <x:v>Shipped water is the bounded translucent-plane baseline. The earlier detailed basin/refraction/reflection/audio draft is not the published implementation. Read the continuation audit before promising or recovering those features.</x:v>
       </x:c>
       <x:c r="B15" s="6"/>
       <x:c r="C15" s="6"/>
@@ -782,7 +838,7 @@
     </x:row>
     <x:row r="21" ht="24" customHeight="1">
       <x:c r="A21" s="6" t="str">
-        <x:v>Before production release, close measured Quest performance, actual controller lifecycle/comfort, long-session sound, finished assets, external playtesting, save migration, content completeness and blocking-defect gates.</x:v>
+        <x:v>Next: establish Tidelight browser/render/save evidence, close Quest water-menu and lifecycle gaps, then prioritize the requested sound/music pass and purposeful exploration. Keep all physical-device and human gates open until measured.</x:v>
       </x:c>
       <x:c r="B21" s="6"/>
       <x:c r="C21" s="6"/>
@@ -814,7 +870,7 @@
     </x:row>
     <x:row r="24" ht="24" customHeight="1">
       <x:c r="A24" s="6" t="str">
-        <x:v>There are no invented delivery dates, staffing commitments or cost estimates. Owner roles require assignment. Physical-device targets and proposed test-batch sizes are planning inputs to verify, not current results.</x:v>
+        <x:v>Historical acceptance: 148 model passes, 1 stale-plan failure; browser steps skipped. Fresh planning checks are separate. No invented hardware approval, staffing, dates, budget, playtime or AAA rating is included.</x:v>
       </x:c>
       <x:c r="B24" s="6"/>
       <x:c r="C24" s="6"/>
@@ -846,7 +902,7 @@
     </x:row>
     <x:row r="27" ht="24" customHeight="1">
       <x:c r="A27" s="34" t="str">
-        <x:v>Canonical JSON SHA-256: e5fa1d8a3476502e514485305e19f4095f419ce8d165203fec6301028488fa8c</x:v>
+        <x:v>Canonical JSON SHA-256: 8d31f942c3913354082adef2f0034cedd120b367a19964acaf3186feecc77a98</x:v>
       </x:c>
       <x:c r="B27" s="34"/>
       <x:c r="C27" s="34"/>
@@ -867,50 +923,52 @@
       <x:c r="H28" s="6"/>
     </x:row>
     <x:row r="29" ht="24" customHeight="1">
-      <x:c r="A29" s="6" t="str">
+      <x:c r="A29" s="36" t="str">
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
       </x:c>
-      <x:c r="B29" s="6"/>
-      <x:c r="C29" s="6"/>
-      <x:c r="D29" s="6"/>
-      <x:c r="E29" s="6"/>
-      <x:c r="F29" s="6"/>
-      <x:c r="G29" s="6"/>
-      <x:c r="H29" s="6"/>
+      <x:c r="B29" s="36"/>
+      <x:c r="C29" s="36"/>
+      <x:c r="D29" s="36"/>
+      <x:c r="E29" s="36"/>
+      <x:c r="F29" s="36"/>
+      <x:c r="G29" s="36"/>
+      <x:c r="H29" s="36"/>
     </x:row>
     <x:row r="30" ht="24" customHeight="1">
-      <x:c r="A30" s="6" t="str">
+      <x:c r="A30" s="36" t="str">
         <x:v>https://v5ma.github.io/vesperfall/roadmap.html</x:v>
       </x:c>
-      <x:c r="B30" s="6"/>
-      <x:c r="C30" s="6"/>
-      <x:c r="D30" s="6"/>
-      <x:c r="E30" s="6"/>
-      <x:c r="F30" s="6"/>
-      <x:c r="G30" s="6"/>
-      <x:c r="H30" s="6"/>
+      <x:c r="B30" s="36"/>
+      <x:c r="C30" s="36"/>
+      <x:c r="D30" s="36"/>
+      <x:c r="E30" s="36"/>
+      <x:c r="F30" s="36"/>
+      <x:c r="G30" s="36"/>
+      <x:c r="H30" s="36"/>
     </x:row>
     <x:row r="31" ht="24" customHeight="1">
-      <x:c r="A31" s="6" t="str">
-        <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/AAA-ROADMAP.md</x:v>
-      </x:c>
-      <x:c r="B31" s="6"/>
-      <x:c r="C31" s="6"/>
-      <x:c r="D31" s="6"/>
-      <x:c r="E31" s="6"/>
-      <x:c r="F31" s="6"/>
-      <x:c r="G31" s="6"/>
-      <x:c r="H31" s="6"/>
+      <x:c r="A31" s="36" t="str">
+        <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/DEVELOPMENT-HANDOFF.md</x:v>
+      </x:c>
+      <x:c r="B31" s="36"/>
+      <x:c r="C31" s="36"/>
+      <x:c r="D31" s="36"/>
+      <x:c r="E31" s="36"/>
+      <x:c r="F31" s="36"/>
+      <x:c r="G31" s="36"/>
+      <x:c r="H31" s="36"/>
     </x:row>
     <x:row r="32" ht="24" customHeight="1">
-      <x:c r="A32" s="6"/>
-      <x:c r="B32" s="6"/>
-      <x:c r="C32" s="6"/>
-      <x:c r="D32" s="6"/>
-      <x:c r="E32" s="6"/>
-      <x:c r="F32" s="6"/>
-      <x:c r="G32" s="6"/>
-      <x:c r="H32" s="6"/>
+      <x:c r="A32" s="36" t="str">
+        <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/CONTINUATION-AUDIT.md</x:v>
+      </x:c>
+      <x:c r="B32" s="36"/>
+      <x:c r="C32" s="36"/>
+      <x:c r="D32" s="36"/>
+      <x:c r="E32" s="36"/>
+      <x:c r="F32" s="36"/>
+      <x:c r="G32" s="36"/>
+      <x:c r="H32" s="36"/>
     </x:row>
     <x:row r="33" ht="24" customHeight="1">
       <x:c r="A33" s="6"/>
@@ -921,6 +979,78 @@
       <x:c r="F33" s="6"/>
       <x:c r="G33" s="6"/>
       <x:c r="H33" s="6"/>
+    </x:row>
+    <x:row r="34" ht="26" customHeight="1">
+      <x:c r="A34" s="38" t="str">
+        <x:v>RESUME WITH THESE EXISTING TASKS</x:v>
+      </x:c>
+      <x:c r="B34" s="38"/>
+      <x:c r="C34" s="38"/>
+      <x:c r="D34" s="38"/>
+      <x:c r="E34" s="38"/>
+      <x:c r="F34" s="38"/>
+      <x:c r="G34" s="38"/>
+      <x:c r="H34" s="38"/>
+    </x:row>
+    <x:row r="36" ht="46" customHeight="1">
+      <x:c r="A36" s="42" t="str">
+        <x:v>V68 / V66: verify the actual 0.12 baseline. Do not treat a successful Pages build, a draft test count or historical Rosefire tests as Tidelight gameplay acceptance.</x:v>
+      </x:c>
+      <x:c r="B36" s="42"/>
+      <x:c r="C36" s="42"/>
+      <x:c r="D36" s="42"/>
+      <x:c r="E36" s="42"/>
+      <x:c r="F36" s="42"/>
+      <x:c r="G36" s="42"/>
+      <x:c r="H36" s="42"/>
+    </x:row>
+    <x:row r="37" ht="46" customHeight="1">
+      <x:c r="A37" s="46" t="str">
+        <x:v>V41 / V61 / V74: finish Quest water settings and verify all Xbox/Quest open, adjust, select, dismiss and recovery paths. Reproduce water footprint, height, ripple-budget and world-clock gaps.</x:v>
+      </x:c>
+      <x:c r="B37" s="46"/>
+      <x:c r="C37" s="46"/>
+      <x:c r="D37" s="46"/>
+      <x:c r="E37" s="46"/>
+      <x:c r="F37" s="46"/>
+      <x:c r="G37" s="46"/>
+      <x:c r="H37" s="46"/>
+    </x:row>
+    <x:row r="38" ht="46" customHeight="1">
+      <x:c r="A38" s="42" t="str">
+        <x:v>V58 / V44: implement water-specific sound, stronger archery/shield/enemy audio and musical transitions. Preserve independent volume buses, mute, captions and warning clarity.</x:v>
+      </x:c>
+      <x:c r="B38" s="42"/>
+      <x:c r="C38" s="42"/>
+      <x:c r="D38" s="42"/>
+      <x:c r="E38" s="42"/>
+      <x:c r="F38" s="42"/>
+      <x:c r="G38" s="42"/>
+      <x:c r="H38" s="42"/>
+    </x:row>
+    <x:row r="39" ht="46" customHeight="1">
+      <x:c r="A39" s="46" t="str">
+        <x:v>V35 / V52 / V54: pursue memorable routes, water destinations and humanoid animation; retain the existing 15 enemy archetypes, First Bell and Bellkeeper Oath.</x:v>
+      </x:c>
+      <x:c r="B39" s="46"/>
+      <x:c r="C39" s="46"/>
+      <x:c r="D39" s="46"/>
+      <x:c r="E39" s="46"/>
+      <x:c r="F39" s="46"/>
+      <x:c r="G39" s="46"/>
+      <x:c r="H39" s="46"/>
+    </x:row>
+    <x:row r="40" ht="46" customHeight="1">
+      <x:c r="A40" s="42" t="str">
+        <x:v>V38 / V59 / V62 / V75: run actual-device comfort, thermal, performance, controller and save-lifecycle checks. Proposed timing budgets are not measurements.</x:v>
+      </x:c>
+      <x:c r="B40" s="42"/>
+      <x:c r="C40" s="42"/>
+      <x:c r="D40" s="42"/>
+      <x:c r="E40" s="42"/>
+      <x:c r="F40" s="42"/>
+      <x:c r="G40" s="42"/>
+      <x:c r="H40" s="42"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -944,6 +1074,13 @@
     <x:mergeCell ref="A29:H29"/>
     <x:mergeCell ref="A30:H30"/>
     <x:mergeCell ref="A31:H31"/>
+    <x:mergeCell ref="A32:H32"/>
+    <x:mergeCell ref="A34:H34"/>
+    <x:mergeCell ref="A36:H36"/>
+    <x:mergeCell ref="A37:H37"/>
+    <x:mergeCell ref="A38:H38"/>
+    <x:mergeCell ref="A39:H39"/>
+    <x:mergeCell ref="A40:H40"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -1005,7 +1142,7 @@
     </x:row>
     <x:row r="3" ht="36" customHeight="1">
       <x:c r="A3" s="12" t="str">
-        <x:v>Canonical snapshot v0.9.0 | 76 retained and new tasks | Status is not AAA certification. Filter any column; edit locally and reconcile with roadmap.json before committing.</x:v>
+        <x:v>v0.12.0 / 76 preserved tasks / September 13 source audit. Partial means the expanded acceptance scope remains open.</x:v>
       </x:c>
       <x:c r="B3" s="12"/>
       <x:c r="C3" s="12"/>
@@ -2543,12 +2680,12 @@
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
       </x:c>
     </x:row>
-    <x:row r="40" ht="124" customHeight="1">
+    <x:row r="40" ht="120" customHeight="1">
       <x:c r="A40" s="6" t="str">
         <x:v>V35</x:v>
       </x:c>
       <x:c r="B40" s="6" t="str">
-        <x:v>Authored crypt/roof transitions and expanded graph vocabulary</x:v>
+        <x:v>Authored crypt, roof and water destinations with expanded route grammar</x:v>
       </x:c>
       <x:c r="C40" s="6" t="str">
         <x:v>Partial</x:v>
@@ -2569,19 +2706,24 @@
         <x:v>None</x:v>
       </x:c>
       <x:c r="I40" s="6" t="str">
-        <x:v>Preserve the established game while closing the stated acceptance gate.</x:v>
+        <x:v>More areas should create memorable choices and reasons to explore, not repeat one room or flood every courtyard.</x:v>
       </x:c>
       <x:c r="J40" s="6" t="str">
-        <x:v>25-district graph expansion shipped. Distinct authored crypt-to-roof transitions and stronger route grammar still need design and native traversal evidence.</x:v>
+        <x:v>Keep the existing 25-district game and reversible upper/lower routes. Add distinctive, collision-tested destinations, escape paths and discoveries. Tidelight water remains decorative until a separately designed, save-compatible traversal feature is approved.</x:v>
       </x:c>
       <x:c r="K40" s="6" t="str">
-        <x:v>Expanded graph implemented; authored transition production remains open.</x:v>
+        <x:v>Partial. Tidelight 0.12.0 water exists in current source. The earlier seven-surface/four-named-district draft, recessed fonts, refracting tile basins and architecture reflections are not established by the shipped implementation.</x:v>
       </x:c>
       <x:c r="L40" s="6" t="str">
         <x:v>dominions-world.js
-HOLLOW-DOMINIONS.md</x:v>
-      </x:c>
-      <x:c r="M40" s="6" t="str"/>
+HOLLOW-DOMINIONS.md
+TIDELIGHT.md
+tidelight.js
+CONTINUATION-AUDIT.md</x:v>
+      </x:c>
+      <x:c r="M40" s="6" t="str">
+        <x:v>0.12.0 Tidelight presentation baseline; authored expansion open</x:v>
+      </x:c>
       <x:c r="N40" s="6" t="str">
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/dominions-world.js</x:v>
       </x:c>
@@ -2675,12 +2817,12 @@
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
       </x:c>
     </x:row>
-    <x:row r="43" ht="124" customHeight="1">
+    <x:row r="43" ht="106" customHeight="1">
       <x:c r="A43" s="6" t="str">
         <x:v>V38</x:v>
       </x:c>
       <x:c r="B43" s="6" t="str">
-        <x:v>Measure physical Quest 3 stereo frame times for Jewelglass and Rosefire</x:v>
+        <x:v>Measure physical Quest 3 stereo frame times for Jewelglass, Rosefire and Tidelight</x:v>
       </x:c>
       <x:c r="C43" s="6" t="str">
         <x:v>Hardware QA</x:v>
@@ -2695,7 +2837,7 @@
         <x:v>Hardware</x:v>
       </x:c>
       <x:c r="G43" s="6" t="str">
-        <x:v>Device QA</x:v>
+        <x:v>Device QA / assignment pending</x:v>
       </x:c>
       <x:c r="H43" s="6" t="str">
         <x:v>None</x:v>
@@ -2704,17 +2846,19 @@
         <x:v>A software fixture cannot tell us how a person feels or how a real device sustains the experience.</x:v>
       </x:c>
       <x:c r="J43" s="6" t="str">
-        <x:v>Measure on device; never infer FPS, comfort or controller alignment from headless emulation.</x:v>
+        <x:v>Measure both eyes, bow/ward visibility, water/caustic legibility and sustained frame times on Quest 3 in both handedness modes. Check reduced effects and AR exclusions. Do not infer hardware FPS, comfort or alignment from emulation.</x:v>
       </x:c>
       <x:c r="K43" s="6" t="str">
         <x:v>No physical device receipt yet.</x:v>
       </x:c>
       <x:c r="L43" s="6" t="str">
-        <x:v>ROSEFIRE.md</x:v>
+        <x:v>ROSEFIRE.md
+TIDELIGHT.md
+CONTINUATION-AUDIT.md</x:v>
       </x:c>
       <x:c r="M43" s="6" t="str"/>
       <x:c r="N43" s="6" t="str">
-        <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
+        <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/ROSEFIRE.md</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="124" customHeight="1">
@@ -2808,7 +2952,7 @@
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/bestiary.js</x:v>
       </x:c>
     </x:row>
-    <x:row r="46" ht="124" customHeight="1">
+    <x:row r="46" ht="134" customHeight="1">
       <x:c r="A46" s="6" t="str">
         <x:v>V41</x:v>
       </x:c>
@@ -2816,7 +2960,7 @@
         <x:v>Xbox focus navigation and paginated Quest spatial menus</x:v>
       </x:c>
       <x:c r="C46" s="6" t="str">
-        <x:v>Implemented</x:v>
+        <x:v>Partial</x:v>
       </x:c>
       <x:c r="D46" s="6" t="str">
         <x:v>P0</x:v>
@@ -2837,14 +2981,16 @@
         <x:v>Avoid forced mouse use or headset removal.</x:v>
       </x:c>
       <x:c r="J46" s="6" t="str">
-        <x:v>Gameplay, settings, seeds, equipment, journal and in-game dialogs can be operated with controller input. System permission prompts are not game-owned.</x:v>
+        <x:v>Every gameplay and game-owned UI path, including water settings, confirmations, recovery, seed entry, audio and accessibility settings, is reachable and dismissible with Xbox and Quest controls without a mouse. Test both handedness modes, neutral-input transitions and return focus. Browser/system permission prompts remain platform-owned.</x:v>
       </x:c>
       <x:c r="K46" s="6" t="str">
-        <x:v>Software release evidence; hardware and human gates remain separate.</x:v>
+        <x:v>Existing Xbox focus and Quest spatial menus are implemented. Current Tidelight adds browser DOM controls but its IDs are absent from the Quest settings list in dominion-controls.js. Full water-settings and close/back parity remains open; historical controller tests do not cover those new controls.</x:v>
       </x:c>
       <x:c r="L46" s="6" t="str">
         <x:v>dominion-controls.js
-tests/dominions-browser.py</x:v>
+tests/dominions-browser.py
+tidelight.js
+CONTINUATION-AUDIT.md</x:v>
       </x:c>
       <x:c r="M46" s="6" t="str">
         <x:v>0.7.0</x:v>
@@ -3128,12 +3274,12 @@
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/pilgrim-save.js</x:v>
       </x:c>
     </x:row>
-    <x:row r="53" ht="124" customHeight="1">
+    <x:row r="53" ht="134" customHeight="1">
       <x:c r="A53" s="6" t="str">
         <x:v>V48</x:v>
       </x:c>
       <x:c r="B53" s="6" t="str">
-        <x:v>Versioned production board and six-sheet workbook</x:v>
+        <x:v>Synchronized canonical production board, six-sheet workbook and cross-chat handoff</x:v>
       </x:c>
       <x:c r="C53" s="6" t="str">
         <x:v>Implemented</x:v>
@@ -3157,20 +3303,22 @@
         <x:v>Make each release close a measurable gap and keep the long-term path inspectable.</x:v>
       </x:c>
       <x:c r="J53" s="6" t="str">
-        <x:v>roadmap.json is canonical; board and workbook show priority, dependencies, owner role, evidence and exit gates. Local edits are clearly separate from committed status.</x:v>
+        <x:v>Keep roadmap.json version aligned with release.json and core.js. Preserve V01-V76; export the six-sheet workbook with matching source digest and live summary formulas. Keep DEVELOPMENT-HANDOFF.md and CONTINUATION-AUDIT.md linked from the board and README. Verify committed files, not browser-local edits.</x:v>
       </x:c>
       <x:c r="K53" s="6" t="str">
-        <x:v>Software release evidence; hardware and human gates remain separate.</x:v>
+        <x:v>September 13 repairs both the stale plan/workbook and the core diagnostic version label, without changing mechanics or save formats. Historical acceptance had 148 model passes and one plan-version failure; fresh checks are recorded separately. Physical/human gates remain open.</x:v>
       </x:c>
       <x:c r="L53" s="6" t="str">
         <x:v>roadmap.json
 roadmap.html
 AAA-PRODUCTION.xlsx
 tests/production.test.cjs
-tests/production-browser.py</x:v>
+tests/production-browser.py
+DEVELOPMENT-HANDOFF.md
+CONTINUATION-AUDIT.md</x:v>
       </x:c>
       <x:c r="M53" s="6" t="str">
-        <x:v>0.9.0</x:v>
+        <x:v>0.9.0 foundation; 0.12.0 planning synchronization</x:v>
       </x:c>
       <x:c r="N53" s="6" t="str">
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
@@ -3314,7 +3462,7 @@
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/oath-model.js</x:v>
       </x:c>
     </x:row>
-    <x:row r="57" ht="124" customHeight="1">
+    <x:row r="57" ht="162" customHeight="1">
       <x:c r="A57" s="6" t="str">
         <x:v>V52</x:v>
       </x:c>
@@ -3343,7 +3491,7 @@
         <x:v>Replace sheer room count with deliberately paced exploration.</x:v>
       </x:c>
       <x:c r="J57" s="6" t="str">
-        <x:v>One polished 20-30 minute target route mixes safe introduction, alternate approach, escalating encounter, discovery and boss payoff. Validate every traversal connector and recovery path. Duration is a design target, not measured content.</x:v>
+        <x:v>One polished 20-30 minute target route mixes safe introduction, alternate approach, escalating encounter, discovery and boss payoff. Validate every traversal connector and recovery path. Duration is a design target, not measured content. Preserve multi-level gothic sightlines and multiple approaches. Plan selective water-adjacent discoveries with purpose; the present water layer does not create new navigable rooms.</x:v>
       </x:c>
       <x:c r="K57" s="6" t="str">
         <x:v>A connected Roseglass/Ivory Crown/Ember Crown progression reuses the collision-tested 25-room world, existing stairs and alternate approaches. Three staged courts are implemented; the proposed 20-30 minute polished duration and authored connector variety are not yet measured or complete.</x:v>
@@ -3351,7 +3499,8 @@
       <x:c r="L57" s="6" t="str">
         <x:v>oath-model.js
 first-bell.js
-tests/oath.test.cjs</x:v>
+tests/oath.test.cjs
+CONTINUATION-AUDIT.md</x:v>
       </x:c>
       <x:c r="M57" s="6" t="str">
         <x:v>0.10.0 First Bell</x:v>
@@ -3400,7 +3549,7 @@
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
       </x:c>
     </x:row>
-    <x:row r="59" ht="124" customHeight="1">
+    <x:row r="59" ht="162" customHeight="1">
       <x:c r="A59" s="6" t="str">
         <x:v>V54</x:v>
       </x:c>
@@ -3429,15 +3578,17 @@
         <x:v>Foreground and character quality must catch up with the architecture.</x:v>
       </x:c>
       <x:c r="J59" s="6" t="str">
-        <x:v>Produce consistent original/licensed meshes, LODs, rigs and materials for one complete vertical slice; registered provenance; review both eye views and close-range silhouette.</x:v>
+        <x:v>Produce consistent original/licensed meshes, LODs, rigs and materials for one complete vertical slice; registered provenance; review both eye views and close-range silhouette. Retain the 15 existing archetypes, including the 12 added outer enemy orders. Improve humanoid/knight silhouettes and counterplay; do not restart the already delivered numerical expansion or copy commercial reference assets.</x:v>
       </x:c>
       <x:c r="K59" s="6" t="str">
         <x:v>Not closed; no completion credit without gate evidence.</x:v>
       </x:c>
-      <x:c r="L59" s="6" t="str"/>
+      <x:c r="L59" s="6" t="str">
+        <x:v>CONTINUATION-AUDIT.md</x:v>
+      </x:c>
       <x:c r="M59" s="6" t="str"/>
       <x:c r="N59" s="6" t="str">
-        <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
+        <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/CONTINUATION-AUDIT.md</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="124" customHeight="1">
@@ -3560,12 +3711,12 @@
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
       </x:c>
     </x:row>
-    <x:row r="63" ht="124" customHeight="1">
+    <x:row r="63" ht="162" customHeight="1">
       <x:c r="A63" s="6" t="str">
         <x:v>V58</x:v>
       </x:c>
       <x:c r="B63" s="6" t="str">
-        <x:v>Long-session headphone mix and notification-rate controls</x:v>
+        <x:v>Production sound/music pass, water acoustics and long-session clarity</x:v>
       </x:c>
       <x:c r="C63" s="6" t="str">
         <x:v>Planned</x:v>
@@ -3586,18 +3737,22 @@
         <x:v>V43, V44, V50</x:v>
       </x:c>
       <x:c r="I63" s="6" t="str">
-        <x:v>Bounded voices alone do not guarantee pleasant sound.</x:v>
+        <x:v>The user explicitly prioritizes much stronger in-game sound and music; precise archery also needs audible material identity and readable threat direction.</x:v>
       </x:c>
       <x:c r="J63" s="6" t="str">
-        <x:v>Add independent notification density/rate controls; test 30-minute sessions with music transitions, simultaneous threats and repeated UI actions. Record human mix feedback and remove tiring repetition.</x:v>
+        <x:v>Improve bow tension/release, crossbow winding/reload, arrow material impacts, shield impact/break, distinct enemy warnings, bells/wind, footsteps, water entries/splashes/drips and room ambience. Add restrained exploration/pressure/recovery/boss transitions; preserve independent buses, mute, captions, quiet mix, controller access and voice budgets. Pass PCM/lifecycle tests and a dated 30-minute human headphone review.</x:v>
       </x:c>
       <x:c r="K63" s="6" t="str">
-        <x:v>Not closed; no completion credit without gate evidence.</x:v>
-      </x:c>
-      <x:c r="L63" s="6" t="str"/>
+        <x:v>Planned production pass. Resonant Hunt audio exists; current tidelight.js does not wire water-specific sounds. Earlier draft descriptions of positional water splashes/footsteps are not shipped evidence.</x:v>
+      </x:c>
+      <x:c r="L63" s="6" t="str">
+        <x:v>RESONANT-HUNT.md
+tidelight.js
+CONTINUATION-AUDIT.md</x:v>
+      </x:c>
       <x:c r="M63" s="6" t="str"/>
       <x:c r="N63" s="6" t="str">
-        <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
+        <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/RESONANT-HUNT.md</x:v>
       </x:c>
     </x:row>
     <x:row r="64" ht="124" customHeight="1">
@@ -3680,7 +3835,7 @@
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
       </x:c>
     </x:row>
-    <x:row r="66" ht="124" customHeight="1">
+    <x:row r="66" ht="162" customHeight="1">
       <x:c r="A66" s="6" t="str">
         <x:v>V61</x:v>
       </x:c>
@@ -3709,15 +3864,17 @@
         <x:v>Different bodies and play spaces need more than a handedness toggle.</x:v>
       </x:c>
       <x:c r="J66" s="6" t="str">
-        <x:v>Configurable action mapping with conflict checks, seated/standing height and reach calibration, turn/motion presets and readable UI. Each can be reset without a mouse.</x:v>
+        <x:v>Configurable action mapping with conflict checks, seated/standing height and reach calibration, turn/motion presets and readable UI. Each can be reset without a mouse. Resolve grip-role conflicts by documenting the current bow-hand shard/free-hand shield mapping; implement physical thrown shards under V24, not an undocumented remap. Cover every new water/audio panel in controller-only tests.</x:v>
       </x:c>
       <x:c r="K66" s="6" t="str">
         <x:v>Not closed; no completion credit without gate evidence.</x:v>
       </x:c>
-      <x:c r="L66" s="6" t="str"/>
+      <x:c r="L66" s="6" t="str">
+        <x:v>CONTINUATION-AUDIT.md</x:v>
+      </x:c>
       <x:c r="M66" s="6" t="str"/>
       <x:c r="N66" s="6" t="str">
-        <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
+        <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/CONTINUATION-AUDIT.md</x:v>
       </x:c>
     </x:row>
     <x:row r="67" ht="124" customHeight="1">
@@ -3760,7 +3917,7 @@
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
       </x:c>
     </x:row>
-    <x:row r="68" ht="124" customHeight="1">
+    <x:row r="68" ht="190" customHeight="1">
       <x:c r="A68" s="6" t="str">
         <x:v>V63</x:v>
       </x:c>
@@ -3789,15 +3946,17 @@
         <x:v>Threats and menus must remain readable beyond one ideal user.</x:v>
       </x:c>
       <x:c r="J68" s="6" t="str">
-        <x:v>Text size/contrast, sound direction captions, color-independent ammunition/enemy signals and reduced-flash mode survive desktop, stereo and passthrough contexts. Human accessibility review required.</x:v>
+        <x:v>Text size/contrast, sound direction captions, color-independent ammunition/enemy signals and reduced-flash mode survive desktop, stereo and passthrough contexts. Human accessibility review required. Preserve the palm-familiar, diegetic status design for VR and supported accessibility fallbacks. The user requested discrete hit points rather than a bar; the existing numerical health model and desktop HUD are a recorded design gap, not authorization to silently change save semantics.</x:v>
       </x:c>
       <x:c r="K68" s="6" t="str">
         <x:v>Not closed; no completion credit without gate evidence.</x:v>
       </x:c>
-      <x:c r="L68" s="6" t="str"/>
+      <x:c r="L68" s="6" t="str">
+        <x:v>CONTINUATION-AUDIT.md</x:v>
+      </x:c>
       <x:c r="M68" s="6" t="str"/>
       <x:c r="N68" s="6" t="str">
-        <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
+        <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/CONTINUATION-AUDIT.md</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="124" customHeight="1">
@@ -3840,7 +3999,7 @@
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
       </x:c>
     </x:row>
-    <x:row r="70" ht="124" customHeight="1">
+    <x:row r="70" ht="148" customHeight="1">
       <x:c r="A70" s="6" t="str">
         <x:v>V65</x:v>
       </x:c>
@@ -3869,7 +4028,7 @@
         <x:v>A published game needs durable progress across later upgrades.</x:v>
       </x:c>
       <x:c r="J70" s="6" t="str">
-        <x:v>Keep fixtures for old supported generator/schema versions, offer explicit local backup/restore and verify interrupted writes, browser quota and update migration. Never silently reset incompatible saves.</x:v>
+        <x:v>Keep fixtures for old supported generator/schema versions, offer explicit local backup/restore and verify interrupted writes, browser quota and update migration. Never silently reset incompatible saves. Any future discrete-hit-point conversion must specify health/healing balance and tested checkpoint migration; retain current health and profiles in presentation-only releases.</x:v>
       </x:c>
       <x:c r="K70" s="6" t="str">
         <x:v>Not closed; no completion credit without gate evidence.</x:v>
@@ -3880,7 +4039,7 @@
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
       </x:c>
     </x:row>
-    <x:row r="71" ht="124" customHeight="1">
+    <x:row r="71" ht="176" customHeight="1">
       <x:c r="A71" s="6" t="str">
         <x:v>V66</x:v>
       </x:c>
@@ -3909,15 +4068,17 @@
         <x:v>Finite smoke tests are not a complete campaign quality gate.</x:v>
       </x:c>
       <x:c r="J71" s="6" t="str">
-        <x:v>Run at least 1000 proposed seed/depth fixtures and 50 lifecycle transitions, tracking unreachable rewards, spawning collisions, NaNs, leaks and progress duplication. Publish failures and seed repros.</x:v>
+        <x:v>Run at least 1000 proposed seed/depth fixtures and 50 lifecycle transitions, tracking unreachable rewards, spawning collisions, NaNs, leaks and progress duplication. Publish failures and seed repros. Add dedicated Tidelight tests for pool placement across depth/seed, standing on high walks above water, actual arrow-water crossings, paused/reduced-effects motion, sector clock resets, AR return and old-save continuation.</x:v>
       </x:c>
       <x:c r="K71" s="6" t="str">
         <x:v>Not closed; no completion credit without gate evidence.</x:v>
       </x:c>
-      <x:c r="L71" s="6" t="str"/>
+      <x:c r="L71" s="6" t="str">
+        <x:v>CONTINUATION-AUDIT.md</x:v>
+      </x:c>
       <x:c r="M71" s="6" t="str"/>
       <x:c r="N71" s="6" t="str">
-        <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
+        <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/CONTINUATION-AUDIT.md</x:v>
       </x:c>
     </x:row>
     <x:row r="72" ht="124" customHeight="1">
@@ -3960,7 +4121,7 @@
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
       </x:c>
     </x:row>
-    <x:row r="73" ht="124" customHeight="1">
+    <x:row r="73" ht="190" customHeight="1">
       <x:c r="A73" s="6" t="str">
         <x:v>V68</x:v>
       </x:c>
@@ -3989,14 +4150,15 @@
         <x:v>Do not confuse a merged commit with a complete verified release.</x:v>
       </x:c>
       <x:c r="J73" s="6" t="str">
-        <x:v>Byte-verified deployment already exists. Add explicit stable/candidate policy, save-safe rollback drill, reproducible asset pipeline and release-note/device-evidence review.</x:v>
+        <x:v>For every finished upgrade, test the actual scoped source, commit and merge without overwriting sibling games, verify GitHub Pages deployment plus public runtime/asset/plan/workbook bytes, then launch the public game. Separate source, test, deployment, hardware and human evidence. Retry transient GitHub faults with backoff; inspect failed jobs instead of polling an unchanged failure list. Preserve explicit rollback and save-compatibility notes.</x:v>
       </x:c>
       <x:c r="K73" s="6" t="str">
-        <x:v>Not closed; no completion credit without gate evidence.</x:v>
+        <x:v>Partial. Tidelight was published, but archived run 34737842771 stopped before browser checks because roadmap 0.11.0 disagreed with release 0.12.0. This planning repair fixes that mismatch; it does not retrospectively turn skipped gameplay acceptance green.</x:v>
       </x:c>
       <x:c r="L73" s="6" t="str">
         <x:v>tests/verify-live.py
-tests/launch.py</x:v>
+tests/launch.py
+CONTINUATION-AUDIT.md</x:v>
       </x:c>
       <x:c r="M73" s="6" t="str"/>
       <x:c r="N73" s="6" t="str">
@@ -4203,7 +4365,7 @@
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
       </x:c>
     </x:row>
-    <x:row r="79" ht="124" customHeight="1">
+    <x:row r="79" ht="190" customHeight="1">
       <x:c r="A79" s="6" t="str">
         <x:v>V74</x:v>
       </x:c>
@@ -4232,15 +4394,19 @@
         <x:v>Repeated additive patches increase the risk of hidden lifecycle regressions.</x:v>
       </x:c>
       <x:c r="J79" s="6" t="str">
-        <x:v>Reduce wrapper-order coupling with explicit lifecycle interfaces and dependency tests; preserve current save fixtures, deterministic physics and controller mappings.</x:v>
+        <x:v>Reduce wrapper-order coupling with explicit lifecycle interfaces and dependency tests; preserve current save fixtures, deterministic physics and controller mappings. Audit current Tidelight: maxRipples is declared by policy but tick uploads all 10 slots; rebuild does not clear ripple timestamps/lastStep; inside() does not match the rendered inset; impact and footstep splash checks omit height. Treat these as source-review findings needing reproductions and tests, not fixes already shipped.</x:v>
       </x:c>
       <x:c r="K79" s="6" t="str">
         <x:v>Not closed; no completion credit without gate evidence.</x:v>
       </x:c>
-      <x:c r="L79" s="6" t="str"/>
+      <x:c r="L79" s="6" t="str">
+        <x:v>tidelight.js
+tidelight-shaders.js
+CONTINUATION-AUDIT.md</x:v>
+      </x:c>
       <x:c r="M79" s="6" t="str"/>
       <x:c r="N79" s="6" t="str">
-        <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
+        <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/tidelight.js</x:v>
       </x:c>
     </x:row>
     <x:row r="80" ht="124" customHeight="1">
@@ -4382,7 +4548,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Redb18996740d4745"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdadc18230c054e81"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4479,13 +4645,13 @@
         <x:v>Playable foundations</x:v>
       </x:c>
       <x:c r="C6" s="6" t="str">
-        <x:v>Implemented</x:v>
+        <x:v>Partial</x:v>
       </x:c>
       <x:c r="D6" s="6" t="str">
         <x:v>None</x:v>
       </x:c>
       <x:c r="E6" s="6" t="str">
-        <x:v>Retain the shipped original browser/VR/AR foundation.</x:v>
+        <x:v>Retain shipped browser/VR/AR foundations and close the newest water-interface and release-evidence gaps.</x:v>
       </x:c>
       <x:c r="F6" s="6" t="str">
         <x:v>Current foundation and input/model/public deployment tests pass; hardware acceptance is not implied.</x:v>
@@ -4496,7 +4662,7 @@
       </x:c>
       <x:c r="H6" s="18" t="n">
         <x:f>COUNTIFS(Backlog!$E$6:$E$81,A6,Backlog!$C$6:$C$81,"Implemented")</x:f>
-        <x:v>32</x:v>
+        <x:v>31</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="112" customHeight="1">
@@ -4684,7 +4850,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0a9104c7460b48cc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R590db8259c084bda"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5049,31 +5215,74 @@
       <x:c r="I15" s="20"/>
       <x:c r="J15" s="6"/>
     </x:row>
-    <x:row r="16">
-      <x:c r="A16" s="6"/>
-      <x:c r="B16" s="6"/>
-      <x:c r="C16" s="6"/>
-      <x:c r="D16" s="6"/>
-      <x:c r="E16" s="6"/>
-      <x:c r="F16" s="6"/>
-      <x:c r="G16" s="6"/>
+    <x:row r="16" ht="140" customHeight="1">
+      <x:c r="A16" s="6" t="str">
+        <x:v>Q11</x:v>
+      </x:c>
+      <x:c r="B16" s="6" t="str">
+        <x:v>Quest 3 / Tidelight</x:v>
+      </x:c>
+      <x:c r="C16" s="6" t="str">
+        <x:v>Water and complete spatial settings</x:v>
+      </x:c>
+      <x:c r="D16" s="6" t="str">
+        <x:v>Reach/change/close all water controls; enforce actual ripple/pool budget; verify both eyes, AR exclusion and repeated XR entry/exit</x:v>
+      </x:c>
+      <x:c r="E16" s="6" t="str">
+        <x:v>V38,V41,V62,V74</x:v>
+      </x:c>
+      <x:c r="F16" s="6" t="str">
+        <x:v>Not run</x:v>
+      </x:c>
+      <x:c r="G16" s="6" t="str">
+        <x:v>Record source/build hash and real headset/browser versions. Policy fields alone are not proof that runtime honors the caps.</x:v>
+      </x:c>
       <x:c r="H16" s="6"/>
       <x:c r="I16" s="6"/>
       <x:c r="J16" s="6"/>
+    </x:row>
+    <x:row r="17" ht="140" customHeight="1">
+      <x:c r="A17" s="47" t="str">
+        <x:v>Q12</x:v>
+      </x:c>
+      <x:c r="B17" s="47" t="str">
+        <x:v>Desktop / water and audio</x:v>
+      </x:c>
+      <x:c r="C17" s="47" t="str">
+        <x:v>Source-to-screen/sound parity</x:v>
+      </x:c>
+      <x:c r="D17" s="47" t="str">
+        <x:v>Seed/depth-specific pools, visible stone, caustics, actual impact/footstep positions and music/water mix; no false claim of reflection/refraction</x:v>
+      </x:c>
+      <x:c r="E17" s="47" t="str">
+        <x:v>V35,V58,V66</x:v>
+      </x:c>
+      <x:c r="F17" s="47" t="str">
+        <x:v>Not run</x:v>
+      </x:c>
+      <x:c r="G17" s="47" t="str">
+        <x:v>Archive actual gameplay screenshots and audio receipts. Recovering a draft does not make its features part of the release.</x:v>
+      </x:c>
+      <x:c r="H17" s="47"/>
+      <x:c r="I17" s="47"/>
+      <x:c r="J17" s="47"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:J2"/>
     <x:mergeCell ref="A3:J3"/>
   </x:mergeCells>
-  <x:dataValidations count="1">
+  <x:dataValidations count="2">
     <x:dataValidation type="list" sqref="F6:F15">
       <x:formula1>"Not run,Software only,Passed on device,Failed on device,Blocked"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="F6:F17">
+      <x:formula1>"Not run,Software only,Pass,Fail,Blocked"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R096389eea6dc41da"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf642ba3e03e74a33"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5162,7 +5371,7 @@
         <x:v>Result / evidence receipt</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="110" customHeight="1">
+    <x:row r="6" ht="165" customHeight="1">
       <x:c r="A6" s="6" t="str">
         <x:v>G01</x:v>
       </x:c>
@@ -5173,7 +5382,7 @@
         <x:v>Engineering</x:v>
       </x:c>
       <x:c r="D6" s="6" t="str">
-        <x:v>Only reviewed game paths change; exact source/build is identified; private story excluded.</x:v>
+        <x:v>Only reviewed game paths change; exact source/build is identified; private story excluded. Canonical roadmap version, release version and core version must agree; the workbook must match every task field and the JSON digest.</x:v>
       </x:c>
       <x:c r="E6" s="6" t="str">
         <x:v>tests and repository diff</x:v>
@@ -5210,7 +5419,7 @@
       </x:c>
       <x:c r="H7" s="6"/>
     </x:row>
-    <x:row r="8" ht="110" customHeight="1">
+    <x:row r="8" ht="165" customHeight="1">
       <x:c r="A8" s="6" t="str">
         <x:v>G03</x:v>
       </x:c>
@@ -5221,7 +5430,7 @@
         <x:v>UX / QA</x:v>
       </x:c>
       <x:c r="D8" s="6" t="str">
-        <x:v>Native Xbox and stereo-XR fixtures pass; essential actions have no mouse-only dead end.</x:v>
+        <x:v>Native Xbox and stereo-XR fixtures pass; essential actions have no mouse-only dead end. Include Tidelight water controls and both Quest handedness settings; historical menus alone do not close the expanded UI gate.</x:v>
       </x:c>
       <x:c r="E8" s="6" t="str">
         <x:v>tests/dominions-browser.py</x:v>
@@ -5258,7 +5467,7 @@
       </x:c>
       <x:c r="H9" s="6"/>
     </x:row>
-    <x:row r="10" ht="110" customHeight="1">
+    <x:row r="10" ht="165" customHeight="1">
       <x:c r="A10" s="6" t="str">
         <x:v>G05</x:v>
       </x:c>
@@ -5269,7 +5478,7 @@
         <x:v>Technical art / audio</x:v>
       </x:c>
       <x:c r="D10" s="6" t="str">
-        <x:v>Native WebGL and stereo audio checks pass; no script errors, broken asset loads or repeating hidden-tab backlog.</x:v>
+        <x:v>Native WebGL and stereo audio checks pass; no script errors, broken asset loads or repeating hidden-tab backlog. Dedicated water render/lifecycle and future water-sound evidence are required; do not substitute release text or a successful Pages build.</x:v>
       </x:c>
       <x:c r="E10" s="6" t="str">
         <x:v>tests/resonant-browser.py; tests/jewelglass-browser.py</x:v>
@@ -5419,7 +5628,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0564014c6268424f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb544c8baba314f48"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5664,7 +5873,7 @@
         <x:v>Open</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" ht="100" customHeight="1">
+    <x:row r="12" ht="145" customHeight="1">
       <x:c r="A12" s="6" t="str">
         <x:v>R07</x:v>
       </x:c>
@@ -5678,16 +5887,16 @@
         <x:v>Production</x:v>
       </x:c>
       <x:c r="E12" s="6" t="str">
-        <x:v>Previous board remained at 0.6 after 0.8 shipped</x:v>
+        <x:v>At audit: Tidelight 0.12.0 shipped while roadmap/workbook remained 0.11.0; archived full-model run had one version failure.</x:v>
       </x:c>
       <x:c r="F12" s="6" t="str">
         <x:v>V48</x:v>
       </x:c>
       <x:c r="G12" s="6" t="str">
-        <x:v>Check version consistency and preserve one canonical JSON plus generated workbook snapshot.</x:v>
+        <x:v>Synchronize canonical plan, workbook and resume docs together; run version/digest tests before publication and preserve the historical failure.</x:v>
       </x:c>
       <x:c r="H12" s="6" t="str">
-        <x:v>Mitigated by checks</x:v>
+        <x:v>Open / repair requires release discipline</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="100" customHeight="1">
@@ -5768,15 +5977,57 @@
         <x:v>Open</x:v>
       </x:c>
     </x:row>
-    <x:row r="16">
-      <x:c r="A16" s="6"/>
-      <x:c r="B16" s="6"/>
-      <x:c r="C16" s="6"/>
-      <x:c r="D16" s="6"/>
-      <x:c r="E16" s="6"/>
-      <x:c r="F16" s="6"/>
-      <x:c r="G16" s="6"/>
-      <x:c r="H16" s="6"/>
+    <x:row r="16" ht="150" customHeight="1">
+      <x:c r="A16" s="6" t="str">
+        <x:v>R11</x:v>
+      </x:c>
+      <x:c r="B16" s="6" t="str">
+        <x:v>Interrupted draft mistaken for published features</x:v>
+      </x:c>
+      <x:c r="C16" s="6" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="D16" s="6" t="str">
+        <x:v>Production / engineering</x:v>
+      </x:c>
+      <x:c r="E16" s="6" t="str">
+        <x:v>The larger water draft described seven surfaces, named extra areas, basin refraction, reflections and sounds absent from current Tidelight source.</x:v>
+      </x:c>
+      <x:c r="F16" s="6" t="str">
+        <x:v>V35,V58,V68</x:v>
+      </x:c>
+      <x:c r="G16" s="6" t="str">
+        <x:v>Inspect current source first; preserve draft intent as future work and do not replay opaque transfer chunks over master.</x:v>
+      </x:c>
+      <x:c r="H16" s="6" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="150" customHeight="1">
+      <x:c r="A17" s="47" t="str">
+        <x:v>R12</x:v>
+      </x:c>
+      <x:c r="B17" s="47" t="str">
+        <x:v>Water policy/lifecycle implementation differs from its intent</x:v>
+      </x:c>
+      <x:c r="C17" s="47" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="D17" s="47" t="str">
+        <x:v>Engineering / technical art</x:v>
+      </x:c>
+      <x:c r="E17" s="47" t="str">
+        <x:v>Ripple-cap, world-clock reset, footprint and height checks need dedicated tests; water controls missing from XR list.</x:v>
+      </x:c>
+      <x:c r="F17" s="47" t="str">
+        <x:v>V38,V41,V66,V74</x:v>
+      </x:c>
+      <x:c r="G17" s="47" t="str">
+        <x:v>Reproduce each finding and add small save-safe fixes with real-frame and controller evidence.</x:v>
+      </x:c>
+      <x:c r="H17" s="47" t="str">
+        <x:v>Open</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -5795,7 +6046,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8e54c835d1604ee7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R83db27770ff14a3a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Synchronize Vesperfall 0.12 production workbook and preserve cross-chat continuation audit
Preserve 76 task IDs, seven milestones, existing six-sheet workbook and concurrent handoff prose. Align canonical planning and diagnostic version with the published Tidelight release, record shipped-vs-draft water scope, exact controller roles, audio/music priorities, missing acceptance, and ordered next actions. Validated in workflow 34774449486: 153 model tests and 16 native planning-board/workbook checks, zero failures. No gameplay mechanics, collision, generator, save-schema or sibling-game changes. Temporary intake removed; physical-device and human review remain open.
</commit_message>
<xml_diff>
--- a/vesperfall/AAA-PRODUCTION.xlsx
+++ b/vesperfall/AAA-PRODUCTION.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="R5422c9ec86e54f0d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="2" r:id="R55a7ea2099fa4869"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Milestones" sheetId="3" r:id="R4b608d0afcc44efb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Device QA" sheetId="4" r:id="R78d077327f794c7e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="5" r:id="R9b625fbc4c40465a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risk Register" sheetId="6" r:id="R0317debfb8b54e62"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="R242c3143bbe74260"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="2" r:id="R59926fb31b304cee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Milestones" sheetId="3" r:id="R006124efab6c4c9c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Device QA" sheetId="4" r:id="R4ba785b8f0b94f51"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="5" r:id="R00e8525b5cfb4e32"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risk Register" sheetId="6" r:id="Re505e8c2936744b2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -22,7 +22,7 @@
     <x:numFmt numFmtId="200" formatCode="0"/>
     <x:numFmt numFmtId="201" formatCode="yyyy-mm-dd"/>
   </x:numFmts>
-  <x:fonts count="8">
+  <x:fonts count="11">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -67,8 +67,24 @@
       <x:color rgb="FF203441"/>
       <x:name val="Calibri"/>
     </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF176B68"/>
+      <x:name val="Calibri"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF243B47"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="5">
+  <x:fills count="8">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -90,6 +106,21 @@
         <x:fgColor rgb="FF176F68"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF176B68"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEFF4F4"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="2">
     <x:border/>
@@ -98,7 +129,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="35">
+  <x:cellXfs count="48">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -195,6 +226,31 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -294,7 +350,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="DeviceMatrix" displayName="DeviceMatrix" ref="A5:J15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="DeviceMatrix" displayName="DeviceMatrix" ref="A5:J17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Device / mode"/>
@@ -328,7 +384,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="ProductionRisks" displayName="ProductionRisks" ref="A5:H15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="ProductionRisks" displayName="ProductionRisks" ref="A5:H17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Risk"/>
@@ -572,7 +628,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="12" t="str">
-        <x:v>v0.11.0 / Rosefire / 2026-09-12. Original gothic shaders extend the existing First Bell game. AAA-level finish remains a quality-gated aspiration, not a hardware certificate.</x:v>
+        <x:v>v0.12.0 / Tidelight / planning audit 2026-09-13. Roadmap, workbook and core diagnostic version labels are synchronized; gameplay mechanics and save formats are unchanged.</x:v>
       </x:c>
       <x:c r="B3" s="12"/>
       <x:c r="C3" s="12"/>
@@ -628,7 +684,7 @@
       <x:c r="B7" s="28"/>
       <x:c r="C7" s="28" t="n">
         <x:f>COUNTIF(Backlog!C6:C81,"Implemented")</x:f>
-        <x:v>35</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="D7" s="28"/>
       <x:c r="E7" s="28" t="n">
@@ -718,7 +774,7 @@
     </x:row>
     <x:row r="15" ht="24" customHeight="1">
       <x:c r="A15" s="6" t="str">
-        <x:v>This release adds ten guided archery lessons and the optional Bellkeeper Oath: three connected encounters, a three-phase boss, recovery beats and saved continuation. V49-V52 and V76 remain Partial until their broader human, hardware and production gates are met.</x:v>
+        <x:v>Shipped water is the bounded translucent-plane baseline. The earlier detailed basin/refraction/reflection/audio draft is not the published implementation. Read the continuation audit before promising or recovering those features.</x:v>
       </x:c>
       <x:c r="B15" s="6"/>
       <x:c r="C15" s="6"/>
@@ -782,7 +838,7 @@
     </x:row>
     <x:row r="21" ht="24" customHeight="1">
       <x:c r="A21" s="6" t="str">
-        <x:v>Before production release, close measured Quest performance, actual controller lifecycle/comfort, long-session sound, finished assets, external playtesting, save migration, content completeness and blocking-defect gates.</x:v>
+        <x:v>Next: establish Tidelight browser/render/save evidence, close Quest water-menu and lifecycle gaps, then prioritize the requested sound/music pass and purposeful exploration. Keep all physical-device and human gates open until measured.</x:v>
       </x:c>
       <x:c r="B21" s="6"/>
       <x:c r="C21" s="6"/>
@@ -814,7 +870,7 @@
     </x:row>
     <x:row r="24" ht="24" customHeight="1">
       <x:c r="A24" s="6" t="str">
-        <x:v>There are no invented delivery dates, staffing commitments or cost estimates. Owner roles require assignment. Physical-device targets and proposed test-batch sizes are planning inputs to verify, not current results.</x:v>
+        <x:v>Historical acceptance: 148 model passes, 1 stale-plan failure; browser steps skipped. Fresh planning checks are separate. No invented hardware approval, staffing, dates, budget, playtime or AAA rating is included.</x:v>
       </x:c>
       <x:c r="B24" s="6"/>
       <x:c r="C24" s="6"/>
@@ -846,7 +902,7 @@
     </x:row>
     <x:row r="27" ht="24" customHeight="1">
       <x:c r="A27" s="34" t="str">
-        <x:v>Canonical JSON SHA-256: e5fa1d8a3476502e514485305e19f4095f419ce8d165203fec6301028488fa8c</x:v>
+        <x:v>Canonical JSON SHA-256: 8d31f942c3913354082adef2f0034cedd120b367a19964acaf3186feecc77a98</x:v>
       </x:c>
       <x:c r="B27" s="34"/>
       <x:c r="C27" s="34"/>
@@ -867,50 +923,52 @@
       <x:c r="H28" s="6"/>
     </x:row>
     <x:row r="29" ht="24" customHeight="1">
-      <x:c r="A29" s="6" t="str">
+      <x:c r="A29" s="36" t="str">
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
       </x:c>
-      <x:c r="B29" s="6"/>
-      <x:c r="C29" s="6"/>
-      <x:c r="D29" s="6"/>
-      <x:c r="E29" s="6"/>
-      <x:c r="F29" s="6"/>
-      <x:c r="G29" s="6"/>
-      <x:c r="H29" s="6"/>
+      <x:c r="B29" s="36"/>
+      <x:c r="C29" s="36"/>
+      <x:c r="D29" s="36"/>
+      <x:c r="E29" s="36"/>
+      <x:c r="F29" s="36"/>
+      <x:c r="G29" s="36"/>
+      <x:c r="H29" s="36"/>
     </x:row>
     <x:row r="30" ht="24" customHeight="1">
-      <x:c r="A30" s="6" t="str">
+      <x:c r="A30" s="36" t="str">
         <x:v>https://v5ma.github.io/vesperfall/roadmap.html</x:v>
       </x:c>
-      <x:c r="B30" s="6"/>
-      <x:c r="C30" s="6"/>
-      <x:c r="D30" s="6"/>
-      <x:c r="E30" s="6"/>
-      <x:c r="F30" s="6"/>
-      <x:c r="G30" s="6"/>
-      <x:c r="H30" s="6"/>
+      <x:c r="B30" s="36"/>
+      <x:c r="C30" s="36"/>
+      <x:c r="D30" s="36"/>
+      <x:c r="E30" s="36"/>
+      <x:c r="F30" s="36"/>
+      <x:c r="G30" s="36"/>
+      <x:c r="H30" s="36"/>
     </x:row>
     <x:row r="31" ht="24" customHeight="1">
-      <x:c r="A31" s="6" t="str">
-        <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/AAA-ROADMAP.md</x:v>
-      </x:c>
-      <x:c r="B31" s="6"/>
-      <x:c r="C31" s="6"/>
-      <x:c r="D31" s="6"/>
-      <x:c r="E31" s="6"/>
-      <x:c r="F31" s="6"/>
-      <x:c r="G31" s="6"/>
-      <x:c r="H31" s="6"/>
+      <x:c r="A31" s="36" t="str">
+        <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/DEVELOPMENT-HANDOFF.md</x:v>
+      </x:c>
+      <x:c r="B31" s="36"/>
+      <x:c r="C31" s="36"/>
+      <x:c r="D31" s="36"/>
+      <x:c r="E31" s="36"/>
+      <x:c r="F31" s="36"/>
+      <x:c r="G31" s="36"/>
+      <x:c r="H31" s="36"/>
     </x:row>
     <x:row r="32" ht="24" customHeight="1">
-      <x:c r="A32" s="6"/>
-      <x:c r="B32" s="6"/>
-      <x:c r="C32" s="6"/>
-      <x:c r="D32" s="6"/>
-      <x:c r="E32" s="6"/>
-      <x:c r="F32" s="6"/>
-      <x:c r="G32" s="6"/>
-      <x:c r="H32" s="6"/>
+      <x:c r="A32" s="36" t="str">
+        <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/CONTINUATION-AUDIT.md</x:v>
+      </x:c>
+      <x:c r="B32" s="36"/>
+      <x:c r="C32" s="36"/>
+      <x:c r="D32" s="36"/>
+      <x:c r="E32" s="36"/>
+      <x:c r="F32" s="36"/>
+      <x:c r="G32" s="36"/>
+      <x:c r="H32" s="36"/>
     </x:row>
     <x:row r="33" ht="24" customHeight="1">
       <x:c r="A33" s="6"/>
@@ -921,6 +979,78 @@
       <x:c r="F33" s="6"/>
       <x:c r="G33" s="6"/>
       <x:c r="H33" s="6"/>
+    </x:row>
+    <x:row r="34" ht="26" customHeight="1">
+      <x:c r="A34" s="38" t="str">
+        <x:v>RESUME WITH THESE EXISTING TASKS</x:v>
+      </x:c>
+      <x:c r="B34" s="38"/>
+      <x:c r="C34" s="38"/>
+      <x:c r="D34" s="38"/>
+      <x:c r="E34" s="38"/>
+      <x:c r="F34" s="38"/>
+      <x:c r="G34" s="38"/>
+      <x:c r="H34" s="38"/>
+    </x:row>
+    <x:row r="36" ht="46" customHeight="1">
+      <x:c r="A36" s="42" t="str">
+        <x:v>V68 / V66: verify the actual 0.12 baseline. Do not treat a successful Pages build, a draft test count or historical Rosefire tests as Tidelight gameplay acceptance.</x:v>
+      </x:c>
+      <x:c r="B36" s="42"/>
+      <x:c r="C36" s="42"/>
+      <x:c r="D36" s="42"/>
+      <x:c r="E36" s="42"/>
+      <x:c r="F36" s="42"/>
+      <x:c r="G36" s="42"/>
+      <x:c r="H36" s="42"/>
+    </x:row>
+    <x:row r="37" ht="46" customHeight="1">
+      <x:c r="A37" s="46" t="str">
+        <x:v>V41 / V61 / V74: finish Quest water settings and verify all Xbox/Quest open, adjust, select, dismiss and recovery paths. Reproduce water footprint, height, ripple-budget and world-clock gaps.</x:v>
+      </x:c>
+      <x:c r="B37" s="46"/>
+      <x:c r="C37" s="46"/>
+      <x:c r="D37" s="46"/>
+      <x:c r="E37" s="46"/>
+      <x:c r="F37" s="46"/>
+      <x:c r="G37" s="46"/>
+      <x:c r="H37" s="46"/>
+    </x:row>
+    <x:row r="38" ht="46" customHeight="1">
+      <x:c r="A38" s="42" t="str">
+        <x:v>V58 / V44: implement water-specific sound, stronger archery/shield/enemy audio and musical transitions. Preserve independent volume buses, mute, captions and warning clarity.</x:v>
+      </x:c>
+      <x:c r="B38" s="42"/>
+      <x:c r="C38" s="42"/>
+      <x:c r="D38" s="42"/>
+      <x:c r="E38" s="42"/>
+      <x:c r="F38" s="42"/>
+      <x:c r="G38" s="42"/>
+      <x:c r="H38" s="42"/>
+    </x:row>
+    <x:row r="39" ht="46" customHeight="1">
+      <x:c r="A39" s="46" t="str">
+        <x:v>V35 / V52 / V54: pursue memorable routes, water destinations and humanoid animation; retain the existing 15 enemy archetypes, First Bell and Bellkeeper Oath.</x:v>
+      </x:c>
+      <x:c r="B39" s="46"/>
+      <x:c r="C39" s="46"/>
+      <x:c r="D39" s="46"/>
+      <x:c r="E39" s="46"/>
+      <x:c r="F39" s="46"/>
+      <x:c r="G39" s="46"/>
+      <x:c r="H39" s="46"/>
+    </x:row>
+    <x:row r="40" ht="46" customHeight="1">
+      <x:c r="A40" s="42" t="str">
+        <x:v>V38 / V59 / V62 / V75: run actual-device comfort, thermal, performance, controller and save-lifecycle checks. Proposed timing budgets are not measurements.</x:v>
+      </x:c>
+      <x:c r="B40" s="42"/>
+      <x:c r="C40" s="42"/>
+      <x:c r="D40" s="42"/>
+      <x:c r="E40" s="42"/>
+      <x:c r="F40" s="42"/>
+      <x:c r="G40" s="42"/>
+      <x:c r="H40" s="42"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -944,6 +1074,13 @@
     <x:mergeCell ref="A29:H29"/>
     <x:mergeCell ref="A30:H30"/>
     <x:mergeCell ref="A31:H31"/>
+    <x:mergeCell ref="A32:H32"/>
+    <x:mergeCell ref="A34:H34"/>
+    <x:mergeCell ref="A36:H36"/>
+    <x:mergeCell ref="A37:H37"/>
+    <x:mergeCell ref="A38:H38"/>
+    <x:mergeCell ref="A39:H39"/>
+    <x:mergeCell ref="A40:H40"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -1005,7 +1142,7 @@
     </x:row>
     <x:row r="3" ht="36" customHeight="1">
       <x:c r="A3" s="12" t="str">
-        <x:v>Canonical snapshot v0.9.0 | 76 retained and new tasks | Status is not AAA certification. Filter any column; edit locally and reconcile with roadmap.json before committing.</x:v>
+        <x:v>v0.12.0 / 76 preserved tasks / September 13 source audit. Partial means the expanded acceptance scope remains open.</x:v>
       </x:c>
       <x:c r="B3" s="12"/>
       <x:c r="C3" s="12"/>
@@ -2543,12 +2680,12 @@
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
       </x:c>
     </x:row>
-    <x:row r="40" ht="124" customHeight="1">
+    <x:row r="40" ht="120" customHeight="1">
       <x:c r="A40" s="6" t="str">
         <x:v>V35</x:v>
       </x:c>
       <x:c r="B40" s="6" t="str">
-        <x:v>Authored crypt/roof transitions and expanded graph vocabulary</x:v>
+        <x:v>Authored crypt, roof and water destinations with expanded route grammar</x:v>
       </x:c>
       <x:c r="C40" s="6" t="str">
         <x:v>Partial</x:v>
@@ -2569,19 +2706,24 @@
         <x:v>None</x:v>
       </x:c>
       <x:c r="I40" s="6" t="str">
-        <x:v>Preserve the established game while closing the stated acceptance gate.</x:v>
+        <x:v>More areas should create memorable choices and reasons to explore, not repeat one room or flood every courtyard.</x:v>
       </x:c>
       <x:c r="J40" s="6" t="str">
-        <x:v>25-district graph expansion shipped. Distinct authored crypt-to-roof transitions and stronger route grammar still need design and native traversal evidence.</x:v>
+        <x:v>Keep the existing 25-district game and reversible upper/lower routes. Add distinctive, collision-tested destinations, escape paths and discoveries. Tidelight water remains decorative until a separately designed, save-compatible traversal feature is approved.</x:v>
       </x:c>
       <x:c r="K40" s="6" t="str">
-        <x:v>Expanded graph implemented; authored transition production remains open.</x:v>
+        <x:v>Partial. Tidelight 0.12.0 water exists in current source. The earlier seven-surface/four-named-district draft, recessed fonts, refracting tile basins and architecture reflections are not established by the shipped implementation.</x:v>
       </x:c>
       <x:c r="L40" s="6" t="str">
         <x:v>dominions-world.js
-HOLLOW-DOMINIONS.md</x:v>
-      </x:c>
-      <x:c r="M40" s="6" t="str"/>
+HOLLOW-DOMINIONS.md
+TIDELIGHT.md
+tidelight.js
+CONTINUATION-AUDIT.md</x:v>
+      </x:c>
+      <x:c r="M40" s="6" t="str">
+        <x:v>0.12.0 Tidelight presentation baseline; authored expansion open</x:v>
+      </x:c>
       <x:c r="N40" s="6" t="str">
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/dominions-world.js</x:v>
       </x:c>
@@ -2675,12 +2817,12 @@
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
       </x:c>
     </x:row>
-    <x:row r="43" ht="124" customHeight="1">
+    <x:row r="43" ht="106" customHeight="1">
       <x:c r="A43" s="6" t="str">
         <x:v>V38</x:v>
       </x:c>
       <x:c r="B43" s="6" t="str">
-        <x:v>Measure physical Quest 3 stereo frame times for Jewelglass and Rosefire</x:v>
+        <x:v>Measure physical Quest 3 stereo frame times for Jewelglass, Rosefire and Tidelight</x:v>
       </x:c>
       <x:c r="C43" s="6" t="str">
         <x:v>Hardware QA</x:v>
@@ -2695,7 +2837,7 @@
         <x:v>Hardware</x:v>
       </x:c>
       <x:c r="G43" s="6" t="str">
-        <x:v>Device QA</x:v>
+        <x:v>Device QA / assignment pending</x:v>
       </x:c>
       <x:c r="H43" s="6" t="str">
         <x:v>None</x:v>
@@ -2704,17 +2846,19 @@
         <x:v>A software fixture cannot tell us how a person feels or how a real device sustains the experience.</x:v>
       </x:c>
       <x:c r="J43" s="6" t="str">
-        <x:v>Measure on device; never infer FPS, comfort or controller alignment from headless emulation.</x:v>
+        <x:v>Measure both eyes, bow/ward visibility, water/caustic legibility and sustained frame times on Quest 3 in both handedness modes. Check reduced effects and AR exclusions. Do not infer hardware FPS, comfort or alignment from emulation.</x:v>
       </x:c>
       <x:c r="K43" s="6" t="str">
         <x:v>No physical device receipt yet.</x:v>
       </x:c>
       <x:c r="L43" s="6" t="str">
-        <x:v>ROSEFIRE.md</x:v>
+        <x:v>ROSEFIRE.md
+TIDELIGHT.md
+CONTINUATION-AUDIT.md</x:v>
       </x:c>
       <x:c r="M43" s="6" t="str"/>
       <x:c r="N43" s="6" t="str">
-        <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
+        <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/ROSEFIRE.md</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="124" customHeight="1">
@@ -2808,7 +2952,7 @@
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/bestiary.js</x:v>
       </x:c>
     </x:row>
-    <x:row r="46" ht="124" customHeight="1">
+    <x:row r="46" ht="134" customHeight="1">
       <x:c r="A46" s="6" t="str">
         <x:v>V41</x:v>
       </x:c>
@@ -2816,7 +2960,7 @@
         <x:v>Xbox focus navigation and paginated Quest spatial menus</x:v>
       </x:c>
       <x:c r="C46" s="6" t="str">
-        <x:v>Implemented</x:v>
+        <x:v>Partial</x:v>
       </x:c>
       <x:c r="D46" s="6" t="str">
         <x:v>P0</x:v>
@@ -2837,14 +2981,16 @@
         <x:v>Avoid forced mouse use or headset removal.</x:v>
       </x:c>
       <x:c r="J46" s="6" t="str">
-        <x:v>Gameplay, settings, seeds, equipment, journal and in-game dialogs can be operated with controller input. System permission prompts are not game-owned.</x:v>
+        <x:v>Every gameplay and game-owned UI path, including water settings, confirmations, recovery, seed entry, audio and accessibility settings, is reachable and dismissible with Xbox and Quest controls without a mouse. Test both handedness modes, neutral-input transitions and return focus. Browser/system permission prompts remain platform-owned.</x:v>
       </x:c>
       <x:c r="K46" s="6" t="str">
-        <x:v>Software release evidence; hardware and human gates remain separate.</x:v>
+        <x:v>Existing Xbox focus and Quest spatial menus are implemented. Current Tidelight adds browser DOM controls but its IDs are absent from the Quest settings list in dominion-controls.js. Full water-settings and close/back parity remains open; historical controller tests do not cover those new controls.</x:v>
       </x:c>
       <x:c r="L46" s="6" t="str">
         <x:v>dominion-controls.js
-tests/dominions-browser.py</x:v>
+tests/dominions-browser.py
+tidelight.js
+CONTINUATION-AUDIT.md</x:v>
       </x:c>
       <x:c r="M46" s="6" t="str">
         <x:v>0.7.0</x:v>
@@ -3128,12 +3274,12 @@
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/pilgrim-save.js</x:v>
       </x:c>
     </x:row>
-    <x:row r="53" ht="124" customHeight="1">
+    <x:row r="53" ht="134" customHeight="1">
       <x:c r="A53" s="6" t="str">
         <x:v>V48</x:v>
       </x:c>
       <x:c r="B53" s="6" t="str">
-        <x:v>Versioned production board and six-sheet workbook</x:v>
+        <x:v>Synchronized canonical production board, six-sheet workbook and cross-chat handoff</x:v>
       </x:c>
       <x:c r="C53" s="6" t="str">
         <x:v>Implemented</x:v>
@@ -3157,20 +3303,22 @@
         <x:v>Make each release close a measurable gap and keep the long-term path inspectable.</x:v>
       </x:c>
       <x:c r="J53" s="6" t="str">
-        <x:v>roadmap.json is canonical; board and workbook show priority, dependencies, owner role, evidence and exit gates. Local edits are clearly separate from committed status.</x:v>
+        <x:v>Keep roadmap.json version aligned with release.json and core.js. Preserve V01-V76; export the six-sheet workbook with matching source digest and live summary formulas. Keep DEVELOPMENT-HANDOFF.md and CONTINUATION-AUDIT.md linked from the board and README. Verify committed files, not browser-local edits.</x:v>
       </x:c>
       <x:c r="K53" s="6" t="str">
-        <x:v>Software release evidence; hardware and human gates remain separate.</x:v>
+        <x:v>September 13 repairs both the stale plan/workbook and the core diagnostic version label, without changing mechanics or save formats. Historical acceptance had 148 model passes and one plan-version failure; fresh checks are recorded separately. Physical/human gates remain open.</x:v>
       </x:c>
       <x:c r="L53" s="6" t="str">
         <x:v>roadmap.json
 roadmap.html
 AAA-PRODUCTION.xlsx
 tests/production.test.cjs
-tests/production-browser.py</x:v>
+tests/production-browser.py
+DEVELOPMENT-HANDOFF.md
+CONTINUATION-AUDIT.md</x:v>
       </x:c>
       <x:c r="M53" s="6" t="str">
-        <x:v>0.9.0</x:v>
+        <x:v>0.9.0 foundation; 0.12.0 planning synchronization</x:v>
       </x:c>
       <x:c r="N53" s="6" t="str">
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
@@ -3314,7 +3462,7 @@
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/oath-model.js</x:v>
       </x:c>
     </x:row>
-    <x:row r="57" ht="124" customHeight="1">
+    <x:row r="57" ht="162" customHeight="1">
       <x:c r="A57" s="6" t="str">
         <x:v>V52</x:v>
       </x:c>
@@ -3343,7 +3491,7 @@
         <x:v>Replace sheer room count with deliberately paced exploration.</x:v>
       </x:c>
       <x:c r="J57" s="6" t="str">
-        <x:v>One polished 20-30 minute target route mixes safe introduction, alternate approach, escalating encounter, discovery and boss payoff. Validate every traversal connector and recovery path. Duration is a design target, not measured content.</x:v>
+        <x:v>One polished 20-30 minute target route mixes safe introduction, alternate approach, escalating encounter, discovery and boss payoff. Validate every traversal connector and recovery path. Duration is a design target, not measured content. Preserve multi-level gothic sightlines and multiple approaches. Plan selective water-adjacent discoveries with purpose; the present water layer does not create new navigable rooms.</x:v>
       </x:c>
       <x:c r="K57" s="6" t="str">
         <x:v>A connected Roseglass/Ivory Crown/Ember Crown progression reuses the collision-tested 25-room world, existing stairs and alternate approaches. Three staged courts are implemented; the proposed 20-30 minute polished duration and authored connector variety are not yet measured or complete.</x:v>
@@ -3351,7 +3499,8 @@
       <x:c r="L57" s="6" t="str">
         <x:v>oath-model.js
 first-bell.js
-tests/oath.test.cjs</x:v>
+tests/oath.test.cjs
+CONTINUATION-AUDIT.md</x:v>
       </x:c>
       <x:c r="M57" s="6" t="str">
         <x:v>0.10.0 First Bell</x:v>
@@ -3400,7 +3549,7 @@
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
       </x:c>
     </x:row>
-    <x:row r="59" ht="124" customHeight="1">
+    <x:row r="59" ht="162" customHeight="1">
       <x:c r="A59" s="6" t="str">
         <x:v>V54</x:v>
       </x:c>
@@ -3429,15 +3578,17 @@
         <x:v>Foreground and character quality must catch up with the architecture.</x:v>
       </x:c>
       <x:c r="J59" s="6" t="str">
-        <x:v>Produce consistent original/licensed meshes, LODs, rigs and materials for one complete vertical slice; registered provenance; review both eye views and close-range silhouette.</x:v>
+        <x:v>Produce consistent original/licensed meshes, LODs, rigs and materials for one complete vertical slice; registered provenance; review both eye views and close-range silhouette. Retain the 15 existing archetypes, including the 12 added outer enemy orders. Improve humanoid/knight silhouettes and counterplay; do not restart the already delivered numerical expansion or copy commercial reference assets.</x:v>
       </x:c>
       <x:c r="K59" s="6" t="str">
         <x:v>Not closed; no completion credit without gate evidence.</x:v>
       </x:c>
-      <x:c r="L59" s="6" t="str"/>
+      <x:c r="L59" s="6" t="str">
+        <x:v>CONTINUATION-AUDIT.md</x:v>
+      </x:c>
       <x:c r="M59" s="6" t="str"/>
       <x:c r="N59" s="6" t="str">
-        <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
+        <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/CONTINUATION-AUDIT.md</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="124" customHeight="1">
@@ -3560,12 +3711,12 @@
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
       </x:c>
     </x:row>
-    <x:row r="63" ht="124" customHeight="1">
+    <x:row r="63" ht="162" customHeight="1">
       <x:c r="A63" s="6" t="str">
         <x:v>V58</x:v>
       </x:c>
       <x:c r="B63" s="6" t="str">
-        <x:v>Long-session headphone mix and notification-rate controls</x:v>
+        <x:v>Production sound/music pass, water acoustics and long-session clarity</x:v>
       </x:c>
       <x:c r="C63" s="6" t="str">
         <x:v>Planned</x:v>
@@ -3586,18 +3737,22 @@
         <x:v>V43, V44, V50</x:v>
       </x:c>
       <x:c r="I63" s="6" t="str">
-        <x:v>Bounded voices alone do not guarantee pleasant sound.</x:v>
+        <x:v>The user explicitly prioritizes much stronger in-game sound and music; precise archery also needs audible material identity and readable threat direction.</x:v>
       </x:c>
       <x:c r="J63" s="6" t="str">
-        <x:v>Add independent notification density/rate controls; test 30-minute sessions with music transitions, simultaneous threats and repeated UI actions. Record human mix feedback and remove tiring repetition.</x:v>
+        <x:v>Improve bow tension/release, crossbow winding/reload, arrow material impacts, shield impact/break, distinct enemy warnings, bells/wind, footsteps, water entries/splashes/drips and room ambience. Add restrained exploration/pressure/recovery/boss transitions; preserve independent buses, mute, captions, quiet mix, controller access and voice budgets. Pass PCM/lifecycle tests and a dated 30-minute human headphone review.</x:v>
       </x:c>
       <x:c r="K63" s="6" t="str">
-        <x:v>Not closed; no completion credit without gate evidence.</x:v>
-      </x:c>
-      <x:c r="L63" s="6" t="str"/>
+        <x:v>Planned production pass. Resonant Hunt audio exists; current tidelight.js does not wire water-specific sounds. Earlier draft descriptions of positional water splashes/footsteps are not shipped evidence.</x:v>
+      </x:c>
+      <x:c r="L63" s="6" t="str">
+        <x:v>RESONANT-HUNT.md
+tidelight.js
+CONTINUATION-AUDIT.md</x:v>
+      </x:c>
       <x:c r="M63" s="6" t="str"/>
       <x:c r="N63" s="6" t="str">
-        <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
+        <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/RESONANT-HUNT.md</x:v>
       </x:c>
     </x:row>
     <x:row r="64" ht="124" customHeight="1">
@@ -3680,7 +3835,7 @@
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
       </x:c>
     </x:row>
-    <x:row r="66" ht="124" customHeight="1">
+    <x:row r="66" ht="162" customHeight="1">
       <x:c r="A66" s="6" t="str">
         <x:v>V61</x:v>
       </x:c>
@@ -3709,15 +3864,17 @@
         <x:v>Different bodies and play spaces need more than a handedness toggle.</x:v>
       </x:c>
       <x:c r="J66" s="6" t="str">
-        <x:v>Configurable action mapping with conflict checks, seated/standing height and reach calibration, turn/motion presets and readable UI. Each can be reset without a mouse.</x:v>
+        <x:v>Configurable action mapping with conflict checks, seated/standing height and reach calibration, turn/motion presets and readable UI. Each can be reset without a mouse. Resolve grip-role conflicts by documenting the current bow-hand shard/free-hand shield mapping; implement physical thrown shards under V24, not an undocumented remap. Cover every new water/audio panel in controller-only tests.</x:v>
       </x:c>
       <x:c r="K66" s="6" t="str">
         <x:v>Not closed; no completion credit without gate evidence.</x:v>
       </x:c>
-      <x:c r="L66" s="6" t="str"/>
+      <x:c r="L66" s="6" t="str">
+        <x:v>CONTINUATION-AUDIT.md</x:v>
+      </x:c>
       <x:c r="M66" s="6" t="str"/>
       <x:c r="N66" s="6" t="str">
-        <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
+        <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/CONTINUATION-AUDIT.md</x:v>
       </x:c>
     </x:row>
     <x:row r="67" ht="124" customHeight="1">
@@ -3760,7 +3917,7 @@
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
       </x:c>
     </x:row>
-    <x:row r="68" ht="124" customHeight="1">
+    <x:row r="68" ht="190" customHeight="1">
       <x:c r="A68" s="6" t="str">
         <x:v>V63</x:v>
       </x:c>
@@ -3789,15 +3946,17 @@
         <x:v>Threats and menus must remain readable beyond one ideal user.</x:v>
       </x:c>
       <x:c r="J68" s="6" t="str">
-        <x:v>Text size/contrast, sound direction captions, color-independent ammunition/enemy signals and reduced-flash mode survive desktop, stereo and passthrough contexts. Human accessibility review required.</x:v>
+        <x:v>Text size/contrast, sound direction captions, color-independent ammunition/enemy signals and reduced-flash mode survive desktop, stereo and passthrough contexts. Human accessibility review required. Preserve the palm-familiar, diegetic status design for VR and supported accessibility fallbacks. The user requested discrete hit points rather than a bar; the existing numerical health model and desktop HUD are a recorded design gap, not authorization to silently change save semantics.</x:v>
       </x:c>
       <x:c r="K68" s="6" t="str">
         <x:v>Not closed; no completion credit without gate evidence.</x:v>
       </x:c>
-      <x:c r="L68" s="6" t="str"/>
+      <x:c r="L68" s="6" t="str">
+        <x:v>CONTINUATION-AUDIT.md</x:v>
+      </x:c>
       <x:c r="M68" s="6" t="str"/>
       <x:c r="N68" s="6" t="str">
-        <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
+        <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/CONTINUATION-AUDIT.md</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="124" customHeight="1">
@@ -3840,7 +3999,7 @@
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
       </x:c>
     </x:row>
-    <x:row r="70" ht="124" customHeight="1">
+    <x:row r="70" ht="148" customHeight="1">
       <x:c r="A70" s="6" t="str">
         <x:v>V65</x:v>
       </x:c>
@@ -3869,7 +4028,7 @@
         <x:v>A published game needs durable progress across later upgrades.</x:v>
       </x:c>
       <x:c r="J70" s="6" t="str">
-        <x:v>Keep fixtures for old supported generator/schema versions, offer explicit local backup/restore and verify interrupted writes, browser quota and update migration. Never silently reset incompatible saves.</x:v>
+        <x:v>Keep fixtures for old supported generator/schema versions, offer explicit local backup/restore and verify interrupted writes, browser quota and update migration. Never silently reset incompatible saves. Any future discrete-hit-point conversion must specify health/healing balance and tested checkpoint migration; retain current health and profiles in presentation-only releases.</x:v>
       </x:c>
       <x:c r="K70" s="6" t="str">
         <x:v>Not closed; no completion credit without gate evidence.</x:v>
@@ -3880,7 +4039,7 @@
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
       </x:c>
     </x:row>
-    <x:row r="71" ht="124" customHeight="1">
+    <x:row r="71" ht="176" customHeight="1">
       <x:c r="A71" s="6" t="str">
         <x:v>V66</x:v>
       </x:c>
@@ -3909,15 +4068,17 @@
         <x:v>Finite smoke tests are not a complete campaign quality gate.</x:v>
       </x:c>
       <x:c r="J71" s="6" t="str">
-        <x:v>Run at least 1000 proposed seed/depth fixtures and 50 lifecycle transitions, tracking unreachable rewards, spawning collisions, NaNs, leaks and progress duplication. Publish failures and seed repros.</x:v>
+        <x:v>Run at least 1000 proposed seed/depth fixtures and 50 lifecycle transitions, tracking unreachable rewards, spawning collisions, NaNs, leaks and progress duplication. Publish failures and seed repros. Add dedicated Tidelight tests for pool placement across depth/seed, standing on high walks above water, actual arrow-water crossings, paused/reduced-effects motion, sector clock resets, AR return and old-save continuation.</x:v>
       </x:c>
       <x:c r="K71" s="6" t="str">
         <x:v>Not closed; no completion credit without gate evidence.</x:v>
       </x:c>
-      <x:c r="L71" s="6" t="str"/>
+      <x:c r="L71" s="6" t="str">
+        <x:v>CONTINUATION-AUDIT.md</x:v>
+      </x:c>
       <x:c r="M71" s="6" t="str"/>
       <x:c r="N71" s="6" t="str">
-        <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
+        <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/CONTINUATION-AUDIT.md</x:v>
       </x:c>
     </x:row>
     <x:row r="72" ht="124" customHeight="1">
@@ -3960,7 +4121,7 @@
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
       </x:c>
     </x:row>
-    <x:row r="73" ht="124" customHeight="1">
+    <x:row r="73" ht="190" customHeight="1">
       <x:c r="A73" s="6" t="str">
         <x:v>V68</x:v>
       </x:c>
@@ -3989,14 +4150,15 @@
         <x:v>Do not confuse a merged commit with a complete verified release.</x:v>
       </x:c>
       <x:c r="J73" s="6" t="str">
-        <x:v>Byte-verified deployment already exists. Add explicit stable/candidate policy, save-safe rollback drill, reproducible asset pipeline and release-note/device-evidence review.</x:v>
+        <x:v>For every finished upgrade, test the actual scoped source, commit and merge without overwriting sibling games, verify GitHub Pages deployment plus public runtime/asset/plan/workbook bytes, then launch the public game. Separate source, test, deployment, hardware and human evidence. Retry transient GitHub faults with backoff; inspect failed jobs instead of polling an unchanged failure list. Preserve explicit rollback and save-compatibility notes.</x:v>
       </x:c>
       <x:c r="K73" s="6" t="str">
-        <x:v>Not closed; no completion credit without gate evidence.</x:v>
+        <x:v>Partial. Tidelight was published, but archived run 34737842771 stopped before browser checks because roadmap 0.11.0 disagreed with release 0.12.0. This planning repair fixes that mismatch; it does not retrospectively turn skipped gameplay acceptance green.</x:v>
       </x:c>
       <x:c r="L73" s="6" t="str">
         <x:v>tests/verify-live.py
-tests/launch.py</x:v>
+tests/launch.py
+CONTINUATION-AUDIT.md</x:v>
       </x:c>
       <x:c r="M73" s="6" t="str"/>
       <x:c r="N73" s="6" t="str">
@@ -4203,7 +4365,7 @@
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
       </x:c>
     </x:row>
-    <x:row r="79" ht="124" customHeight="1">
+    <x:row r="79" ht="190" customHeight="1">
       <x:c r="A79" s="6" t="str">
         <x:v>V74</x:v>
       </x:c>
@@ -4232,15 +4394,19 @@
         <x:v>Repeated additive patches increase the risk of hidden lifecycle regressions.</x:v>
       </x:c>
       <x:c r="J79" s="6" t="str">
-        <x:v>Reduce wrapper-order coupling with explicit lifecycle interfaces and dependency tests; preserve current save fixtures, deterministic physics and controller mappings.</x:v>
+        <x:v>Reduce wrapper-order coupling with explicit lifecycle interfaces and dependency tests; preserve current save fixtures, deterministic physics and controller mappings. Audit current Tidelight: maxRipples is declared by policy but tick uploads all 10 slots; rebuild does not clear ripple timestamps/lastStep; inside() does not match the rendered inset; impact and footstep splash checks omit height. Treat these as source-review findings needing reproductions and tests, not fixes already shipped.</x:v>
       </x:c>
       <x:c r="K79" s="6" t="str">
         <x:v>Not closed; no completion credit without gate evidence.</x:v>
       </x:c>
-      <x:c r="L79" s="6" t="str"/>
+      <x:c r="L79" s="6" t="str">
+        <x:v>tidelight.js
+tidelight-shaders.js
+CONTINUATION-AUDIT.md</x:v>
+      </x:c>
       <x:c r="M79" s="6" t="str"/>
       <x:c r="N79" s="6" t="str">
-        <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
+        <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/tidelight.js</x:v>
       </x:c>
     </x:row>
     <x:row r="80" ht="124" customHeight="1">
@@ -4382,7 +4548,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Redb18996740d4745"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdadc18230c054e81"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4479,13 +4645,13 @@
         <x:v>Playable foundations</x:v>
       </x:c>
       <x:c r="C6" s="6" t="str">
-        <x:v>Implemented</x:v>
+        <x:v>Partial</x:v>
       </x:c>
       <x:c r="D6" s="6" t="str">
         <x:v>None</x:v>
       </x:c>
       <x:c r="E6" s="6" t="str">
-        <x:v>Retain the shipped original browser/VR/AR foundation.</x:v>
+        <x:v>Retain shipped browser/VR/AR foundations and close the newest water-interface and release-evidence gaps.</x:v>
       </x:c>
       <x:c r="F6" s="6" t="str">
         <x:v>Current foundation and input/model/public deployment tests pass; hardware acceptance is not implied.</x:v>
@@ -4496,7 +4662,7 @@
       </x:c>
       <x:c r="H6" s="18" t="n">
         <x:f>COUNTIFS(Backlog!$E$6:$E$81,A6,Backlog!$C$6:$C$81,"Implemented")</x:f>
-        <x:v>32</x:v>
+        <x:v>31</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="112" customHeight="1">
@@ -4684,7 +4850,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0a9104c7460b48cc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R590db8259c084bda"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5049,31 +5215,74 @@
       <x:c r="I15" s="20"/>
       <x:c r="J15" s="6"/>
     </x:row>
-    <x:row r="16">
-      <x:c r="A16" s="6"/>
-      <x:c r="B16" s="6"/>
-      <x:c r="C16" s="6"/>
-      <x:c r="D16" s="6"/>
-      <x:c r="E16" s="6"/>
-      <x:c r="F16" s="6"/>
-      <x:c r="G16" s="6"/>
+    <x:row r="16" ht="140" customHeight="1">
+      <x:c r="A16" s="6" t="str">
+        <x:v>Q11</x:v>
+      </x:c>
+      <x:c r="B16" s="6" t="str">
+        <x:v>Quest 3 / Tidelight</x:v>
+      </x:c>
+      <x:c r="C16" s="6" t="str">
+        <x:v>Water and complete spatial settings</x:v>
+      </x:c>
+      <x:c r="D16" s="6" t="str">
+        <x:v>Reach/change/close all water controls; enforce actual ripple/pool budget; verify both eyes, AR exclusion and repeated XR entry/exit</x:v>
+      </x:c>
+      <x:c r="E16" s="6" t="str">
+        <x:v>V38,V41,V62,V74</x:v>
+      </x:c>
+      <x:c r="F16" s="6" t="str">
+        <x:v>Not run</x:v>
+      </x:c>
+      <x:c r="G16" s="6" t="str">
+        <x:v>Record source/build hash and real headset/browser versions. Policy fields alone are not proof that runtime honors the caps.</x:v>
+      </x:c>
       <x:c r="H16" s="6"/>
       <x:c r="I16" s="6"/>
       <x:c r="J16" s="6"/>
+    </x:row>
+    <x:row r="17" ht="140" customHeight="1">
+      <x:c r="A17" s="47" t="str">
+        <x:v>Q12</x:v>
+      </x:c>
+      <x:c r="B17" s="47" t="str">
+        <x:v>Desktop / water and audio</x:v>
+      </x:c>
+      <x:c r="C17" s="47" t="str">
+        <x:v>Source-to-screen/sound parity</x:v>
+      </x:c>
+      <x:c r="D17" s="47" t="str">
+        <x:v>Seed/depth-specific pools, visible stone, caustics, actual impact/footstep positions and music/water mix; no false claim of reflection/refraction</x:v>
+      </x:c>
+      <x:c r="E17" s="47" t="str">
+        <x:v>V35,V58,V66</x:v>
+      </x:c>
+      <x:c r="F17" s="47" t="str">
+        <x:v>Not run</x:v>
+      </x:c>
+      <x:c r="G17" s="47" t="str">
+        <x:v>Archive actual gameplay screenshots and audio receipts. Recovering a draft does not make its features part of the release.</x:v>
+      </x:c>
+      <x:c r="H17" s="47"/>
+      <x:c r="I17" s="47"/>
+      <x:c r="J17" s="47"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:J2"/>
     <x:mergeCell ref="A3:J3"/>
   </x:mergeCells>
-  <x:dataValidations count="1">
+  <x:dataValidations count="2">
     <x:dataValidation type="list" sqref="F6:F15">
       <x:formula1>"Not run,Software only,Passed on device,Failed on device,Blocked"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="F6:F17">
+      <x:formula1>"Not run,Software only,Pass,Fail,Blocked"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R096389eea6dc41da"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf642ba3e03e74a33"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5162,7 +5371,7 @@
         <x:v>Result / evidence receipt</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="110" customHeight="1">
+    <x:row r="6" ht="165" customHeight="1">
       <x:c r="A6" s="6" t="str">
         <x:v>G01</x:v>
       </x:c>
@@ -5173,7 +5382,7 @@
         <x:v>Engineering</x:v>
       </x:c>
       <x:c r="D6" s="6" t="str">
-        <x:v>Only reviewed game paths change; exact source/build is identified; private story excluded.</x:v>
+        <x:v>Only reviewed game paths change; exact source/build is identified; private story excluded. Canonical roadmap version, release version and core version must agree; the workbook must match every task field and the JSON digest.</x:v>
       </x:c>
       <x:c r="E6" s="6" t="str">
         <x:v>tests and repository diff</x:v>
@@ -5210,7 +5419,7 @@
       </x:c>
       <x:c r="H7" s="6"/>
     </x:row>
-    <x:row r="8" ht="110" customHeight="1">
+    <x:row r="8" ht="165" customHeight="1">
       <x:c r="A8" s="6" t="str">
         <x:v>G03</x:v>
       </x:c>
@@ -5221,7 +5430,7 @@
         <x:v>UX / QA</x:v>
       </x:c>
       <x:c r="D8" s="6" t="str">
-        <x:v>Native Xbox and stereo-XR fixtures pass; essential actions have no mouse-only dead end.</x:v>
+        <x:v>Native Xbox and stereo-XR fixtures pass; essential actions have no mouse-only dead end. Include Tidelight water controls and both Quest handedness settings; historical menus alone do not close the expanded UI gate.</x:v>
       </x:c>
       <x:c r="E8" s="6" t="str">
         <x:v>tests/dominions-browser.py</x:v>
@@ -5258,7 +5467,7 @@
       </x:c>
       <x:c r="H9" s="6"/>
     </x:row>
-    <x:row r="10" ht="110" customHeight="1">
+    <x:row r="10" ht="165" customHeight="1">
       <x:c r="A10" s="6" t="str">
         <x:v>G05</x:v>
       </x:c>
@@ -5269,7 +5478,7 @@
         <x:v>Technical art / audio</x:v>
       </x:c>
       <x:c r="D10" s="6" t="str">
-        <x:v>Native WebGL and stereo audio checks pass; no script errors, broken asset loads or repeating hidden-tab backlog.</x:v>
+        <x:v>Native WebGL and stereo audio checks pass; no script errors, broken asset loads or repeating hidden-tab backlog. Dedicated water render/lifecycle and future water-sound evidence are required; do not substitute release text or a successful Pages build.</x:v>
       </x:c>
       <x:c r="E10" s="6" t="str">
         <x:v>tests/resonant-browser.py; tests/jewelglass-browser.py</x:v>
@@ -5419,7 +5628,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0564014c6268424f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb544c8baba314f48"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5664,7 +5873,7 @@
         <x:v>Open</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" ht="100" customHeight="1">
+    <x:row r="12" ht="145" customHeight="1">
       <x:c r="A12" s="6" t="str">
         <x:v>R07</x:v>
       </x:c>
@@ -5678,16 +5887,16 @@
         <x:v>Production</x:v>
       </x:c>
       <x:c r="E12" s="6" t="str">
-        <x:v>Previous board remained at 0.6 after 0.8 shipped</x:v>
+        <x:v>At audit: Tidelight 0.12.0 shipped while roadmap/workbook remained 0.11.0; archived full-model run had one version failure.</x:v>
       </x:c>
       <x:c r="F12" s="6" t="str">
         <x:v>V48</x:v>
       </x:c>
       <x:c r="G12" s="6" t="str">
-        <x:v>Check version consistency and preserve one canonical JSON plus generated workbook snapshot.</x:v>
+        <x:v>Synchronize canonical plan, workbook and resume docs together; run version/digest tests before publication and preserve the historical failure.</x:v>
       </x:c>
       <x:c r="H12" s="6" t="str">
-        <x:v>Mitigated by checks</x:v>
+        <x:v>Open / repair requires release discipline</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="100" customHeight="1">
@@ -5768,15 +5977,57 @@
         <x:v>Open</x:v>
       </x:c>
     </x:row>
-    <x:row r="16">
-      <x:c r="A16" s="6"/>
-      <x:c r="B16" s="6"/>
-      <x:c r="C16" s="6"/>
-      <x:c r="D16" s="6"/>
-      <x:c r="E16" s="6"/>
-      <x:c r="F16" s="6"/>
-      <x:c r="G16" s="6"/>
-      <x:c r="H16" s="6"/>
+    <x:row r="16" ht="150" customHeight="1">
+      <x:c r="A16" s="6" t="str">
+        <x:v>R11</x:v>
+      </x:c>
+      <x:c r="B16" s="6" t="str">
+        <x:v>Interrupted draft mistaken for published features</x:v>
+      </x:c>
+      <x:c r="C16" s="6" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="D16" s="6" t="str">
+        <x:v>Production / engineering</x:v>
+      </x:c>
+      <x:c r="E16" s="6" t="str">
+        <x:v>The larger water draft described seven surfaces, named extra areas, basin refraction, reflections and sounds absent from current Tidelight source.</x:v>
+      </x:c>
+      <x:c r="F16" s="6" t="str">
+        <x:v>V35,V58,V68</x:v>
+      </x:c>
+      <x:c r="G16" s="6" t="str">
+        <x:v>Inspect current source first; preserve draft intent as future work and do not replay opaque transfer chunks over master.</x:v>
+      </x:c>
+      <x:c r="H16" s="6" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="150" customHeight="1">
+      <x:c r="A17" s="47" t="str">
+        <x:v>R12</x:v>
+      </x:c>
+      <x:c r="B17" s="47" t="str">
+        <x:v>Water policy/lifecycle implementation differs from its intent</x:v>
+      </x:c>
+      <x:c r="C17" s="47" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="D17" s="47" t="str">
+        <x:v>Engineering / technical art</x:v>
+      </x:c>
+      <x:c r="E17" s="47" t="str">
+        <x:v>Ripple-cap, world-clock reset, footprint and height checks need dedicated tests; water controls missing from XR list.</x:v>
+      </x:c>
+      <x:c r="F17" s="47" t="str">
+        <x:v>V38,V41,V66,V74</x:v>
+      </x:c>
+      <x:c r="G17" s="47" t="str">
+        <x:v>Reproduce each finding and add small save-safe fixes with real-frame and controller evidence.</x:v>
+      </x:c>
+      <x:c r="H17" s="47" t="str">
+        <x:v>Open</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -5795,7 +6046,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8e54c835d1604ee7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R83db27770ff14a3a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Synchronize Surestep 0.13.0 release, continuation record and artifact-authored production workbook
</commit_message>
<xml_diff>
--- a/vesperfall/AAA-PRODUCTION.xlsx
+++ b/vesperfall/AAA-PRODUCTION.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="R242c3143bbe74260"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="2" r:id="R59926fb31b304cee"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Milestones" sheetId="3" r:id="R006124efab6c4c9c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Device QA" sheetId="4" r:id="R4ba785b8f0b94f51"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="5" r:id="R00e8525b5cfb4e32"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risk Register" sheetId="6" r:id="Re505e8c2936744b2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="Rdd6885be96804f48"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="2" r:id="R082cd50e961f428b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Milestones" sheetId="3" r:id="Ra681cf1889c64316"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Device QA" sheetId="4" r:id="Rf69a3bbb99bb462a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="5" r:id="R6784a3c53166430d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risk Register" sheetId="6" r:id="R5f77ef7909194d03"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -628,7 +628,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="12" t="str">
-        <x:v>v0.12.0 / Tidelight / planning audit 2026-09-13. Roadmap, workbook and core diagnostic version labels are synchronized; gameplay mechanics and save formats are unchanged.</x:v>
+        <x:v>v0.13.0 / Surestep / 2026-09-14. Fast Xbox arrow selection, Quest water settings and tracked-hand menus, and procedural humanoid foot planting. Existing save formats and simulation remain unchanged.</x:v>
       </x:c>
       <x:c r="B3" s="12"/>
       <x:c r="C3" s="12"/>
@@ -774,7 +774,7 @@
     </x:row>
     <x:row r="15" ht="24" customHeight="1">
       <x:c r="A15" s="6" t="str">
-        <x:v>Shipped water is the bounded translucent-plane baseline. The earlier detailed basin/refraction/reflection/audio draft is not the published implementation. Read the continuation audit before promising or recovering those features.</x:v>
+        <x:v>Surestep closes the bounded missing Quest water-settings item. Humanoid IK is a procedural foundation, not finished production art. The older basin/reflection/audio draft remains unshipped; water lifecycle findings remain open.</x:v>
       </x:c>
       <x:c r="B15" s="6"/>
       <x:c r="C15" s="6"/>
@@ -838,7 +838,7 @@
     </x:row>
     <x:row r="21" ht="24" customHeight="1">
       <x:c r="A21" s="6" t="str">
-        <x:v>Next: establish Tidelight browser/render/save evidence, close Quest water-menu and lifecycle gaps, then prioritize the requested sound/music pass and purposeful exploration. Keep all physical-device and human gates open until measured.</x:v>
+        <x:v>Next: water lifecycle/budget hardening, the requested sound/music pass, physical controller/hand-tracking review and purposeful exploration. Broad accessibility and production-art tasks remain Partial or open.</x:v>
       </x:c>
       <x:c r="B21" s="6"/>
       <x:c r="C21" s="6"/>
@@ -870,7 +870,7 @@
     </x:row>
     <x:row r="24" ht="24" customHeight="1">
       <x:c r="A24" s="6" t="str">
-        <x:v>Historical acceptance: 148 model passes, 1 stale-plan failure; browser steps skipped. Fresh planning checks are separate. No invented hardware approval, staffing, dates, budget, playtime or AAA rating is included.</x:v>
+        <x:v>Surestep adds 17 deterministic tests (170 total at initial local review) plus a rendered Xbox/controller/hand-joint journey. Use the exact workflow artifacts for acceptance and publication status. No physical-device or human approval is implied.</x:v>
       </x:c>
       <x:c r="B24" s="6"/>
       <x:c r="C24" s="6"/>
@@ -902,7 +902,7 @@
     </x:row>
     <x:row r="27" ht="24" customHeight="1">
       <x:c r="A27" s="34" t="str">
-        <x:v>Canonical JSON SHA-256: 8d31f942c3913354082adef2f0034cedd120b367a19964acaf3186feecc77a98</x:v>
+        <x:v>Canonical JSON SHA-256: 382ce526249c7e8b10748abb72a92780f9d3c331bc77773da4c974e462640608</x:v>
       </x:c>
       <x:c r="B27" s="34"/>
       <x:c r="C27" s="34"/>
@@ -1805,7 +1805,7 @@
         <x:v>Presentation</x:v>
       </x:c>
       <x:c r="G19" s="6" t="str">
-        <x:v>Art / audio / assignment pending</x:v>
+        <x:v>Art / audio</x:v>
       </x:c>
       <x:c r="H19" s="6" t="str">
         <x:v>None</x:v>
@@ -1817,11 +1817,15 @@
         <x:v>Spatial sound, reflective equipment and readable procedural creatures exist. Authored rigged enemy/hand assets, animation blending and polished reactions remain open.</x:v>
       </x:c>
       <x:c r="K19" s="6" t="str">
-        <x:v>Audio and procedural art implemented; character-production and human-review gates open.</x:v>
+        <x:v>Surestep adds articulated procedural knees/elbows, distance-driven steps and world-space foot planting for the 12 outer humanoid archetypes. Fixed-length IK and reset/freeze cases have model coverage. Authored production meshes, mocap/blending, hit reactions and human art review remain open.</x:v>
       </x:c>
       <x:c r="L19" s="6" t="str">
         <x:v>resonance-audio.js
-dominion-art.js</x:v>
+dominion-art.js
+surestep-art.js
+surestep-model.js
+tests/surestep.test.cjs
+SURESTEP.md</x:v>
       </x:c>
       <x:c r="M19" s="6" t="str"/>
       <x:c r="N19" s="6" t="str">
@@ -2972,7 +2976,7 @@
         <x:v>Comfort</x:v>
       </x:c>
       <x:c r="G46" s="6" t="str">
-        <x:v>UX / accessibility / assignment pending</x:v>
+        <x:v>UX / accessibility</x:v>
       </x:c>
       <x:c r="H46" s="6" t="str">
         <x:v>V07</x:v>
@@ -2984,13 +2988,14 @@
         <x:v>Every gameplay and game-owned UI path, including water settings, confirmations, recovery, seed entry, audio and accessibility settings, is reachable and dismissible with Xbox and Quest controls without a mouse. Test both handedness modes, neutral-input transitions and return focus. Browser/system permission prompts remain platform-owned.</x:v>
       </x:c>
       <x:c r="K46" s="6" t="str">
-        <x:v>Existing Xbox focus and Quest spatial menus are implemented. Current Tidelight adds browser DOM controls but its IDs are absent from the Quest settings list in dominion-controls.js. Full water-settings and close/back parity remains open; historical controller tests do not cover those new controls.</x:v>
+        <x:v>Surestep implements the missing paginated Quest water settings and adds optional tracked-hand ray/pinch menu input. Xbox down selects Blink and left cycles stocked, unlocked damage arrows outside menus/quiver. Tracking loss, held-pinch acquisition and controller handover are explicit software gates in tests/surestep-browser.py. Full accessibility/remapping and physical-device approval remain open.</x:v>
       </x:c>
       <x:c r="L46" s="6" t="str">
         <x:v>dominion-controls.js
+quest-hands.js
+tests/surestep-browser.py
 tests/dominions-browser.py
-tidelight.js
-CONTINUATION-AUDIT.md</x:v>
+SURESTEP.md</x:v>
       </x:c>
       <x:c r="M46" s="6" t="str">
         <x:v>0.7.0</x:v>
@@ -3557,7 +3562,7 @@
         <x:v>Original rigged enemy, bow-hand and shield production assets</x:v>
       </x:c>
       <x:c r="C59" s="6" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Partial</x:v>
       </x:c>
       <x:c r="D59" s="6" t="str">
         <x:v>P0</x:v>
@@ -3569,7 +3574,7 @@
         <x:v>Art</x:v>
       </x:c>
       <x:c r="G59" s="6" t="str">
-        <x:v>Technical art / assignment pending</x:v>
+        <x:v>Technical art</x:v>
       </x:c>
       <x:c r="H59" s="6" t="str">
         <x:v>V14, V50</x:v>
@@ -3581,10 +3586,14 @@
         <x:v>Produce consistent original/licensed meshes, LODs, rigs and materials for one complete vertical slice; registered provenance; review both eye views and close-range silhouette. Retain the 15 existing archetypes, including the 12 added outer enemy orders. Improve humanoid/knight silhouettes and counterplay; do not restart the already delivered numerical expansion or copy commercial reference assets.</x:v>
       </x:c>
       <x:c r="K59" s="6" t="str">
-        <x:v>Not closed; no completion credit without gate evidence.</x:v>
+        <x:v>Original procedural humanoids now have two-bone legs, articulated arms, smaller helmets and less oversized torsos. Movement drives foot contact and terrain sampling; no hitbox changes. This is a procedural animation foundation, not a completed production mesh/LOD/retargeting pipeline.</x:v>
       </x:c>
       <x:c r="L59" s="6" t="str">
-        <x:v>CONTINUATION-AUDIT.md</x:v>
+        <x:v>dominion-art.js
+surestep-art.js
+surestep-model.js
+tests/surestep.test.cjs
+SURESTEP.md</x:v>
       </x:c>
       <x:c r="M59" s="6" t="str"/>
       <x:c r="N59" s="6" t="str">
@@ -3855,7 +3864,7 @@
         <x:v>Comfort</x:v>
       </x:c>
       <x:c r="G66" s="6" t="str">
-        <x:v>UX / accessibility / assignment pending</x:v>
+        <x:v>UX / accessibility</x:v>
       </x:c>
       <x:c r="H66" s="6" t="str">
         <x:v>V49, V41</x:v>
@@ -3867,10 +3876,12 @@
         <x:v>Configurable action mapping with conflict checks, seated/standing height and reach calibration, turn/motion presets and readable UI. Each can be reset without a mouse. Resolve grip-role conflicts by documenting the current bow-hand shard/free-hand shield mapping; implement physical thrown shards under V24, not an undocumented remap. Cover every new water/audio panel in controller-only tests.</x:v>
       </x:c>
       <x:c r="K66" s="6" t="str">
-        <x:v>Not closed; no completion credit without gate evidence.</x:v>
+        <x:v>Water controls and both handedness choices are exposed to tracked controllers and tracked-hand UI. Full rebinding/conflict checking, seated/reach calibration and hardware comfort presets remain unimplemented.</x:v>
       </x:c>
       <x:c r="L66" s="6" t="str">
-        <x:v>CONTINUATION-AUDIT.md</x:v>
+        <x:v>dominion-controls.js
+quest-hands.js
+SURESTEP.md</x:v>
       </x:c>
       <x:c r="M66" s="6" t="str"/>
       <x:c r="N66" s="6" t="str">
@@ -4141,7 +4152,7 @@
         <x:v>Foundation</x:v>
       </x:c>
       <x:c r="G73" s="6" t="str">
-        <x:v>Engineering / assignment pending</x:v>
+        <x:v>Engineering</x:v>
       </x:c>
       <x:c r="H73" s="6" t="str">
         <x:v>V48, V65</x:v>
@@ -4153,11 +4164,13 @@
         <x:v>For every finished upgrade, test the actual scoped source, commit and merge without overwriting sibling games, verify GitHub Pages deployment plus public runtime/asset/plan/workbook bytes, then launch the public game. Separate source, test, deployment, hardware and human evidence. Retry transient GitHub faults with backoff; inspect failed jobs instead of polling an unchanged failure list. Preserve explicit rollback and save-compatibility notes.</x:v>
       </x:c>
       <x:c r="K73" s="6" t="str">
-        <x:v>Partial. Tidelight was published, but archived run 34737842771 stopped before browser checks because roadmap 0.11.0 disagreed with release 0.12.0. This planning repair fixes that mismatch; it does not retrospectively turn skipped gameplay acceptance green.</x:v>
+        <x:v>Surestep has a dedicated source/browser acceptance workflow and public byte verification. Final per-run receipts distinguish tested source, merged publication and hardware review. The older failed Tidelight run remains historical evidence and is not retroactively credited.</x:v>
       </x:c>
       <x:c r="L73" s="6" t="str">
         <x:v>tests/verify-live.py
+tests/surestep-browser.py
 tests/launch.py
+SURESTEP.md
 CONTINUATION-AUDIT.md</x:v>
       </x:c>
       <x:c r="M73" s="6" t="str"/>
@@ -4548,7 +4561,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdadc18230c054e81"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf3469a0f7e5c4856"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4850,7 +4863,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R590db8259c084bda"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbc2a63471cca4f66"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5282,7 +5295,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf642ba3e03e74a33"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R024be00c2b374b71"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5628,7 +5641,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb544c8baba314f48"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R488444541fd6446e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6046,7 +6059,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R83db27770ff14a3a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9643fc5ebe3d4a56"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Release Vesperfall 0.13.0 Surestep: quick arrows, planted humanoid gait and Quest hand-menu UI
Scoped source from 8518d7f808376923b87bb09193728e4509a6ad4e. Preserve concurrent master c044d8c3a742e83d176bd52c0ba95a33b000c7bd and all sibling games. No save schema, generator, combat or hitbox changes.

170 model tests and canonical six-sheet/76-task workbook checks pass. Existing Dominions 26-check Xbox/VR/AR and Pilgrim 37-check save/recovery browser journeys passed in run 34939761064. Final Surestep hand-menu browser acceptance runs in 34942891520; publication workflow compares live bytes and repeats actual input/launch acceptance. Physical Quest 3 and Xbox certification remain open.

No temporary source transport files or write-enabled staging workflows enter master.
</commit_message>
<xml_diff>
--- a/vesperfall/AAA-PRODUCTION.xlsx
+++ b/vesperfall/AAA-PRODUCTION.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="R242c3143bbe74260"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="2" r:id="R59926fb31b304cee"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Milestones" sheetId="3" r:id="R006124efab6c4c9c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Device QA" sheetId="4" r:id="R4ba785b8f0b94f51"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="5" r:id="R00e8525b5cfb4e32"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risk Register" sheetId="6" r:id="Re505e8c2936744b2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="Rdd6885be96804f48"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="2" r:id="R082cd50e961f428b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Milestones" sheetId="3" r:id="Ra681cf1889c64316"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Device QA" sheetId="4" r:id="Rf69a3bbb99bb462a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="5" r:id="R6784a3c53166430d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risk Register" sheetId="6" r:id="R5f77ef7909194d03"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -628,7 +628,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="12" t="str">
-        <x:v>v0.12.0 / Tidelight / planning audit 2026-09-13. Roadmap, workbook and core diagnostic version labels are synchronized; gameplay mechanics and save formats are unchanged.</x:v>
+        <x:v>v0.13.0 / Surestep / 2026-09-14. Fast Xbox arrow selection, Quest water settings and tracked-hand menus, and procedural humanoid foot planting. Existing save formats and simulation remain unchanged.</x:v>
       </x:c>
       <x:c r="B3" s="12"/>
       <x:c r="C3" s="12"/>
@@ -774,7 +774,7 @@
     </x:row>
     <x:row r="15" ht="24" customHeight="1">
       <x:c r="A15" s="6" t="str">
-        <x:v>Shipped water is the bounded translucent-plane baseline. The earlier detailed basin/refraction/reflection/audio draft is not the published implementation. Read the continuation audit before promising or recovering those features.</x:v>
+        <x:v>Surestep closes the bounded missing Quest water-settings item. Humanoid IK is a procedural foundation, not finished production art. The older basin/reflection/audio draft remains unshipped; water lifecycle findings remain open.</x:v>
       </x:c>
       <x:c r="B15" s="6"/>
       <x:c r="C15" s="6"/>
@@ -838,7 +838,7 @@
     </x:row>
     <x:row r="21" ht="24" customHeight="1">
       <x:c r="A21" s="6" t="str">
-        <x:v>Next: establish Tidelight browser/render/save evidence, close Quest water-menu and lifecycle gaps, then prioritize the requested sound/music pass and purposeful exploration. Keep all physical-device and human gates open until measured.</x:v>
+        <x:v>Next: water lifecycle/budget hardening, the requested sound/music pass, physical controller/hand-tracking review and purposeful exploration. Broad accessibility and production-art tasks remain Partial or open.</x:v>
       </x:c>
       <x:c r="B21" s="6"/>
       <x:c r="C21" s="6"/>
@@ -870,7 +870,7 @@
     </x:row>
     <x:row r="24" ht="24" customHeight="1">
       <x:c r="A24" s="6" t="str">
-        <x:v>Historical acceptance: 148 model passes, 1 stale-plan failure; browser steps skipped. Fresh planning checks are separate. No invented hardware approval, staffing, dates, budget, playtime or AAA rating is included.</x:v>
+        <x:v>Surestep adds 17 deterministic tests (170 total at initial local review) plus a rendered Xbox/controller/hand-joint journey. Use the exact workflow artifacts for acceptance and publication status. No physical-device or human approval is implied.</x:v>
       </x:c>
       <x:c r="B24" s="6"/>
       <x:c r="C24" s="6"/>
@@ -902,7 +902,7 @@
     </x:row>
     <x:row r="27" ht="24" customHeight="1">
       <x:c r="A27" s="34" t="str">
-        <x:v>Canonical JSON SHA-256: 8d31f942c3913354082adef2f0034cedd120b367a19964acaf3186feecc77a98</x:v>
+        <x:v>Canonical JSON SHA-256: 382ce526249c7e8b10748abb72a92780f9d3c331bc77773da4c974e462640608</x:v>
       </x:c>
       <x:c r="B27" s="34"/>
       <x:c r="C27" s="34"/>
@@ -1805,7 +1805,7 @@
         <x:v>Presentation</x:v>
       </x:c>
       <x:c r="G19" s="6" t="str">
-        <x:v>Art / audio / assignment pending</x:v>
+        <x:v>Art / audio</x:v>
       </x:c>
       <x:c r="H19" s="6" t="str">
         <x:v>None</x:v>
@@ -1817,11 +1817,15 @@
         <x:v>Spatial sound, reflective equipment and readable procedural creatures exist. Authored rigged enemy/hand assets, animation blending and polished reactions remain open.</x:v>
       </x:c>
       <x:c r="K19" s="6" t="str">
-        <x:v>Audio and procedural art implemented; character-production and human-review gates open.</x:v>
+        <x:v>Surestep adds articulated procedural knees/elbows, distance-driven steps and world-space foot planting for the 12 outer humanoid archetypes. Fixed-length IK and reset/freeze cases have model coverage. Authored production meshes, mocap/blending, hit reactions and human art review remain open.</x:v>
       </x:c>
       <x:c r="L19" s="6" t="str">
         <x:v>resonance-audio.js
-dominion-art.js</x:v>
+dominion-art.js
+surestep-art.js
+surestep-model.js
+tests/surestep.test.cjs
+SURESTEP.md</x:v>
       </x:c>
       <x:c r="M19" s="6" t="str"/>
       <x:c r="N19" s="6" t="str">
@@ -2972,7 +2976,7 @@
         <x:v>Comfort</x:v>
       </x:c>
       <x:c r="G46" s="6" t="str">
-        <x:v>UX / accessibility / assignment pending</x:v>
+        <x:v>UX / accessibility</x:v>
       </x:c>
       <x:c r="H46" s="6" t="str">
         <x:v>V07</x:v>
@@ -2984,13 +2988,14 @@
         <x:v>Every gameplay and game-owned UI path, including water settings, confirmations, recovery, seed entry, audio and accessibility settings, is reachable and dismissible with Xbox and Quest controls without a mouse. Test both handedness modes, neutral-input transitions and return focus. Browser/system permission prompts remain platform-owned.</x:v>
       </x:c>
       <x:c r="K46" s="6" t="str">
-        <x:v>Existing Xbox focus and Quest spatial menus are implemented. Current Tidelight adds browser DOM controls but its IDs are absent from the Quest settings list in dominion-controls.js. Full water-settings and close/back parity remains open; historical controller tests do not cover those new controls.</x:v>
+        <x:v>Surestep implements the missing paginated Quest water settings and adds optional tracked-hand ray/pinch menu input. Xbox down selects Blink and left cycles stocked, unlocked damage arrows outside menus/quiver. Tracking loss, held-pinch acquisition and controller handover are explicit software gates in tests/surestep-browser.py. Full accessibility/remapping and physical-device approval remain open.</x:v>
       </x:c>
       <x:c r="L46" s="6" t="str">
         <x:v>dominion-controls.js
+quest-hands.js
+tests/surestep-browser.py
 tests/dominions-browser.py
-tidelight.js
-CONTINUATION-AUDIT.md</x:v>
+SURESTEP.md</x:v>
       </x:c>
       <x:c r="M46" s="6" t="str">
         <x:v>0.7.0</x:v>
@@ -3557,7 +3562,7 @@
         <x:v>Original rigged enemy, bow-hand and shield production assets</x:v>
       </x:c>
       <x:c r="C59" s="6" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Partial</x:v>
       </x:c>
       <x:c r="D59" s="6" t="str">
         <x:v>P0</x:v>
@@ -3569,7 +3574,7 @@
         <x:v>Art</x:v>
       </x:c>
       <x:c r="G59" s="6" t="str">
-        <x:v>Technical art / assignment pending</x:v>
+        <x:v>Technical art</x:v>
       </x:c>
       <x:c r="H59" s="6" t="str">
         <x:v>V14, V50</x:v>
@@ -3581,10 +3586,14 @@
         <x:v>Produce consistent original/licensed meshes, LODs, rigs and materials for one complete vertical slice; registered provenance; review both eye views and close-range silhouette. Retain the 15 existing archetypes, including the 12 added outer enemy orders. Improve humanoid/knight silhouettes and counterplay; do not restart the already delivered numerical expansion or copy commercial reference assets.</x:v>
       </x:c>
       <x:c r="K59" s="6" t="str">
-        <x:v>Not closed; no completion credit without gate evidence.</x:v>
+        <x:v>Original procedural humanoids now have two-bone legs, articulated arms, smaller helmets and less oversized torsos. Movement drives foot contact and terrain sampling; no hitbox changes. This is a procedural animation foundation, not a completed production mesh/LOD/retargeting pipeline.</x:v>
       </x:c>
       <x:c r="L59" s="6" t="str">
-        <x:v>CONTINUATION-AUDIT.md</x:v>
+        <x:v>dominion-art.js
+surestep-art.js
+surestep-model.js
+tests/surestep.test.cjs
+SURESTEP.md</x:v>
       </x:c>
       <x:c r="M59" s="6" t="str"/>
       <x:c r="N59" s="6" t="str">
@@ -3855,7 +3864,7 @@
         <x:v>Comfort</x:v>
       </x:c>
       <x:c r="G66" s="6" t="str">
-        <x:v>UX / accessibility / assignment pending</x:v>
+        <x:v>UX / accessibility</x:v>
       </x:c>
       <x:c r="H66" s="6" t="str">
         <x:v>V49, V41</x:v>
@@ -3867,10 +3876,12 @@
         <x:v>Configurable action mapping with conflict checks, seated/standing height and reach calibration, turn/motion presets and readable UI. Each can be reset without a mouse. Resolve grip-role conflicts by documenting the current bow-hand shard/free-hand shield mapping; implement physical thrown shards under V24, not an undocumented remap. Cover every new water/audio panel in controller-only tests.</x:v>
       </x:c>
       <x:c r="K66" s="6" t="str">
-        <x:v>Not closed; no completion credit without gate evidence.</x:v>
+        <x:v>Water controls and both handedness choices are exposed to tracked controllers and tracked-hand UI. Full rebinding/conflict checking, seated/reach calibration and hardware comfort presets remain unimplemented.</x:v>
       </x:c>
       <x:c r="L66" s="6" t="str">
-        <x:v>CONTINUATION-AUDIT.md</x:v>
+        <x:v>dominion-controls.js
+quest-hands.js
+SURESTEP.md</x:v>
       </x:c>
       <x:c r="M66" s="6" t="str"/>
       <x:c r="N66" s="6" t="str">
@@ -4141,7 +4152,7 @@
         <x:v>Foundation</x:v>
       </x:c>
       <x:c r="G73" s="6" t="str">
-        <x:v>Engineering / assignment pending</x:v>
+        <x:v>Engineering</x:v>
       </x:c>
       <x:c r="H73" s="6" t="str">
         <x:v>V48, V65</x:v>
@@ -4153,11 +4164,13 @@
         <x:v>For every finished upgrade, test the actual scoped source, commit and merge without overwriting sibling games, verify GitHub Pages deployment plus public runtime/asset/plan/workbook bytes, then launch the public game. Separate source, test, deployment, hardware and human evidence. Retry transient GitHub faults with backoff; inspect failed jobs instead of polling an unchanged failure list. Preserve explicit rollback and save-compatibility notes.</x:v>
       </x:c>
       <x:c r="K73" s="6" t="str">
-        <x:v>Partial. Tidelight was published, but archived run 34737842771 stopped before browser checks because roadmap 0.11.0 disagreed with release 0.12.0. This planning repair fixes that mismatch; it does not retrospectively turn skipped gameplay acceptance green.</x:v>
+        <x:v>Surestep has a dedicated source/browser acceptance workflow and public byte verification. Final per-run receipts distinguish tested source, merged publication and hardware review. The older failed Tidelight run remains historical evidence and is not retroactively credited.</x:v>
       </x:c>
       <x:c r="L73" s="6" t="str">
         <x:v>tests/verify-live.py
+tests/surestep-browser.py
 tests/launch.py
+SURESTEP.md
 CONTINUATION-AUDIT.md</x:v>
       </x:c>
       <x:c r="M73" s="6" t="str"/>
@@ -4548,7 +4561,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdadc18230c054e81"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf3469a0f7e5c4856"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4850,7 +4863,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R590db8259c084bda"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbc2a63471cca4f66"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5282,7 +5295,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf642ba3e03e74a33"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R024be00c2b374b71"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5628,7 +5641,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb544c8baba314f48"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R488444541fd6446e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6046,7 +6059,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R83db27770ff14a3a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9643fc5ebe3d4a56"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Complete Returning Bell release metadata, canonical workbook, VR handover and retained-mode acceptance
</commit_message>
<xml_diff>
--- a/vesperfall/AAA-PRODUCTION.xlsx
+++ b/vesperfall/AAA-PRODUCTION.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="Rdd6885be96804f48"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="2" r:id="R082cd50e961f428b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Milestones" sheetId="3" r:id="Ra681cf1889c64316"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Device QA" sheetId="4" r:id="Rf69a3bbb99bb462a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="5" r:id="R6784a3c53166430d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risk Register" sheetId="6" r:id="R5f77ef7909194d03"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="R04e223e2c83d4cd3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="2" r:id="R8d6abd6dac5b4f68"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Milestones" sheetId="3" r:id="R918b188a90434ac3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Device QA" sheetId="4" r:id="Rc70b0a0267dc40a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="5" r:id="R86a2a346690a4a9f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risk Register" sheetId="6" r:id="R12f205022bb74aab"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -628,7 +628,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="12" t="str">
-        <x:v>v0.13.0 / Surestep / 2026-09-14. Fast Xbox arrow selection, Quest water settings and tracked-hand menus, and procedural humanoid foot planting. Existing save formats and simulation remain unchanged.</x:v>
+        <x:v>v0.14.0 / The Returning Bell / 2026-09-15. Authored opening, interlocking approaches, reversible screens, a lasting return gate and discovery-limited AR inspection. Legacy saved geography and direct controls are preserved.</x:v>
       </x:c>
       <x:c r="B3" s="12"/>
       <x:c r="C3" s="12"/>
@@ -774,7 +774,7 @@
     </x:row>
     <x:row r="15" ht="24" customHeight="1">
       <x:c r="A15" s="6" t="str">
-        <x:v>Surestep closes the bounded missing Quest water-settings item. Humanoid IK is a procedural foundation, not finished production art. The older basin/reflection/audio draft remains unshipped; water lifecycle findings remain open.</x:v>
+        <x:v>Returning Bell is the default fresh expedition, not a replacement engine. It has a complete ring-and-return objective; its blessing leads explicitly into retained Endless content. The next authored chapter and external playtest evidence remain open.</x:v>
       </x:c>
       <x:c r="B15" s="6"/>
       <x:c r="C15" s="6"/>
@@ -838,7 +838,7 @@
     </x:row>
     <x:row r="21" ht="24" customHeight="1">
       <x:c r="A21" s="6" t="str">
-        <x:v>Next: water lifecycle/budget hardening, the requested sound/music pass, physical controller/hand-tracking review and purposeful exploration. Broad accessibility and production-art tasks remain Partial or open.</x:v>
+        <x:v>Next: unfamiliar-player and replay observation, physical VR/AR and Xbox checks, then targeted level readability, sound and frame-budget refinements. Do not expand room count ahead of proving place mastery.</x:v>
       </x:c>
       <x:c r="B21" s="6"/>
       <x:c r="C21" s="6"/>
@@ -870,7 +870,7 @@
     </x:row>
     <x:row r="24" ht="24" customHeight="1">
       <x:c r="A24" s="6" t="str">
-        <x:v>Surestep adds 17 deterministic tests (170 total at initial local review) plus a rendered Xbox/controller/hand-joint journey. Use the exact workflow artifacts for acceptance and publication status. No physical-device or human approval is implied.</x:v>
+        <x:v>Use the exact Returning Bell workflow source and reports for acceptance. Model routes, rendered input, publication, physical hardware and human enjoyment are separate evidence gates. No physical or human approval is implied.</x:v>
       </x:c>
       <x:c r="B24" s="6"/>
       <x:c r="C24" s="6"/>
@@ -902,7 +902,7 @@
     </x:row>
     <x:row r="27" ht="24" customHeight="1">
       <x:c r="A27" s="34" t="str">
-        <x:v>Canonical JSON SHA-256: 382ce526249c7e8b10748abb72a92780f9d3c331bc77773da4c974e462640608</x:v>
+        <x:v>Canonical JSON SHA-256: 1e4e9688091823beeb5b185f5c95bacb544b05d9a673c963ec355b1a2fd4223d</x:v>
       </x:c>
       <x:c r="B27" s="34"/>
       <x:c r="C27" s="34"/>
@@ -2988,17 +2988,19 @@
         <x:v>Every gameplay and game-owned UI path, including water settings, confirmations, recovery, seed entry, audio and accessibility settings, is reachable and dismissible with Xbox and Quest controls without a mouse. Test both handedness modes, neutral-input transitions and return focus. Browser/system permission prompts remain platform-owned.</x:v>
       </x:c>
       <x:c r="K46" s="6" t="str">
-        <x:v>Surestep implements the missing paginated Quest water settings and adds optional tracked-hand ray/pinch menu input. Xbox down selects Blink and left cycles stocked, unlocked damage arrows outside menus/quiver. Tracking loss, held-pinch acquisition and controller handover are explicit software gates in tests/surestep-browser.py. Full accessibility/remapping and physical-device approval remain open.</x:v>
+        <x:v>Surestep implements the missing paginated Quest water settings and adds optional tracked-hand ray/pinch menu input. Xbox down selects Blink and left cycles stocked, unlocked damage arrows outside menus/quiver. Tracking loss, held-pinch acquisition and controller handover are explicit software gates in tests/surestep-browser.py. Full accessibility/remapping and physical-device approval remain open. Returning Bell interactions retain direct Xbox controls; the AR Architect's Table shares controller-ray/stick and joint-pinch menus. Game-owned confirmations still use the existing save guard.</x:v>
       </x:c>
       <x:c r="L46" s="6" t="str">
         <x:v>dominion-controls.js
 quest-hands.js
 tests/surestep-browser.py
 tests/dominions-browser.py
-SURESTEP.md</x:v>
+SURESTEP.md
+returning-bell.js
+tests/returning-bell-browser.py</x:v>
       </x:c>
       <x:c r="M46" s="6" t="str">
-        <x:v>0.7.0</x:v>
+        <x:v>0.13.0</x:v>
       </x:c>
       <x:c r="N46" s="6" t="str">
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/dominion-controls.js</x:v>
@@ -3361,11 +3363,12 @@
         <x:v>A new player can learn nock/draw, cancel, reload, shield, Blink, shard step, pickups and quiver in either handedness, then enter a short scored encounter. Record completion, confusion and fatigue.</x:v>
       </x:c>
       <x:c r="K54" s="6" t="str">
-        <x:v>Ten playable lessons now verify actual outcomes, with device-specific hints and a spatial Quest coach. Skips are recorded separately. Software-only: first-user confusion, reversed-hand ergonomics and fatigue remain to be measured.</x:v>
+        <x:v>Ten playable lessons now verify actual outcomes, with device-specific hints and a spatial Quest coach. Skips are recorded separately. Software-only: first-user confusion, reversed-hand ergonomics and fatigue remain to be measured. Returning Bell replaces the default fresh opening; all guided First Bell lessons remain explicitly available. Physical onboarding and newcomer study remain open.</x:v>
       </x:c>
       <x:c r="L54" s="6" t="str">
         <x:v>first-bell.js
-tests/first-bell-browser.py</x:v>
+tests/first-bell-browser.py
+returning-bell.js</x:v>
       </x:c>
       <x:c r="M54" s="6" t="str">
         <x:v>0.10.0 First Bell</x:v>
@@ -3406,7 +3409,7 @@
         <x:v>Coordinate telegraphed melee/ranged attacks, limit unavoidable overlap and offscreen attacks, preserve escape routes and add recovery beats. Replay fixed-seed stress encounters.</x:v>
       </x:c>
       <x:c r="K55" s="6" t="str">
-        <x:v>The optional Oath coordinates three staged encounters with front-hemisphere initiation, bolt/windup budgets and recovery supplies. The original Endless mode is unchanged. Broad seed/human difficulty evaluation remains open.</x:v>
+        <x:v>The optional Oath coordinates three staged encounters with front-hemisphere initiation, bolt/windup budgets and recovery supplies. The original Endless mode is unchanged. Broad seed/human difficulty evaluation remains open. Returning Bell deliberately places five retained defenders along different approaches; it does not claim a new global director or patrol system.</x:v>
       </x:c>
       <x:c r="L55" s="6" t="str">
         <x:v>oath-model.js
@@ -3499,16 +3502,22 @@
         <x:v>One polished 20-30 minute target route mixes safe introduction, alternate approach, escalating encounter, discovery and boss payoff. Validate every traversal connector and recovery path. Duration is a design target, not measured content. Preserve multi-level gothic sightlines and multiple approaches. Plan selective water-adjacent discoveries with purpose; the present water layer does not create new navigable rooms.</x:v>
       </x:c>
       <x:c r="K57" s="6" t="str">
-        <x:v>A connected Roseglass/Ivory Crown/Ember Crown progression reuses the collision-tested 25-room world, existing stairs and alternate approaches. Three staged courts are implemented; the proposed 20-30 minute polished duration and authored connector variety are not yet measured or complete.</x:v>
+        <x:v>The Returning Bell is a separate authored opening with seven connected places, two actual stair approaches, real Blink connectors, reversible collision-backed screens, a persistent return gate, and a ring-and-return objective. Development slice, not a measured 20-30 minute finished campaign. Software route/save/native-input checks are separate from unfamiliar-player and physical-device review.</x:v>
       </x:c>
       <x:c r="L57" s="6" t="str">
         <x:v>oath-model.js
 first-bell.js
 tests/oath.test.cjs
-CONTINUATION-AUDIT.md</x:v>
+CONTINUATION-AUDIT.md
+returning-bell-model.js
+returning-bell-art.js
+returning-bell.js
+tests/returning-bell.test.cjs
+tests/returning-bell-browser.py
+RETURNING-BELL.md</x:v>
       </x:c>
       <x:c r="M57" s="6" t="str">
-        <x:v>0.10.0 First Bell</x:v>
+        <x:v>0.14.0 Returning Bell</x:v>
       </x:c>
       <x:c r="N57" s="6" t="str">
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/oath-model.js</x:v>
@@ -3595,7 +3604,9 @@
 tests/surestep.test.cjs
 SURESTEP.md</x:v>
       </x:c>
-      <x:c r="M59" s="6" t="str"/>
+      <x:c r="M59" s="6" t="str">
+        <x:v>0.13.0</x:v>
+      </x:c>
       <x:c r="N59" s="6" t="str">
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/CONTINUATION-AUDIT.md</x:v>
       </x:c>
@@ -3688,10 +3699,10 @@
         <x:v>Original environmental narrative and reward presentation</x:v>
       </x:c>
       <x:c r="C62" s="6" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Partial</x:v>
       </x:c>
       <x:c r="D62" s="6" t="str">
-        <x:v>P1</x:v>
+        <x:v>P0</x:v>
       </x:c>
       <x:c r="E62" s="6" t="str">
         <x:v>M3</x:v>
@@ -3712,10 +3723,16 @@
         <x:v>Public-only lore, landmarks and discoveries connect the world; skippable/accessible presentation; no private story content enters this repository without permission.</x:v>
       </x:c>
       <x:c r="K62" s="6" t="str">
-        <x:v>Not closed; no completion credit without gate evidence.</x:v>
-      </x:c>
-      <x:c r="L62" s="6" t="str"/>
-      <x:c r="M62" s="6" t="str"/>
+        <x:v>The authored refuge, basin/statue landmarks, silent tower signal, screen winch and service-side return connection express one original environmental objective. Newcomer recognition, discovery, audio and finished-art review remain open.</x:v>
+      </x:c>
+      <x:c r="L62" s="6" t="str">
+        <x:v>returning-bell-model.js
+returning-bell-art.js
+RETURNING-BELL.md</x:v>
+      </x:c>
+      <x:c r="M62" s="6" t="str">
+        <x:v>0.14.0 Returning Bell</x:v>
+      </x:c>
       <x:c r="N62" s="6" t="str">
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
       </x:c>
@@ -3999,7 +4016,7 @@
         <x:v>Test whether the experience is enjoyable and understandable.</x:v>
       </x:c>
       <x:c r="J69" s="6" t="str">
-        <x:v>Record at least 8 external playtest sessions as a proposed first research batch, including new/experienced players. Track task success, deaths, confusion, route discovery, fatigue and whether they choose another run. No automated score substitutes.</x:v>
+        <x:v>Record at least 8 external playtest sessions as a proposed first research batch, including new/experienced players. Track task success, deaths, confusion, route discovery, fatigue and whether they choose another run. No automated score substitutes. For Returning Bell, record whether players form a plan, recognize the screen tradeoff and return gate, and exploit learning on replay without coaching.</x:v>
       </x:c>
       <x:c r="K69" s="6" t="str">
         <x:v>Not closed; no completion credit without gate evidence.</x:v>
@@ -4494,7 +4511,7 @@
         <x:v>Publish one complete integrated slice, including onboarding, traversal, encounter pacing, boss payoff and saved continuation; collect human feedback before producing additional bosses.</x:v>
       </x:c>
       <x:c r="K81" s="6" t="str">
-        <x:v>First Bell integrates teaching, a scored staged route, three-phase boss and checkpoint continuation in the maintained game. Source/model and native-input checks are distinct from physical hardware and human approval.</x:v>
+        <x:v>First Bell integrates teaching, a scored staged route, three-phase boss and checkpoint continuation in the maintained game. Source/model and native-input checks are distinct from physical hardware and human approval. The authored opening is a ring-and-return chapter, not an additional boss fight. Its completion offers an explicit blessing continuation into retained Endless content; the next authored chapter remains open.</x:v>
       </x:c>
       <x:c r="L81" s="6" t="str">
         <x:v>FIRST-BELL.md
@@ -4561,7 +4578,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf3469a0f7e5c4856"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5d822f81608f4c37"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4720,7 +4737,7 @@
         <x:v>M1</x:v>
       </x:c>
       <x:c r="E8" s="6" t="str">
-        <x:v>Turn mechanics into a deliberately paced signature adventure.</x:v>
+        <x:v>Make the authored Returning Bell opening legible and replayable, then extend its route grammar from observed evidence.</x:v>
       </x:c>
       <x:c r="F8" s="6" t="str">
         <x:v>Coordinated encounters, authored route grammar, first boss and viable run choices survive native and human playtests.</x:v>
@@ -4863,7 +4880,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbc2a63471cca4f66"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0b8da52c479245f3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5054,10 +5071,10 @@
         <x:v>Quest 3 / AR</x:v>
       </x:c>
       <x:c r="C9" s="6" t="str">
-        <x:v>Stationary Sanctuary</x:v>
+        <x:v>Sanctuary and Architect's Table</x:v>
       </x:c>
       <x:c r="D9" s="6" t="str">
-        <x:v>Clear space, permission denial, safe stationary controls and expedition restoration</x:v>
+        <x:v>Passthrough, virtual-table placement/recenter/layers, tracked controllers and pinch UI, and exact paused-expedition restoration</x:v>
       </x:c>
       <x:c r="E9" s="6" t="str">
         <x:v>V42,V62</x:v>
@@ -5066,7 +5083,7 @@
         <x:v>Not run</x:v>
       </x:c>
       <x:c r="G9" s="6" t="str">
-        <x:v>Record real passthrough visibility; no real-world occlusion claim.</x:v>
+        <x:v>Record physical visibility, reach and legibility. Table has no detected physical anchor or real-world occlusion.</x:v>
       </x:c>
       <x:c r="H9" s="6"/>
       <x:c r="I9" s="20"/>
@@ -5295,7 +5312,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R024be00c2b374b71"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3b70417f8b0e4893"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5641,7 +5658,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R488444541fd6446e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R37138cd3a7ee477c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5770,13 +5787,13 @@
         <x:v>Production / level design</x:v>
       </x:c>
       <x:c r="E7" s="6" t="str">
-        <x:v>Many procedural rooms do not establish quality</x:v>
+        <x:v>Authored opening exists, but newcomer understanding and replay enjoyment are unmeasured</x:v>
       </x:c>
       <x:c r="F7" s="6" t="str">
         <x:v>V49,V50,V51,V52,V76</x:v>
       </x:c>
       <x:c r="G7" s="6" t="str">
-        <x:v>Finish one cohesive onboarding-to-boss route before expanding content.</x:v>
+        <x:v>Observe recognition, route choice and replay before producing another chapter.</x:v>
       </x:c>
       <x:c r="H7" s="6" t="str">
         <x:v>Open</x:v>
@@ -5822,13 +5839,13 @@
         <x:v>Engineering / QA</x:v>
       </x:c>
       <x:c r="E9" s="6" t="str">
-        <x:v>Local saves are not cloud backup; only current generator supported</x:v>
+        <x:v>Local storage is not cloud backup; two immutable layout identities now require ongoing fixtures</x:v>
       </x:c>
       <x:c r="F9" s="6" t="str">
         <x:v>V65,V75</x:v>
       </x:c>
       <x:c r="G9" s="6" t="str">
-        <x:v>Publish limitations; add migration/backup fixtures before incompatible changes.</x:v>
+        <x:v>Retain the original Surestep checkpoint fixture; reconstruct chapter mechanisms before validating restored positions.</x:v>
       </x:c>
       <x:c r="H9" s="6" t="str">
         <x:v>Open</x:v>
@@ -6059,7 +6076,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9643fc5ebe3d4a56"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7941389e42334f3d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Synchronize Open Line 0.15.0 metadata, artifact-authored workbook, library record and layout-aware acceptance
</commit_message>
<xml_diff>
--- a/vesperfall/AAA-PRODUCTION.xlsx
+++ b/vesperfall/AAA-PRODUCTION.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="R04e223e2c83d4cd3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="2" r:id="R8d6abd6dac5b4f68"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Milestones" sheetId="3" r:id="R918b188a90434ac3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Device QA" sheetId="4" r:id="Rc70b0a0267dc40a7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="5" r:id="R86a2a346690a4a9f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risk Register" sheetId="6" r:id="R12f205022bb74aab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="R66aca5130e7a4437"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="2" r:id="R65e48c1f26e44c35"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Milestones" sheetId="3" r:id="R719808806d024500"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Device QA" sheetId="4" r:id="R009f8eb704ce4cae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="5" r:id="R0bfa9186fb2845e2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risk Register" sheetId="6" r:id="R77d0a770f3b6437e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -628,7 +628,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="12" t="str">
-        <x:v>v0.14.0 / The Returning Bell / 2026-09-15. Authored opening, interlocking approaches, reversible screens, a lasting return gate and discovery-limited AR inspection. Legacy saved geography and direct controls are preserved.</x:v>
+        <x:v>v0.15.0 / Open Line / 2026-09-15. A shorter exposed stair and a shared shot lane make screen state matter. Shoot the brass release or use gallery control. Old layouts, saves and direct controls remain.</x:v>
       </x:c>
       <x:c r="B3" s="12"/>
       <x:c r="C3" s="12"/>
@@ -774,7 +774,7 @@
     </x:row>
     <x:row r="15" ht="24" customHeight="1">
       <x:c r="A15" s="6" t="str">
-        <x:v>Returning Bell is the default fresh expedition, not a replacement engine. It has a complete ring-and-return objective; its blessing leads explicitly into retained Endless content. The next authored chapter and external playtest evidence remain open.</x:v>
+        <x:v>The same seven-place chapter supports flanking approaches, the new central stair and a learned signal shot. Knowledge changes how the place can be used. Completion still leads into retained Endless. Human first/replay understanding, final art and physical-device acceptance remain open.</x:v>
       </x:c>
       <x:c r="B15" s="6"/>
       <x:c r="C15" s="6"/>
@@ -902,7 +902,7 @@
     </x:row>
     <x:row r="27" ht="24" customHeight="1">
       <x:c r="A27" s="34" t="str">
-        <x:v>Canonical JSON SHA-256: 1e4e9688091823beeb5b185f5c95bacb544b05d9a673c963ec355b1a2fd4223d</x:v>
+        <x:v>Canonical roadmap.json SHA-256: c6a74f2441453dc178b2d2c9d5f66cfc840b41866b50c5f62d2bed1475cad6d3</x:v>
       </x:c>
       <x:c r="B27" s="34"/>
       <x:c r="C27" s="34"/>
@@ -3502,7 +3502,7 @@
         <x:v>One polished 20-30 minute target route mixes safe introduction, alternate approach, escalating encounter, discovery and boss payoff. Validate every traversal connector and recovery path. Duration is a design target, not measured content. Preserve multi-level gothic sightlines and multiple approaches. Plan selective water-adjacent discoveries with purpose; the present water layer does not create new navigable rooms.</x:v>
       </x:c>
       <x:c r="K57" s="6" t="str">
-        <x:v>The Returning Bell is a separate authored opening with seven connected places, two actual stair approaches, real Blink connectors, reversible collision-backed screens, a persistent return gate, and a ring-and-return objective. Development slice, not a measured 20-30 minute finished campaign. Software route/save/native-input checks are separate from unfamiliar-player and physical-device review.</x:v>
+        <x:v>Open Line refines the existing seven-place chapter instead of expanding it. A new versioned central stair shares the screen's cover/shot tradeoff with a repositioned existing watcher. Ordinary arrows can lift the brass release; the gallery still reverses it. A learned signal shot can complete without entering the tower. Model and controller-driven route comparisons record actual distance, simulation time, health and shots; human comprehension, enjoyment and the original finished-slice gate remain open.</x:v>
       </x:c>
       <x:c r="L57" s="6" t="str">
         <x:v>oath-model.js
@@ -3514,10 +3514,14 @@
 returning-bell.js
 tests/returning-bell.test.cjs
 tests/returning-bell-browser.py
-RETURNING-BELL.md</x:v>
+RETURNING-BELL.md
+OPEN-LINE.md
+returning-bell-lanes.js
+tests/open-line.test.cjs
+tests/open-line-browser.py</x:v>
       </x:c>
       <x:c r="M57" s="6" t="str">
-        <x:v>0.14.0 Returning Bell</x:v>
+        <x:v>0.15.0 Open Line</x:v>
       </x:c>
       <x:c r="N57" s="6" t="str">
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/oath-model.js</x:v>
@@ -3723,15 +3727,19 @@
         <x:v>Public-only lore, landmarks and discoveries connect the world; skippable/accessible presentation; no private story content enters this repository without permission.</x:v>
       </x:c>
       <x:c r="K62" s="6" t="str">
-        <x:v>The authored refuge, basin/statue landmarks, silent tower signal, screen winch and service-side return connection express one original environmental objective. Newcomer recognition, discovery, audio and finished-art review remain open.</x:v>
+        <x:v>Open Line links a visible brass release and cable to the actual moving screens, labels the exposed short stair, and preserves the recognizable refuge gate. Functional cues express speed/exposure versus observation/control. Recognition and environmental-story understanding require unfamiliar-player observation; no human narrative rating is claimed.</x:v>
       </x:c>
       <x:c r="L62" s="6" t="str">
         <x:v>returning-bell-model.js
 returning-bell-art.js
-RETURNING-BELL.md</x:v>
+RETURNING-BELL.md
+OPEN-LINE.md
+returning-bell-lanes.js
+tests/open-line.test.cjs
+tests/open-line-browser.py</x:v>
       </x:c>
       <x:c r="M62" s="6" t="str">
-        <x:v>0.14.0 Returning Bell</x:v>
+        <x:v>0.15.0 Open Line</x:v>
       </x:c>
       <x:c r="N62" s="6" t="str">
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
@@ -4059,10 +4067,17 @@
         <x:v>Keep fixtures for old supported generator/schema versions, offer explicit local backup/restore and verify interrupted writes, browser quota and update migration. Never silently reset incompatible saves. Any future discrete-hit-point conversion must specify health/healing balance and tested checkpoint migration; retain current health and profiles in presentation-only releases.</x:v>
       </x:c>
       <x:c r="K70" s="6" t="str">
-        <x:v>Not closed; no completion credit without gate evidence.</x:v>
-      </x:c>
-      <x:c r="L70" s="6" t="str"/>
-      <x:c r="M70" s="6" t="str"/>
+        <x:v>Legacy hollow-dominions-1 and returning-bell-1 fixtures remain. Open Line adds returning-bell-2 and captures/restores the actual layout identity; mechanism geometry is rebuilt before supported-position checks, including a player saved inside the raised-screen crossing. This compatibility work does not complete export, backup, storage eviction or general migration tooling.</x:v>
+      </x:c>
+      <x:c r="L70" s="6" t="str">
+        <x:v>OPEN-LINE.md
+returning-bell-lanes.js
+tests/open-line.test.cjs
+tests/open-line-browser.py</x:v>
+      </x:c>
+      <x:c r="M70" s="6" t="str">
+        <x:v>0.15.0 Open Line</x:v>
+      </x:c>
       <x:c r="N70" s="6" t="str">
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
       </x:c>
@@ -4181,16 +4196,22 @@
         <x:v>For every finished upgrade, test the actual scoped source, commit and merge without overwriting sibling games, verify GitHub Pages deployment plus public runtime/asset/plan/workbook bytes, then launch the public game. Separate source, test, deployment, hardware and human evidence. Retry transient GitHub faults with backoff; inspect failed jobs instead of polling an unchanged failure list. Preserve explicit rollback and save-compatibility notes.</x:v>
       </x:c>
       <x:c r="K73" s="6" t="str">
-        <x:v>Surestep has a dedicated source/browser acceptance workflow and public byte verification. Final per-run receipts distinguish tested source, merged publication and hardware review. The older failed Tidelight run remains historical evidence and is not retroactively credited.</x:v>
+        <x:v>Open Line retains exact-source model/workbook checks, four controller-driven route comparisons, full first-person VR/AR/hand/save regression and separate public-byte/launch verification. Preserve unsuccessful receipts and separate model, rendered software, physical-device and human evidence. Public success is recorded only in the matching publication receipt.</x:v>
       </x:c>
       <x:c r="L73" s="6" t="str">
         <x:v>tests/verify-live.py
 tests/surestep-browser.py
 tests/launch.py
 SURESTEP.md
-CONTINUATION-AUDIT.md</x:v>
-      </x:c>
-      <x:c r="M73" s="6" t="str"/>
+CONTINUATION-AUDIT.md
+OPEN-LINE.md
+returning-bell-lanes.js
+tests/open-line.test.cjs
+tests/open-line-browser.py</x:v>
+      </x:c>
+      <x:c r="M73" s="6" t="str">
+        <x:v>0.15.0 Open Line</x:v>
+      </x:c>
       <x:c r="N73" s="6" t="str">
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/tests/verify-live.py</x:v>
       </x:c>
@@ -4511,15 +4532,19 @@
         <x:v>Publish one complete integrated slice, including onboarding, traversal, encounter pacing, boss payoff and saved continuation; collect human feedback before producing additional bosses.</x:v>
       </x:c>
       <x:c r="K81" s="6" t="str">
-        <x:v>First Bell integrates teaching, a scored staged route, three-phase boss and checkpoint continuation in the maintained game. Source/model and native-input checks are distinct from physical hardware and human approval. The authored opening is a ring-and-return chapter, not an additional boss fight. Its completion offers an explicit blessing continuation into retained Endless content; the next authored chapter remains open.</x:v>
+        <x:v>The authored opening retains the ordinary sector reward once and explicitly continues into Endless after its blessing. Open Line strengthens route purpose and a knowledge-based signal approach without adding a new boss or second authored chapter. Existing First Bell/Oath remain. External first/replay play and physical-device acceptance remain open.</x:v>
       </x:c>
       <x:c r="L81" s="6" t="str">
         <x:v>FIRST-BELL.md
 tests/first-bell-browser.py
-tests/pilgrim.test.cjs</x:v>
+tests/pilgrim.test.cjs
+OPEN-LINE.md
+returning-bell-lanes.js
+tests/open-line.test.cjs
+tests/open-line-browser.py</x:v>
       </x:c>
       <x:c r="M81" s="6" t="str">
-        <x:v>0.10.0 First Bell</x:v>
+        <x:v>0.15.0 Open Line</x:v>
       </x:c>
       <x:c r="N81" s="6" t="str">
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/FIRST-BELL.md</x:v>
@@ -4578,7 +4603,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5d822f81608f4c37"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R373c21fad46c4e38"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4880,7 +4905,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0b8da52c479245f3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R76b144a13271420c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5312,7 +5337,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3b70417f8b0e4893"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra624d9879f0446de"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5658,7 +5683,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R37138cd3a7ee477c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd8221a135a074da9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5839,13 +5864,13 @@
         <x:v>Engineering / QA</x:v>
       </x:c>
       <x:c r="E9" s="6" t="str">
-        <x:v>Local storage is not cloud backup; two immutable layout identities now require ongoing fixtures</x:v>
+        <x:v>Local storage is not cloud backup; three immutable layout identities now require ongoing fixtures</x:v>
       </x:c>
       <x:c r="F9" s="6" t="str">
         <x:v>V65,V75</x:v>
       </x:c>
       <x:c r="G9" s="6" t="str">
-        <x:v>Retain the original Surestep checkpoint fixture; reconstruct chapter mechanisms before validating restored positions.</x:v>
+        <x:v>Retain the original Surestep and Returning Bell v1 fixtures; rebuild each saved layout and screen/gate state before validating positions. Do not remove v2 restore support during an art rollback.</x:v>
       </x:c>
       <x:c r="H9" s="6" t="str">
         <x:v>Open</x:v>
@@ -6076,7 +6101,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7941389e42334f3d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf2a3309bdb014552"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Synchronize Goldwind 0.16.0 roadmap and workbook; measure render-bound throw input without changing gameplay
</commit_message>
<xml_diff>
--- a/vesperfall/AAA-PRODUCTION.xlsx
+++ b/vesperfall/AAA-PRODUCTION.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="R66aca5130e7a4437"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="2" r:id="R65e48c1f26e44c35"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Milestones" sheetId="3" r:id="R719808806d024500"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Device QA" sheetId="4" r:id="R009f8eb704ce4cae"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="5" r:id="R0bfa9186fb2845e2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risk Register" sheetId="6" r:id="R77d0a770f3b6437e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="R25c4428087cd417a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="2" r:id="R00092acda6d0464c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Milestones" sheetId="3" r:id="R82e512fbaf704c45"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Device QA" sheetId="4" r:id="R56a1554f64cf41ec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="5" r:id="Rff4599357f8c4c0e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risk Register" sheetId="6" r:id="R3f4c801032044f33"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -628,7 +628,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="12" t="str">
-        <x:v>v0.15.0 / Open Line / 2026-09-15. A shorter exposed stair and a shared shot lane make screen state matter. Shoot the brass release or use gallery control. Old layouts, saves and direct controls remain.</x:v>
+        <x:v>v0.16.0 / Goldwind / 2026-09-17. Opt-in physical bow: golden teleport draw, thrown escape disk, directional shield and reach quiver. Open Line geography, Classic/crossbow, Xbox and all saved layouts remain.</x:v>
       </x:c>
       <x:c r="B3" s="12"/>
       <x:c r="C3" s="12"/>
@@ -774,7 +774,7 @@
     </x:row>
     <x:row r="15" ht="24" customHeight="1">
       <x:c r="A15" s="6" t="str">
-        <x:v>The same seven-place chapter supports flanking approaches, the new central stair and a learned signal shot. Knowledge changes how the place can be used. Completion still leads into retained Endless. Human first/replay understanding, final art and physical-device acceptance remain open.</x:v>
+        <x:v>Prove the physical actions inside the existing cathedral before extending modular generation. Real arrow flight, supported landings and deliberate throws matter more than adding rooms. No new enemy roster or second chapter is included.</x:v>
       </x:c>
       <x:c r="B15" s="6"/>
       <x:c r="C15" s="6"/>
@@ -838,7 +838,7 @@
     </x:row>
     <x:row r="21" ht="24" customHeight="1">
       <x:c r="A21" s="6" t="str">
-        <x:v>Next: unfamiliar-player and replay observation, physical VR/AR and Xbox checks, then targeted level readability, sound and frame-budget refinements. Do not expand room count ahead of proving place mastery.</x:v>
+        <x:v>Next: physical Quest/Xbox and unfamiliar/repeat-player observation of Goldwind in Open Line; then reusable authored encounter relationships, separate travel/shot validation and deterministic streams.</x:v>
       </x:c>
       <x:c r="B21" s="6"/>
       <x:c r="C21" s="6"/>
@@ -870,7 +870,7 @@
     </x:row>
     <x:row r="24" ht="24" customHeight="1">
       <x:c r="A24" s="6" t="str">
-        <x:v>Use the exact Returning Bell workflow source and reports for acceptance. Model routes, rendered input, publication, physical hardware and human enjoyment are separate evidence gates. No physical or human approval is implied.</x:v>
+        <x:v>Use GOLDWIND.md and its exact publication receipt. Model fixtures, rendered synthetic input, public bytes, physical hardware and human enjoyment are separate evidence. No device or human gate is certified.</x:v>
       </x:c>
       <x:c r="B24" s="6"/>
       <x:c r="C24" s="6"/>
@@ -902,7 +902,7 @@
     </x:row>
     <x:row r="27" ht="24" customHeight="1">
       <x:c r="A27" s="34" t="str">
-        <x:v>Canonical roadmap.json SHA-256: c6a74f2441453dc178b2d2c9d5f66cfc840b41866b50c5f62d2bed1475cad6d3</x:v>
+        <x:v>Canonical roadmap.json SHA-256: 0189dec4b3dbf791dd5ac6eb7c8f913c64280c5766dfb472cb8fe5166791dfb7</x:v>
       </x:c>
       <x:c r="B27" s="34"/>
       <x:c r="C27" s="34"/>
@@ -1264,7 +1264,7 @@
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/index.html</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="124" customHeight="1">
+    <x:row r="7" ht="195" customHeight="1">
       <x:c r="A7" s="6" t="str">
         <x:v>V02</x:v>
       </x:c>
@@ -1296,15 +1296,20 @@
         <x:v>Real controller poses produce direction and power; losses never fire a stale arrow.</x:v>
       </x:c>
       <x:c r="K7" s="6" t="str">
-        <x:v>Source implemented; software regression coverage. Physical acceptance is separate.</x:v>
+        <x:v>Source implemented; software regression coverage. Physical acceptance is separate. Goldwind adds an opt-in physical bow preset; exact model, native input and publication outcomes belong in its versioned evidence receipt. Classic/crossbow and Xbox remain. Real-device ergonomics and human acceptance are not closed.</x:v>
       </x:c>
       <x:c r="L7" s="6" t="str">
         <x:v>input.js
 tests/core.test.cjs
-tests/browser.py</x:v>
+tests/browser.py
+GOLDWIND.md
+goldwind-model.js
+goldwind-xr.js
+tests/goldwind.test.cjs
+tests/goldwind-browser.py</x:v>
       </x:c>
       <x:c r="M7" s="6" t="str">
-        <x:v>Baseline through 0.6.0</x:v>
+        <x:v>0.16.0 Goldwind</x:v>
       </x:c>
       <x:c r="N7" s="6" t="str">
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/input.js</x:v>
@@ -1355,7 +1360,7 @@
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/core.js</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="124" customHeight="1">
+    <x:row r="9" ht="195" customHeight="1">
       <x:c r="A9" s="6" t="str">
         <x:v>V04</x:v>
       </x:c>
@@ -1384,17 +1389,23 @@
         <x:v>Preserve the established game while closing the stated acceptance gate.</x:v>
       </x:c>
       <x:c r="J9" s="6" t="str">
-        <x:v>Shared projectile/preview first-hit collision; a widened upper-gallery target. A clear preview is not automatic aiming or permission to pass through solids.</x:v>
+        <x:v>Shared projectile/preview first-hit collision; a widened upper-gallery target. A clear preview is not automatic aiming or permission to pass through solids. Goldwind travel is a temporary physically nocked golden arrow, not an equipment toggle. Its default hides arc/ring; an optional drawing-only path cannot authorize invalid landings.</x:v>
       </x:c>
       <x:c r="K9" s="6" t="str">
-        <x:v>Source implemented; software regression coverage. Physical acceptance is separate.</x:v>
-      </x:c>
-      <x:c r="L9" s="6" t="str"/>
+        <x:v>Source implemented; software regression coverage. Physical acceptance is separate. Goldwind adds an opt-in physical bow preset; exact model, native input and publication outcomes belong in its versioned evidence receipt. Classic/crossbow and Xbox remain. Real-device ergonomics and human acceptance are not closed.</x:v>
+      </x:c>
+      <x:c r="L9" s="6" t="str">
+        <x:v>GOLDWIND.md
+goldwind-model.js
+goldwind-xr.js
+tests/goldwind.test.cjs
+tests/goldwind-browser.py</x:v>
+      </x:c>
       <x:c r="M9" s="6" t="str">
-        <x:v>Baseline through 0.6.0</x:v>
+        <x:v>0.16.0 Goldwind</x:v>
       </x:c>
       <x:c r="N9" s="6" t="str">
-        <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
+        <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/GOLDWIND.md</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="124" customHeight="1">
@@ -1959,7 +1970,7 @@
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
       </x:c>
     </x:row>
-    <x:row r="23" ht="124" customHeight="1">
+    <x:row r="23" ht="195" customHeight="1">
       <x:c r="A23" s="6" t="str">
         <x:v>V18</x:v>
       </x:c>
@@ -1991,17 +2002,23 @@
         <x:v>Front-face swept blocking before body impact; side/rear exposure, guard cost, tracking cancellation and no simultaneous firing.</x:v>
       </x:c>
       <x:c r="K23" s="6" t="str">
-        <x:v>Source implemented; software regression coverage. Physical acceptance is separate.</x:v>
-      </x:c>
-      <x:c r="L23" s="6" t="str"/>
+        <x:v>Source implemented; software regression coverage. Physical acceptance is separate. Goldwind adds an opt-in physical bow preset; exact model, native input and publication outcomes belong in its versioned evidence receipt. Classic/crossbow and Xbox remain. Real-device ergonomics and human acceptance are not closed.</x:v>
+      </x:c>
+      <x:c r="L23" s="6" t="str">
+        <x:v>GOLDWIND.md
+goldwind-model.js
+goldwind-xr.js
+tests/goldwind.test.cjs
+tests/goldwind-browser.py</x:v>
+      </x:c>
       <x:c r="M23" s="6" t="str">
-        <x:v>Baseline through 0.6.0</x:v>
+        <x:v>0.16.0 Goldwind</x:v>
       </x:c>
       <x:c r="N23" s="6" t="str">
-        <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="24" ht="124" customHeight="1">
+        <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/GOLDWIND.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="195" customHeight="1">
       <x:c r="A24" s="6" t="str">
         <x:v>V19</x:v>
       </x:c>
@@ -2030,17 +2047,23 @@
         <x:v>Preserve the established game while closing the stated acceptance gate.</x:v>
       </x:c>
       <x:c r="J24" s="6" t="str">
-        <x:v>Short unobstructed microdashes, no cliff crossing or tunneling. Physical thrown-shard gestures are not implemented.</x:v>
+        <x:v>Retain supported-ground button steps in Classic/Xbox. Goldwind's thrown disk must resolve real flight before one charged relocation, with continuous support, footprint clearance and no cliff crossing or wall tunneling.</x:v>
       </x:c>
       <x:c r="K24" s="6" t="str">
-        <x:v>Source implemented; software regression coverage. Physical acceptance is separate.</x:v>
-      </x:c>
-      <x:c r="L24" s="6" t="str"/>
+        <x:v>Source implemented; software regression coverage. Physical acceptance is separate. Goldwind adds an opt-in physical bow preset; exact model, native input and publication outcomes belong in its versioned evidence receipt. Classic/crossbow and Xbox remain. Real-device ergonomics and human acceptance are not closed.</x:v>
+      </x:c>
+      <x:c r="L24" s="6" t="str">
+        <x:v>GOLDWIND.md
+goldwind-model.js
+goldwind-xr.js
+tests/goldwind.test.cjs
+tests/goldwind-browser.py</x:v>
+      </x:c>
       <x:c r="M24" s="6" t="str">
-        <x:v>Baseline through 0.6.0</x:v>
+        <x:v>0.16.0 Goldwind</x:v>
       </x:c>
       <x:c r="N24" s="6" t="str">
-        <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
+        <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/GOLDWIND.md</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="124" customHeight="1">
@@ -2220,7 +2243,7 @@
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/tests/unchained-combat.py</x:v>
       </x:c>
     </x:row>
-    <x:row r="29" ht="124" customHeight="1">
+    <x:row r="29" ht="195" customHeight="1">
       <x:c r="A29" s="6" t="str">
         <x:v>V24</x:v>
       </x:c>
@@ -2228,7 +2251,7 @@
         <x:v>Physical thrown shard and richer vertical route families</x:v>
       </x:c>
       <x:c r="C29" s="6" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Partial</x:v>
       </x:c>
       <x:c r="D29" s="6" t="str">
         <x:v>P1</x:v>
@@ -2252,12 +2275,20 @@
         <x:v>Readable trajectories, safe valid landings, comfortable two-handed controls and alternative routes; no forced headset motion.</x:v>
       </x:c>
       <x:c r="K29" s="6" t="str">
-        <x:v>Not closed.</x:v>
-      </x:c>
-      <x:c r="L29" s="6" t="str"/>
-      <x:c r="M29" s="6" t="str"/>
+        <x:v>Physical disk acquisition, recent-motion release recognition, swept flight and supported-ground relocation are implemented for the Goldwind bow preset. A drop, pose jump, missing tracking or blocked impact cannot teleport. Richer generated route families and physical-device approval remain open.</x:v>
+      </x:c>
+      <x:c r="L29" s="6" t="str">
+        <x:v>GOLDWIND.md
+goldwind-model.js
+goldwind-xr.js
+tests/goldwind.test.cjs
+tests/goldwind-browser.py</x:v>
+      </x:c>
+      <x:c r="M29" s="6" t="str">
+        <x:v>0.16.0 Goldwind</x:v>
+      </x:c>
       <x:c r="N29" s="6" t="str">
-        <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
+        <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/GOLDWIND.md</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="124" customHeight="1">
@@ -2956,7 +2987,7 @@
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/bestiary.js</x:v>
       </x:c>
     </x:row>
-    <x:row r="46" ht="134" customHeight="1">
+    <x:row r="46" ht="195" customHeight="1">
       <x:c r="A46" s="6" t="str">
         <x:v>V41</x:v>
       </x:c>
@@ -2976,7 +3007,7 @@
         <x:v>Comfort</x:v>
       </x:c>
       <x:c r="G46" s="6" t="str">
-        <x:v>UX / accessibility</x:v>
+        <x:v>UX / accessibility / assignment pending</x:v>
       </x:c>
       <x:c r="H46" s="6" t="str">
         <x:v>V07</x:v>
@@ -2988,7 +3019,7 @@
         <x:v>Every gameplay and game-owned UI path, including water settings, confirmations, recovery, seed entry, audio and accessibility settings, is reachable and dismissible with Xbox and Quest controls without a mouse. Test both handedness modes, neutral-input transitions and return focus. Browser/system permission prompts remain platform-owned.</x:v>
       </x:c>
       <x:c r="K46" s="6" t="str">
-        <x:v>Surestep implements the missing paginated Quest water settings and adds optional tracked-hand ray/pinch menu input. Xbox down selects Blink and left cycles stocked, unlocked damage arrows outside menus/quiver. Tracking loss, held-pinch acquisition and controller handover are explicit software gates in tests/surestep-browser.py. Full accessibility/remapping and physical-device approval remain open. Returning Bell interactions retain direct Xbox controls; the AR Architect's Table shares controller-ray/stick and joint-pinch menus. Game-owned confirmations still use the existing save guard.</x:v>
+        <x:v>Surestep implements the missing paginated Quest water settings and adds optional tracked-hand ray/pinch menu input. Xbox down selects Blink and left cycles stocked, unlocked damage arrows outside menus/quiver. Tracking loss, held-pinch acquisition and controller handover are explicit software gates in tests/surestep-browser.py. Full accessibility/remapping and physical-device approval remain open. Returning Bell interactions retain direct Xbox controls; the AR Architect's Table shares controller-ray/stick and joint-pinch menus. Game-owned confirmations still use the existing save guard. Goldwind adds an opt-in physical bow preset; exact model, native input and publication outcomes belong in its versioned evidence receipt. Classic/crossbow and Xbox remain. Real-device ergonomics and human acceptance are not closed.</x:v>
       </x:c>
       <x:c r="L46" s="6" t="str">
         <x:v>dominion-controls.js
@@ -2997,10 +3028,15 @@
 tests/dominions-browser.py
 SURESTEP.md
 returning-bell.js
-tests/returning-bell-browser.py</x:v>
+tests/returning-bell-browser.py
+GOLDWIND.md
+goldwind-model.js
+goldwind-xr.js
+tests/goldwind.test.cjs
+tests/goldwind-browser.py</x:v>
       </x:c>
       <x:c r="M46" s="6" t="str">
-        <x:v>0.13.0</x:v>
+        <x:v>0.16.0 Goldwind</x:v>
       </x:c>
       <x:c r="N46" s="6" t="str">
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/dominion-controls.js</x:v>
@@ -3142,7 +3178,7 @@
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/resonance-audio.js</x:v>
       </x:c>
     </x:row>
-    <x:row r="50" ht="124" customHeight="1">
+    <x:row r="50" ht="195" customHeight="1">
       <x:c r="A50" s="6" t="str">
         <x:v>V45</x:v>
       </x:c>
@@ -3171,18 +3207,23 @@
         <x:v>Move information and decisions into the physical archery loop.</x:v>
       </x:c>
       <x:c r="J50" s="6" t="str">
-        <x:v>Palm-up status, near-hand trigger pulls, six-arrow selection and a three-second slow-time reserve work without slowing headset tracking.</x:v>
+        <x:v>Palm-up status, near-hand trigger pulls, six-arrow selection and a three-second slow-time reserve work without slowing headset tracking. Classic retains six-arrow radial selection. Goldwind reveals five damage-arrow models near the bow; a fresh other-hand trigger at a stocked arrow selects it. Travel is a separate gesture.</x:v>
       </x:c>
       <x:c r="K50" s="6" t="str">
-        <x:v>Software release evidence; hardware and human gates remain separate.</x:v>
+        <x:v>Software release evidence; hardware and human gates remain separate. Goldwind adds an opt-in physical bow preset; exact model, native input and publication outcomes belong in its versioned evidence receipt. Classic/crossbow and Xbox remain. Real-device ergonomics and human acceptance are not closed.</x:v>
       </x:c>
       <x:c r="L50" s="6" t="str">
         <x:v>ritual-model.js
 resonance-ritual.js
-tests/resonant-browser.py</x:v>
+tests/resonant-browser.py
+GOLDWIND.md
+goldwind-model.js
+goldwind-xr.js
+tests/goldwind.test.cjs
+tests/goldwind-browser.py</x:v>
       </x:c>
       <x:c r="M50" s="6" t="str">
-        <x:v>0.8.0</x:v>
+        <x:v>0.16.0 Goldwind</x:v>
       </x:c>
       <x:c r="N50" s="6" t="str">
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/ritual-model.js</x:v>
@@ -3331,7 +3372,7 @@
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
       </x:c>
     </x:row>
-    <x:row r="54" ht="124" customHeight="1">
+    <x:row r="54" ht="195" customHeight="1">
       <x:c r="A54" s="6" t="str">
         <x:v>V49</x:v>
       </x:c>
@@ -3363,15 +3404,20 @@
         <x:v>A new player can learn nock/draw, cancel, reload, shield, Blink, shard step, pickups and quiver in either handedness, then enter a short scored encounter. Record completion, confusion and fatigue.</x:v>
       </x:c>
       <x:c r="K54" s="6" t="str">
-        <x:v>Ten playable lessons now verify actual outcomes, with device-specific hints and a spatial Quest coach. Skips are recorded separately. Software-only: first-user confusion, reversed-hand ergonomics and fatigue remain to be measured. Returning Bell replaces the default fresh opening; all guided First Bell lessons remain explicitly available. Physical onboarding and newcomer study remain open.</x:v>
+        <x:v>Ten playable lessons now verify actual outcomes, with device-specific hints and a spatial Quest coach. Skips are recorded separately. Software-only: first-user confusion, reversed-hand ergonomics and fatigue remain to be measured. Returning Bell replaces the default fresh opening; all guided First Bell lessons remain explicitly available. Physical onboarding and newcomer study remain open. Goldwind adds an opt-in physical bow preset; exact model, native input and publication outcomes belong in its versioned evidence receipt. Classic/crossbow and Xbox remain. Real-device ergonomics and human acceptance are not closed.</x:v>
       </x:c>
       <x:c r="L54" s="6" t="str">
         <x:v>first-bell.js
 tests/first-bell-browser.py
-returning-bell.js</x:v>
+returning-bell.js
+GOLDWIND.md
+goldwind-model.js
+goldwind-xr.js
+tests/goldwind.test.cjs
+tests/goldwind-browser.py</x:v>
       </x:c>
       <x:c r="M54" s="6" t="str">
-        <x:v>0.10.0 First Bell</x:v>
+        <x:v>0.16.0 Goldwind</x:v>
       </x:c>
       <x:c r="N54" s="6" t="str">
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/first-bell.js</x:v>
@@ -4035,7 +4081,7 @@
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
       </x:c>
     </x:row>
-    <x:row r="70" ht="148" customHeight="1">
+    <x:row r="70" ht="195" customHeight="1">
       <x:c r="A70" s="6" t="str">
         <x:v>V65</x:v>
       </x:c>
@@ -4067,19 +4113,24 @@
         <x:v>Keep fixtures for old supported generator/schema versions, offer explicit local backup/restore and verify interrupted writes, browser quota and update migration. Never silently reset incompatible saves. Any future discrete-hit-point conversion must specify health/healing balance and tested checkpoint migration; retain current health and profiles in presentation-only releases.</x:v>
       </x:c>
       <x:c r="K70" s="6" t="str">
-        <x:v>Legacy hollow-dominions-1 and returning-bell-1 fixtures remain. Open Line adds returning-bell-2 and captures/restores the actual layout identity; mechanism geometry is rebuilt before supported-position checks, including a player saved inside the raised-screen crossing. This compatibility work does not complete export, backup, storage eviction or general migration tooling.</x:v>
+        <x:v>Legacy hollow-dominions-1 and returning-bell-1 fixtures remain. Open Line adds returning-bell-2 and captures/restores the actual layout identity; mechanism geometry is rebuilt before supported-position checks, including a player saved inside the raised-screen crossing. This compatibility work does not complete export, backup, storage eviction or general migration tooling. Goldwind adds an opt-in physical bow preset; exact model, native input and publication outcomes belong in its versioned evidence receipt. Classic/crossbow and Xbox remain. Real-device ergonomics and human acceptance are not closed.</x:v>
       </x:c>
       <x:c r="L70" s="6" t="str">
         <x:v>OPEN-LINE.md
 returning-bell-lanes.js
 tests/open-line.test.cjs
-tests/open-line-browser.py</x:v>
+tests/open-line-browser.py
+GOLDWIND.md
+goldwind-model.js
+goldwind-xr.js
+tests/goldwind.test.cjs
+tests/goldwind-browser.py</x:v>
       </x:c>
       <x:c r="M70" s="6" t="str">
-        <x:v>0.15.0 Open Line</x:v>
+        <x:v>0.16.0 Goldwind</x:v>
       </x:c>
       <x:c r="N70" s="6" t="str">
-        <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
+        <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/OPEN-LINE.md</x:v>
       </x:c>
     </x:row>
     <x:row r="71" ht="176" customHeight="1">
@@ -4164,7 +4215,7 @@
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
       </x:c>
     </x:row>
-    <x:row r="73" ht="190" customHeight="1">
+    <x:row r="73" ht="195" customHeight="1">
       <x:c r="A73" s="6" t="str">
         <x:v>V68</x:v>
       </x:c>
@@ -4184,7 +4235,7 @@
         <x:v>Foundation</x:v>
       </x:c>
       <x:c r="G73" s="6" t="str">
-        <x:v>Engineering</x:v>
+        <x:v>Engineering / assignment pending</x:v>
       </x:c>
       <x:c r="H73" s="6" t="str">
         <x:v>V48, V65</x:v>
@@ -4196,7 +4247,7 @@
         <x:v>For every finished upgrade, test the actual scoped source, commit and merge without overwriting sibling games, verify GitHub Pages deployment plus public runtime/asset/plan/workbook bytes, then launch the public game. Separate source, test, deployment, hardware and human evidence. Retry transient GitHub faults with backoff; inspect failed jobs instead of polling an unchanged failure list. Preserve explicit rollback and save-compatibility notes.</x:v>
       </x:c>
       <x:c r="K73" s="6" t="str">
-        <x:v>Open Line retains exact-source model/workbook checks, four controller-driven route comparisons, full first-person VR/AR/hand/save regression and separate public-byte/launch verification. Preserve unsuccessful receipts and separate model, rendered software, physical-device and human evidence. Public success is recorded only in the matching publication receipt.</x:v>
+        <x:v>Open Line retains exact-source model/workbook checks, four controller-driven route comparisons, full first-person VR/AR/hand/save regression and separate public-byte/launch verification. Preserve unsuccessful receipts and separate model, rendered software, physical-device and human evidence. Public success is recorded only in the matching publication receipt. Goldwind adds an opt-in physical bow preset; exact model, native input and publication outcomes belong in its versioned evidence receipt. Classic/crossbow and Xbox remain. Real-device ergonomics and human acceptance are not closed.</x:v>
       </x:c>
       <x:c r="L73" s="6" t="str">
         <x:v>tests/verify-live.py
@@ -4207,10 +4258,15 @@
 OPEN-LINE.md
 returning-bell-lanes.js
 tests/open-line.test.cjs
-tests/open-line-browser.py</x:v>
+tests/open-line-browser.py
+GOLDWIND.md
+goldwind-model.js
+goldwind-xr.js
+tests/goldwind.test.cjs
+tests/goldwind-browser.py</x:v>
       </x:c>
       <x:c r="M73" s="6" t="str">
-        <x:v>0.15.0 Open Line</x:v>
+        <x:v>0.16.0 Goldwind</x:v>
       </x:c>
       <x:c r="N73" s="6" t="str">
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/tests/verify-live.py</x:v>
@@ -4603,7 +4659,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R373c21fad46c4e38"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R958360007258475a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4905,7 +4961,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R76b144a13271420c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb645a74757f84a3a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5021,10 +5077,10 @@
         <x:v>Both handedness settings</x:v>
       </x:c>
       <x:c r="D6" s="6" t="str">
-        <x:v>Draw, cancel, physical/button reload, shield, quiver and pickup pull</x:v>
+        <x:v>Classic and Goldwind bow, both handedness settings, near-nock face-button travel, deliberate disk release/drop, shield-binding alternatives, physical quiver and retained crossbow</x:v>
       </x:c>
       <x:c r="E6" s="6" t="str">
-        <x:v>V08,V25,V61</x:v>
+        <x:v>V02,V04,V18,V24,V25,V45,V61</x:v>
       </x:c>
       <x:c r="F6" s="6" t="str">
         <x:v>Not run</x:v>
@@ -5125,7 +5181,7 @@
         <x:v>Sleep / visibility / tracking</x:v>
       </x:c>
       <x:c r="D10" s="6" t="str">
-        <x:v>Suspend while drawing, hide/unhide, end session, continue checkpoint and floor alignment</x:v>
+        <x:v>Suspend while drawing or holding/flying disk; hand/controller changes; held input acquisition; no stray release or save loss</x:v>
       </x:c>
       <x:c r="E10" s="6" t="str">
         <x:v>V75</x:v>
@@ -5337,7 +5393,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra624d9879f0446de"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R037fb1aaadb14064"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5683,7 +5739,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd8221a135a074da9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R46a5c22e2a4c4f25"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6101,7 +6157,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf2a3309bdb014552"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R732fc0fbe20745ae"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Implement Pilgrimage 0.17.0 generated chapters and default Goldwind with synchronized production records
</commit_message>
<xml_diff>
--- a/vesperfall/AAA-PRODUCTION.xlsx
+++ b/vesperfall/AAA-PRODUCTION.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="R25c4428087cd417a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="2" r:id="R00092acda6d0464c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Milestones" sheetId="3" r:id="R82e512fbaf704c45"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Device QA" sheetId="4" r:id="R56a1554f64cf41ec"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="5" r:id="Rff4599357f8c4c0e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risk Register" sheetId="6" r:id="R3f4c801032044f33"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="Rc50c1ceff00f4f12"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="2" r:id="Rce9ecfbbab764395"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Milestones" sheetId="3" r:id="Rbe121485c9f04f01"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Device QA" sheetId="4" r:id="R8b67e3760ecd48c2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="5" r:id="Rd1420e2d8d284c41"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risk Register" sheetId="6" r:id="Rfec055500df44bf3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -628,7 +628,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="12" t="str">
-        <x:v>v0.16.0 / Goldwind / 2026-09-17. Opt-in physical bow: golden teleport draw, thrown escape disk, directional shield and reach quiver. Open Line geography, Classic/crossbow, Xbox and all saved layouts remain.</x:v>
+        <x:v>v0.17.0 / Pilgrimage / September 17, 2026. Goldwind defaults; two seeded chapter families link shooting, crossing, galleries and service returns. Explicit Classic preferences and all legacy saves remain.</x:v>
       </x:c>
       <x:c r="B3" s="12"/>
       <x:c r="C3" s="12"/>
@@ -774,7 +774,7 @@
     </x:row>
     <x:row r="15" ht="24" customHeight="1">
       <x:c r="A15" s="6" t="str">
-        <x:v>Prove the physical actions inside the existing cathedral before extending modular generation. Real arrow flight, supported landings and deliberate throws matter more than adding rooms. No new enemy roster or second chapter is included.</x:v>
+        <x:v>Two complete chapter families, not arbitrary room scatter: Lantern Causeway exposure contrasts with Ashen Archive stacks and ceilings. Ordinary recovery, real relay shots and saved return gates remain central.</x:v>
       </x:c>
       <x:c r="B15" s="6"/>
       <x:c r="C15" s="6"/>
@@ -838,7 +838,7 @@
     </x:row>
     <x:row r="21" ht="24" customHeight="1">
       <x:c r="A21" s="6" t="str">
-        <x:v>Next: physical Quest/Xbox and unfamiliar/repeat-player observation of Goldwind in Open Line; then reusable authored encounter relationships, separate travel/shot validation and deterministic streams.</x:v>
+        <x:v>Next: test whether fresh and returning players predict shutter exposure, recognize the service return, and choose another shot angle. Extend the module catalogue only after those observations.</x:v>
       </x:c>
       <x:c r="B21" s="6"/>
       <x:c r="C21" s="6"/>
@@ -870,7 +870,7 @@
     </x:row>
     <x:row r="24" ht="24" customHeight="1">
       <x:c r="A24" s="6" t="str">
-        <x:v>Use GOLDWIND.md and its exact publication receipt. Model fixtures, rendered synthetic input, public bytes, physical hardware and human enjoyment are separate evidence. No device or human gate is certified.</x:v>
+        <x:v>Read PILGRIMAGE.md and its exact public receipt. Model samples, rendered synthetic input, public bytes, physical hardware and human understanding are separate evidence. No hardware or human gate is certified.</x:v>
       </x:c>
       <x:c r="B24" s="6"/>
       <x:c r="C24" s="6"/>
@@ -902,7 +902,7 @@
     </x:row>
     <x:row r="27" ht="24" customHeight="1">
       <x:c r="A27" s="34" t="str">
-        <x:v>Canonical roadmap.json SHA-256: 0189dec4b3dbf791dd5ac6eb7c8f913c64280c5766dfb472cb8fe5166791dfb7</x:v>
+        <x:v>Canonical roadmap.json SHA-256: d5c978532a19bdc3e6310501421c700d7d2b39a64a878251531654e5e9b0c6dd</x:v>
       </x:c>
       <x:c r="B27" s="34"/>
       <x:c r="C27" s="34"/>
@@ -960,7 +960,7 @@
     </x:row>
     <x:row r="32" ht="24" customHeight="1">
       <x:c r="A32" s="36" t="str">
-        <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/CONTINUATION-AUDIT.md</x:v>
+        <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/PILGRIMAGE.md</x:v>
       </x:c>
       <x:c r="B32" s="36"/>
       <x:c r="C32" s="36"/>
@@ -994,7 +994,7 @@
     </x:row>
     <x:row r="36" ht="46" customHeight="1">
       <x:c r="A36" s="42" t="str">
-        <x:v>V68 / V66: verify the actual 0.12 baseline. Do not treat a successful Pages build, a draft test count or historical Rosefire tests as Tidelight gameplay acceptance.</x:v>
+        <x:v>V52 / V50 / V64: observe purposeful choices in both generated chapters, not merely successful completion or room count.</x:v>
       </x:c>
       <x:c r="B36" s="42"/>
       <x:c r="C36" s="42"/>
@@ -1006,7 +1006,7 @@
     </x:row>
     <x:row r="37" ht="46" customHeight="1">
       <x:c r="A37" s="46" t="str">
-        <x:v>V41 / V61 / V74: finish Quest water settings and verify all Xbox/Quest open, adjust, select, dismiss and recovery paths. Reproduce water footprint, height, ripple-budget and world-clock gaps.</x:v>
+        <x:v>V02 / V04 / V24 / V62: validate default Goldwind, alternate Classic, both handedness roles and real physical throw/draw recovery.</x:v>
       </x:c>
       <x:c r="B37" s="46"/>
       <x:c r="C37" s="46"/>
@@ -1018,7 +1018,7 @@
     </x:row>
     <x:row r="38" ht="46" customHeight="1">
       <x:c r="A38" s="42" t="str">
-        <x:v>V58 / V44: implement water-specific sound, stronger archery/shield/enemy audio and musical transitions. Preserve independent volume buses, mute, captions and warning clarity.</x:v>
+        <x:v>V15 / V65 / V66: retain all five layout readers, stable seeds and tiers, mechanism-first restore and one-time rewards.</x:v>
       </x:c>
       <x:c r="B38" s="42"/>
       <x:c r="C38" s="42"/>
@@ -1030,7 +1030,7 @@
     </x:row>
     <x:row r="39" ht="46" customHeight="1">
       <x:c r="A39" s="46" t="str">
-        <x:v>V35 / V52 / V54: pursue memorable routes, water destinations and humanoid animation; retain the existing 15 enemy archetypes, First Bell and Bellkeeper Oath.</x:v>
+        <x:v>V56 / V57 / V58: strengthen chapter-specific visual and audio communication after actual route review, without hiding geometry problems.</x:v>
       </x:c>
       <x:c r="B39" s="46"/>
       <x:c r="C39" s="46"/>
@@ -1042,7 +1042,7 @@
     </x:row>
     <x:row r="40" ht="46" customHeight="1">
       <x:c r="A40" s="42" t="str">
-        <x:v>V38 / V59 / V62 / V75: run actual-device comfort, thermal, performance, controller and save-lifecycle checks. Proposed timing budgets are not measurements.</x:v>
+        <x:v>V59 / V62 / V75 / V68: record physical performance and lifecycle; verify published bytes and preserve unsuccessful test evidence.</x:v>
       </x:c>
       <x:c r="B40" s="42"/>
       <x:c r="C40" s="42"/>
@@ -1142,7 +1142,7 @@
     </x:row>
     <x:row r="3" ht="36" customHeight="1">
       <x:c r="A3" s="12" t="str">
-        <x:v>v0.12.0 / 76 preserved tasks / September 13 source audit. Partial means the expanded acceptance scope remains open.</x:v>
+        <x:v>v0.17.0 / 76 preserved tasks / Pilgrimage. Partial means the full original acceptance gate remains open.</x:v>
       </x:c>
       <x:c r="B3" s="12"/>
       <x:c r="C3" s="12"/>
@@ -1238,7 +1238,7 @@
         <x:v>Foundation</x:v>
       </x:c>
       <x:c r="G6" s="6" t="str">
-        <x:v>Engineering / assignment pending</x:v>
+        <x:v>Engineering</x:v>
       </x:c>
       <x:c r="H6" s="6" t="str">
         <x:v>None</x:v>
@@ -1264,7 +1264,7 @@
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/index.html</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="195" customHeight="1">
+    <x:row r="7" ht="190" customHeight="1">
       <x:c r="A7" s="6" t="str">
         <x:v>V02</x:v>
       </x:c>
@@ -1284,7 +1284,7 @@
         <x:v>Archery</x:v>
       </x:c>
       <x:c r="G7" s="6" t="str">
-        <x:v>Gameplay / assignment pending</x:v>
+        <x:v>Gameplay</x:v>
       </x:c>
       <x:c r="H7" s="6" t="str">
         <x:v>None</x:v>
@@ -1296,7 +1296,7 @@
         <x:v>Real controller poses produce direction and power; losses never fire a stale arrow.</x:v>
       </x:c>
       <x:c r="K7" s="6" t="str">
-        <x:v>Source implemented; software regression coverage. Physical acceptance is separate. Goldwind adds an opt-in physical bow preset; exact model, native input and publication outcomes belong in its versioned evidence receipt. Classic/crossbow and Xbox remain. Real-device ergonomics and human acceptance are not closed.</x:v>
+        <x:v>Pilgrimage 0.17.0: Goldwind now defaults for fresh settings; explicitly stored Classic remains available. Both presets are tested intentionally rather than mislabeling old-control tests as new-default tests. Earlier implementation evidence remains in the referenced release notes. Exact accepted revisions belong in publication receipts; hardware and human gates remain separate.</x:v>
       </x:c>
       <x:c r="L7" s="6" t="str">
         <x:v>input.js
@@ -1306,10 +1306,16 @@
 goldwind-model.js
 goldwind-xr.js
 tests/goldwind.test.cjs
-tests/goldwind-browser.py</x:v>
+tests/goldwind-browser.py
+PILGRIMAGE.md
+pilgrimage-model.js
+pilgrimage-view.js
+tests/pilgrimage.test.cjs
+tests/pilgrimage-driver.cjs
+tests/pilgrimage-browser.py</x:v>
       </x:c>
       <x:c r="M7" s="6" t="str">
-        <x:v>0.16.0 Goldwind</x:v>
+        <x:v>0.17.0 Pilgrimage</x:v>
       </x:c>
       <x:c r="N7" s="6" t="str">
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/input.js</x:v>
@@ -1335,7 +1341,7 @@
         <x:v>Combat</x:v>
       </x:c>
       <x:c r="G8" s="6" t="str">
-        <x:v>Gameplay / assignment pending</x:v>
+        <x:v>Gameplay</x:v>
       </x:c>
       <x:c r="H8" s="6" t="str">
         <x:v>None</x:v>
@@ -1360,7 +1366,7 @@
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/core.js</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="195" customHeight="1">
+    <x:row r="9" ht="190" customHeight="1">
       <x:c r="A9" s="6" t="str">
         <x:v>V04</x:v>
       </x:c>
@@ -1380,7 +1386,7 @@
         <x:v>Traversal</x:v>
       </x:c>
       <x:c r="G9" s="6" t="str">
-        <x:v>Level design / assignment pending</x:v>
+        <x:v>Level design</x:v>
       </x:c>
       <x:c r="H9" s="6" t="str">
         <x:v>None</x:v>
@@ -1392,23 +1398,29 @@
         <x:v>Shared projectile/preview first-hit collision; a widened upper-gallery target. A clear preview is not automatic aiming or permission to pass through solids. Goldwind travel is a temporary physically nocked golden arrow, not an equipment toggle. Its default hides arc/ring; an optional drawing-only path cannot authorize invalid landings.</x:v>
       </x:c>
       <x:c r="K9" s="6" t="str">
-        <x:v>Source implemented; software regression coverage. Physical acceptance is separate. Goldwind adds an opt-in physical bow preset; exact model, native input and publication outcomes belong in its versioned evidence receipt. Classic/crossbow and Xbox remain. Real-device ergonomics and human acceptance are not closed.</x:v>
+        <x:v>Pilgrimage 0.17.0: The new catalogue records supported upper landing surfaces and separate projectile connections. Low and arcing Blink trajectories use actual launch curves and collision; Archive roofs legitimately reject obstructed high arcs. Earlier implementation evidence remains in the referenced release notes. Exact accepted revisions belong in publication receipts; hardware and human gates remain separate.</x:v>
       </x:c>
       <x:c r="L9" s="6" t="str">
         <x:v>GOLDWIND.md
 goldwind-model.js
 goldwind-xr.js
 tests/goldwind.test.cjs
-tests/goldwind-browser.py</x:v>
+tests/goldwind-browser.py
+PILGRIMAGE.md
+pilgrimage-model.js
+pilgrimage-view.js
+tests/pilgrimage.test.cjs
+tests/pilgrimage-driver.cjs
+tests/pilgrimage-browser.py</x:v>
       </x:c>
       <x:c r="M9" s="6" t="str">
-        <x:v>0.16.0 Goldwind</x:v>
+        <x:v>0.17.0 Pilgrimage</x:v>
       </x:c>
       <x:c r="N9" s="6" t="str">
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/GOLDWIND.md</x:v>
       </x:c>
     </x:row>
-    <x:row r="10" ht="124" customHeight="1">
+    <x:row r="10" ht="190" customHeight="1">
       <x:c r="A10" s="6" t="str">
         <x:v>V05</x:v>
       </x:c>
@@ -1428,7 +1440,7 @@
         <x:v>World</x:v>
       </x:c>
       <x:c r="G10" s="6" t="str">
-        <x:v>Level design / assignment pending</x:v>
+        <x:v>Level design</x:v>
       </x:c>
       <x:c r="H10" s="6" t="str">
         <x:v>None</x:v>
@@ -1440,14 +1452,20 @@
         <x:v>25 seeded districts with nonuniform plans, connected ground approaches and reversible elevated loops. Same seed/depth reproduces the layout. No streaming-world claim.</x:v>
       </x:c>
       <x:c r="K10" s="6" t="str">
-        <x:v>Source implemented; software regression coverage. Physical acceptance is separate.</x:v>
+        <x:v>Pilgrimage 0.17.0: Pilgrimage adds a bounded catalogue assembler with mirrored module sides, distinct tile families, tested ground sockets, separate random streams and immutable chapter identifiers. This is not arbitrary WFC or recovered In Death source. Earlier implementation evidence remains in the referenced release notes. Exact accepted revisions belong in publication receipts; hardware and human gates remain separate.</x:v>
       </x:c>
       <x:c r="L10" s="6" t="str">
         <x:v>dominions-world.js
-tests/dominions.test.cjs</x:v>
+tests/dominions.test.cjs
+PILGRIMAGE.md
+pilgrimage-model.js
+pilgrimage-view.js
+tests/pilgrimage.test.cjs
+tests/pilgrimage-driver.cjs
+tests/pilgrimage-browser.py</x:v>
       </x:c>
       <x:c r="M10" s="6" t="str">
-        <x:v>0.7.0</x:v>
+        <x:v>0.17.0 Pilgrimage</x:v>
       </x:c>
       <x:c r="N10" s="6" t="str">
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/dominions-world.js</x:v>
@@ -1473,7 +1491,7 @@
         <x:v>Progression</x:v>
       </x:c>
       <x:c r="G11" s="6" t="str">
-        <x:v>Engineering / assignment pending</x:v>
+        <x:v>Engineering</x:v>
       </x:c>
       <x:c r="H11" s="6" t="str">
         <x:v>None</x:v>
@@ -1519,7 +1537,7 @@
         <x:v>Comfort</x:v>
       </x:c>
       <x:c r="G12" s="6" t="str">
-        <x:v>UX / accessibility / assignment pending</x:v>
+        <x:v>UX / accessibility</x:v>
       </x:c>
       <x:c r="H12" s="6" t="str">
         <x:v>None</x:v>
@@ -1561,7 +1579,7 @@
         <x:v>Hardware</x:v>
       </x:c>
       <x:c r="G13" s="6" t="str">
-        <x:v>Device QA / assignment pending</x:v>
+        <x:v>Device QA</x:v>
       </x:c>
       <x:c r="H13" s="6" t="str">
         <x:v>None</x:v>
@@ -1601,7 +1619,7 @@
         <x:v>Hardware</x:v>
       </x:c>
       <x:c r="G14" s="6" t="str">
-        <x:v>Device QA / assignment pending</x:v>
+        <x:v>Device QA</x:v>
       </x:c>
       <x:c r="H14" s="6" t="str">
         <x:v>None</x:v>
@@ -1641,7 +1659,7 @@
         <x:v>Hardware</x:v>
       </x:c>
       <x:c r="G15" s="6" t="str">
-        <x:v>Device QA / assignment pending</x:v>
+        <x:v>Device QA</x:v>
       </x:c>
       <x:c r="H15" s="6" t="str">
         <x:v>None</x:v>
@@ -1681,7 +1699,7 @@
         <x:v>World</x:v>
       </x:c>
       <x:c r="G16" s="6" t="str">
-        <x:v>Level design / assignment pending</x:v>
+        <x:v>Level design</x:v>
       </x:c>
       <x:c r="H16" s="6" t="str">
         <x:v>None</x:v>
@@ -1727,7 +1745,7 @@
         <x:v>Archery</x:v>
       </x:c>
       <x:c r="G17" s="6" t="str">
-        <x:v>Gameplay / assignment pending</x:v>
+        <x:v>Gameplay</x:v>
       </x:c>
       <x:c r="H17" s="6" t="str">
         <x:v>None</x:v>
@@ -1773,7 +1791,7 @@
         <x:v>Combat</x:v>
       </x:c>
       <x:c r="G18" s="6" t="str">
-        <x:v>Gameplay / assignment pending</x:v>
+        <x:v>Gameplay</x:v>
       </x:c>
       <x:c r="H18" s="6" t="str">
         <x:v>V26</x:v>
@@ -1843,7 +1861,7 @@
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/resonance-audio.js</x:v>
       </x:c>
     </x:row>
-    <x:row r="20" ht="124" customHeight="1">
+    <x:row r="20" ht="190" customHeight="1">
       <x:c r="A20" s="6" t="str">
         <x:v>V15</x:v>
       </x:c>
@@ -1863,7 +1881,7 @@
         <x:v>Progression</x:v>
       </x:c>
       <x:c r="G20" s="6" t="str">
-        <x:v>Engineering / assignment pending</x:v>
+        <x:v>Engineering</x:v>
       </x:c>
       <x:c r="H20" s="6" t="str">
         <x:v>V06, V21</x:v>
@@ -1875,16 +1893,22 @@
         <x:v>Regenerate the exact world; restore enemies, supplies, projectiles, equipment and timers; preserve banked receipts in one bounded envelope. Continue waits paused. Practice/AR cannot overwrite scored saves.</x:v>
       </x:c>
       <x:c r="K20" s="6" t="str">
-        <x:v>Model and native browser/controller release gates; physical lifecycle QA remains open.</x:v>
+        <x:v>Pilgrimage 0.17.0: Both new chapter identities, tier snapshot, geometry signature, relay targets, shutters and persistent service gates restore before supported player positions are accepted. Interrupted arrows and a checkpoint inside an opened gate are tested. Earlier implementation evidence remains in the referenced release notes. Exact accepted revisions belong in publication receipts; hardware and human gates remain separate.</x:v>
       </x:c>
       <x:c r="L20" s="6" t="str">
         <x:v>pilgrim-save.js
 pilgrim-rest.js
 tests/pilgrim.test.cjs
-tests/pilgrim-browser.py</x:v>
+tests/pilgrim-browser.py
+PILGRIMAGE.md
+pilgrimage-model.js
+pilgrimage-view.js
+tests/pilgrimage.test.cjs
+tests/pilgrimage-driver.cjs
+tests/pilgrimage-browser.py</x:v>
       </x:c>
       <x:c r="M20" s="6" t="str">
-        <x:v>0.9.0</x:v>
+        <x:v>0.17.0 Pilgrimage</x:v>
       </x:c>
       <x:c r="N20" s="6" t="str">
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/pilgrim-save.js</x:v>
@@ -1910,7 +1934,7 @@
         <x:v>Testing</x:v>
       </x:c>
       <x:c r="G21" s="6" t="str">
-        <x:v>QA / play research / assignment pending</x:v>
+        <x:v>QA / play research</x:v>
       </x:c>
       <x:c r="H21" s="6" t="str">
         <x:v>None</x:v>
@@ -1950,7 +1974,7 @@
         <x:v>Online</x:v>
       </x:c>
       <x:c r="G22" s="6" t="str">
-        <x:v>Online engineering / assignment pending</x:v>
+        <x:v>Online engineering</x:v>
       </x:c>
       <x:c r="H22" s="6" t="str">
         <x:v>None</x:v>
@@ -1990,7 +2014,7 @@
         <x:v>Combat</x:v>
       </x:c>
       <x:c r="G23" s="6" t="str">
-        <x:v>Gameplay / assignment pending</x:v>
+        <x:v>Gameplay</x:v>
       </x:c>
       <x:c r="H23" s="6" t="str">
         <x:v>None</x:v>
@@ -2038,7 +2062,7 @@
         <x:v>Traversal</x:v>
       </x:c>
       <x:c r="G24" s="6" t="str">
-        <x:v>Level design / assignment pending</x:v>
+        <x:v>Level design</x:v>
       </x:c>
       <x:c r="H24" s="6" t="str">
         <x:v>None</x:v>
@@ -2086,7 +2110,7 @@
         <x:v>Archery</x:v>
       </x:c>
       <x:c r="G25" s="6" t="str">
-        <x:v>Gameplay / assignment pending</x:v>
+        <x:v>Gameplay</x:v>
       </x:c>
       <x:c r="H25" s="6" t="str">
         <x:v>None</x:v>
@@ -2128,7 +2152,7 @@
         <x:v>Progression</x:v>
       </x:c>
       <x:c r="G26" s="6" t="str">
-        <x:v>Engineering / assignment pending</x:v>
+        <x:v>Engineering</x:v>
       </x:c>
       <x:c r="H26" s="6" t="str">
         <x:v>None</x:v>
@@ -2174,7 +2198,7 @@
         <x:v>Presentation</x:v>
       </x:c>
       <x:c r="G27" s="6" t="str">
-        <x:v>Art / audio / assignment pending</x:v>
+        <x:v>Art / audio</x:v>
       </x:c>
       <x:c r="H27" s="6" t="str">
         <x:v>None</x:v>
@@ -2220,7 +2244,7 @@
         <x:v>Testing</x:v>
       </x:c>
       <x:c r="G28" s="6" t="str">
-        <x:v>QA / play research / assignment pending</x:v>
+        <x:v>QA / play research</x:v>
       </x:c>
       <x:c r="H28" s="6" t="str">
         <x:v>None</x:v>
@@ -2243,7 +2267,7 @@
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/tests/unchained-combat.py</x:v>
       </x:c>
     </x:row>
-    <x:row r="29" ht="195" customHeight="1">
+    <x:row r="29" ht="190" customHeight="1">
       <x:c r="A29" s="6" t="str">
         <x:v>V24</x:v>
       </x:c>
@@ -2263,7 +2287,7 @@
         <x:v>Traversal</x:v>
       </x:c>
       <x:c r="G29" s="6" t="str">
-        <x:v>Level design / assignment pending</x:v>
+        <x:v>Level design</x:v>
       </x:c>
       <x:c r="H29" s="6" t="str">
         <x:v>None</x:v>
@@ -2275,17 +2299,23 @@
         <x:v>Readable trajectories, safe valid landings, comfortable two-handed controls and alternative routes; no forced headset motion.</x:v>
       </x:c>
       <x:c r="K29" s="6" t="str">
-        <x:v>Physical disk acquisition, recent-motion release recognition, swept flight and supported-ground relocation are implemented for the Goldwind bow preset. A drop, pose jump, missing tracking or blocked impact cannot teleport. Richer generated route families and physical-device approval remain open.</x:v>
+        <x:v>Pilgrimage 0.17.0: The default physical bow and thrown disk now operate in generated court/gallery/service encounter families. Physical-device throw feel, tracking and comfort remain open. Earlier implementation evidence remains in the referenced release notes. Exact accepted revisions belong in publication receipts; hardware and human gates remain separate.</x:v>
       </x:c>
       <x:c r="L29" s="6" t="str">
         <x:v>GOLDWIND.md
 goldwind-model.js
 goldwind-xr.js
 tests/goldwind.test.cjs
-tests/goldwind-browser.py</x:v>
+tests/goldwind-browser.py
+PILGRIMAGE.md
+pilgrimage-model.js
+pilgrimage-view.js
+tests/pilgrimage.test.cjs
+tests/pilgrimage-driver.cjs
+tests/pilgrimage-browser.py</x:v>
       </x:c>
       <x:c r="M29" s="6" t="str">
-        <x:v>0.16.0 Goldwind</x:v>
+        <x:v>0.17.0 Pilgrimage</x:v>
       </x:c>
       <x:c r="N29" s="6" t="str">
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/GOLDWIND.md</x:v>
@@ -2311,7 +2341,7 @@
         <x:v>Archery</x:v>
       </x:c>
       <x:c r="G30" s="6" t="str">
-        <x:v>Gameplay / assignment pending</x:v>
+        <x:v>Gameplay</x:v>
       </x:c>
       <x:c r="H30" s="6" t="str">
         <x:v>V02, V12</x:v>
@@ -2357,7 +2387,7 @@
         <x:v>Combat</x:v>
       </x:c>
       <x:c r="G31" s="6" t="str">
-        <x:v>Gameplay / assignment pending</x:v>
+        <x:v>Gameplay</x:v>
       </x:c>
       <x:c r="H31" s="6" t="str">
         <x:v>None</x:v>
@@ -2399,7 +2429,7 @@
         <x:v>Traversal</x:v>
       </x:c>
       <x:c r="G32" s="6" t="str">
-        <x:v>Level design / assignment pending</x:v>
+        <x:v>Level design</x:v>
       </x:c>
       <x:c r="H32" s="6" t="str">
         <x:v>None</x:v>
@@ -2441,7 +2471,7 @@
         <x:v>Practice</x:v>
       </x:c>
       <x:c r="G33" s="6" t="str">
-        <x:v>Gameplay / UX / assignment pending</x:v>
+        <x:v>Gameplay / UX</x:v>
       </x:c>
       <x:c r="H33" s="6" t="str">
         <x:v>None</x:v>
@@ -2483,7 +2513,7 @@
         <x:v>Archery</x:v>
       </x:c>
       <x:c r="G34" s="6" t="str">
-        <x:v>Gameplay / assignment pending</x:v>
+        <x:v>Gameplay</x:v>
       </x:c>
       <x:c r="H34" s="6" t="str">
         <x:v>None</x:v>
@@ -2525,7 +2555,7 @@
         <x:v>Future</x:v>
       </x:c>
       <x:c r="G35" s="6" t="str">
-        <x:v>Gameplay / assignment pending</x:v>
+        <x:v>Gameplay</x:v>
       </x:c>
       <x:c r="H35" s="6" t="str">
         <x:v>V25</x:v>
@@ -2567,7 +2597,7 @@
         <x:v>Art</x:v>
       </x:c>
       <x:c r="G36" s="6" t="str">
-        <x:v>Technical art / assignment pending</x:v>
+        <x:v>Technical art</x:v>
       </x:c>
       <x:c r="H36" s="6" t="str">
         <x:v>None</x:v>
@@ -2609,7 +2639,7 @@
         <x:v>Traversal</x:v>
       </x:c>
       <x:c r="G37" s="6" t="str">
-        <x:v>Level design / assignment pending</x:v>
+        <x:v>Level design</x:v>
       </x:c>
       <x:c r="H37" s="6" t="str">
         <x:v>None</x:v>
@@ -2651,7 +2681,7 @@
         <x:v>Art</x:v>
       </x:c>
       <x:c r="G38" s="6" t="str">
-        <x:v>Technical art / assignment pending</x:v>
+        <x:v>Technical art</x:v>
       </x:c>
       <x:c r="H38" s="6" t="str">
         <x:v>None</x:v>
@@ -2673,7 +2703,7 @@
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
       </x:c>
     </x:row>
-    <x:row r="39" ht="124" customHeight="1">
+    <x:row r="39" ht="190" customHeight="1">
       <x:c r="A39" s="6" t="str">
         <x:v>V34</x:v>
       </x:c>
@@ -2693,7 +2723,7 @@
         <x:v>Navigation</x:v>
       </x:c>
       <x:c r="G39" s="6" t="str">
-        <x:v>UX / level design / assignment pending</x:v>
+        <x:v>UX / level design</x:v>
       </x:c>
       <x:c r="H39" s="6" t="str">
         <x:v>None</x:v>
@@ -2705,17 +2735,24 @@
         <x:v>Use actual room outlines, gold skywalk and reliquary markers. No player steering or auto-completion.</x:v>
       </x:c>
       <x:c r="K39" s="6" t="str">
-        <x:v>Source implemented; software regression coverage. Physical acceptance is separate.</x:v>
-      </x:c>
-      <x:c r="L39" s="6" t="str"/>
+        <x:v>Pilgrimage 0.17.0: The atlas and in-headset known-places list reflect the actual generated chapter and discovered regions. AR inspection reconstructs its seed, stage, tier and mechanism state, without disclosing undiscovered geometry. Earlier implementation evidence remains in the referenced release notes. Exact accepted revisions belong in publication receipts; hardware and human gates remain separate.</x:v>
+      </x:c>
+      <x:c r="L39" s="6" t="str">
+        <x:v>PILGRIMAGE.md
+pilgrimage-model.js
+pilgrimage-view.js
+tests/pilgrimage.test.cjs
+tests/pilgrimage-driver.cjs
+tests/pilgrimage-browser.py</x:v>
+      </x:c>
       <x:c r="M39" s="6" t="str">
-        <x:v>Baseline through 0.6.0</x:v>
+        <x:v>0.17.0 Pilgrimage</x:v>
       </x:c>
       <x:c r="N39" s="6" t="str">
-        <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="40" ht="120" customHeight="1">
+        <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/PILGRIMAGE.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="190" customHeight="1">
       <x:c r="A40" s="6" t="str">
         <x:v>V35</x:v>
       </x:c>
@@ -2735,7 +2772,7 @@
         <x:v>World</x:v>
       </x:c>
       <x:c r="G40" s="6" t="str">
-        <x:v>Level design / assignment pending</x:v>
+        <x:v>Level design</x:v>
       </x:c>
       <x:c r="H40" s="6" t="str">
         <x:v>None</x:v>
@@ -2747,17 +2784,23 @@
         <x:v>Keep the existing 25-district game and reversible upper/lower routes. Add distinctive, collision-tested destinations, escape paths and discoveries. Tidelight water remains decorative until a separately designed, save-compatible traversal feature is approved.</x:v>
       </x:c>
       <x:c r="K40" s="6" t="str">
-        <x:v>Partial. Tidelight 0.12.0 water exists in current source. The earlier seven-surface/four-named-district draft, recessed fonts, refracting tile basins and architecture reflections are not established by the shipped implementation.</x:v>
+        <x:v>Pilgrimage 0.17.0: The Lantern Causeway uses exposed crossing and wind-gallery relationships; The Ashen Archive uses roofs, columns and alternating stacks to interrupt shot geometry. Both include ordinary service routes and a lasting local return gate. No new water gameplay or swimming is introduced. Earlier implementation evidence remains in the referenced release notes. Exact accepted revisions belong in publication receipts; hardware and human gates remain separate.</x:v>
       </x:c>
       <x:c r="L40" s="6" t="str">
         <x:v>dominions-world.js
 HOLLOW-DOMINIONS.md
 TIDELIGHT.md
 tidelight.js
-CONTINUATION-AUDIT.md</x:v>
+CONTINUATION-AUDIT.md
+PILGRIMAGE.md
+pilgrimage-model.js
+pilgrimage-view.js
+tests/pilgrimage.test.cjs
+tests/pilgrimage-driver.cjs
+tests/pilgrimage-browser.py</x:v>
       </x:c>
       <x:c r="M40" s="6" t="str">
-        <x:v>0.12.0 Tidelight presentation baseline; authored expansion open</x:v>
+        <x:v>0.17.0 Pilgrimage</x:v>
       </x:c>
       <x:c r="N40" s="6" t="str">
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/dominions-world.js</x:v>
@@ -2783,7 +2826,7 @@
         <x:v>Testing</x:v>
       </x:c>
       <x:c r="G41" s="6" t="str">
-        <x:v>QA / play research / assignment pending</x:v>
+        <x:v>QA / play research</x:v>
       </x:c>
       <x:c r="H41" s="6" t="str">
         <x:v>None</x:v>
@@ -2849,7 +2892,7 @@
         <x:v>0.11.0 Rosefire</x:v>
       </x:c>
       <x:c r="N42" s="6" t="str">
-        <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
+        <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/JEWELGLASS.md</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="106" customHeight="1">
@@ -2872,7 +2915,7 @@
         <x:v>Hardware</x:v>
       </x:c>
       <x:c r="G43" s="6" t="str">
-        <x:v>Device QA / assignment pending</x:v>
+        <x:v>Device QA</x:v>
       </x:c>
       <x:c r="H43" s="6" t="str">
         <x:v>None</x:v>
@@ -2916,7 +2959,7 @@
         <x:v>World</x:v>
       </x:c>
       <x:c r="G44" s="6" t="str">
-        <x:v>Level design / assignment pending</x:v>
+        <x:v>Level design</x:v>
       </x:c>
       <x:c r="H44" s="6" t="str">
         <x:v>V05</x:v>
@@ -2961,7 +3004,7 @@
         <x:v>Combat</x:v>
       </x:c>
       <x:c r="G45" s="6" t="str">
-        <x:v>Gameplay / assignment pending</x:v>
+        <x:v>Gameplay</x:v>
       </x:c>
       <x:c r="H45" s="6" t="str">
         <x:v>V26</x:v>
@@ -2987,7 +3030,7 @@
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/bestiary.js</x:v>
       </x:c>
     </x:row>
-    <x:row r="46" ht="195" customHeight="1">
+    <x:row r="46" ht="190" customHeight="1">
       <x:c r="A46" s="6" t="str">
         <x:v>V41</x:v>
       </x:c>
@@ -3007,7 +3050,7 @@
         <x:v>Comfort</x:v>
       </x:c>
       <x:c r="G46" s="6" t="str">
-        <x:v>UX / accessibility / assignment pending</x:v>
+        <x:v>UX / accessibility</x:v>
       </x:c>
       <x:c r="H46" s="6" t="str">
         <x:v>V07</x:v>
@@ -3019,7 +3062,7 @@
         <x:v>Every gameplay and game-owned UI path, including water settings, confirmations, recovery, seed entry, audio and accessibility settings, is reachable and dismissible with Xbox and Quest controls without a mouse. Test both handedness modes, neutral-input transitions and return focus. Browser/system permission prompts remain platform-owned.</x:v>
       </x:c>
       <x:c r="K46" s="6" t="str">
-        <x:v>Surestep implements the missing paginated Quest water settings and adds optional tracked-hand ray/pinch menu input. Xbox down selects Blink and left cycles stocked, unlocked damage arrows outside menus/quiver. Tracking loss, held-pinch acquisition and controller handover are explicit software gates in tests/surestep-browser.py. Full accessibility/remapping and physical-device approval remain open. Returning Bell interactions retain direct Xbox controls; the AR Architect's Table shares controller-ray/stick and joint-pinch menus. Game-owned confirmations still use the existing save guard. Goldwind adds an opt-in physical bow preset; exact model, native input and publication outcomes belong in its versioned evidence receipt. Classic/crossbow and Xbox remain. Real-device ergonomics and human acceptance are not closed.</x:v>
+        <x:v>Pilgrimage 0.17.0: Pilgrimage start, mechanism interactions, chapter rewards, save/continue, journal and known-place menus share existing Xbox and Quest paths. Synthetic acceptance remains distinct from real-device approval. Earlier implementation evidence remains in the referenced release notes. Exact accepted revisions belong in publication receipts; hardware and human gates remain separate.</x:v>
       </x:c>
       <x:c r="L46" s="6" t="str">
         <x:v>dominion-controls.js
@@ -3033,10 +3076,16 @@
 goldwind-model.js
 goldwind-xr.js
 tests/goldwind.test.cjs
-tests/goldwind-browser.py</x:v>
+tests/goldwind-browser.py
+PILGRIMAGE.md
+pilgrimage-model.js
+pilgrimage-view.js
+tests/pilgrimage.test.cjs
+tests/pilgrimage-driver.cjs
+tests/pilgrimage-browser.py</x:v>
       </x:c>
       <x:c r="M46" s="6" t="str">
-        <x:v>0.16.0 Goldwind</x:v>
+        <x:v>0.17.0 Pilgrimage</x:v>
       </x:c>
       <x:c r="N46" s="6" t="str">
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/dominion-controls.js</x:v>
@@ -3062,7 +3111,7 @@
         <x:v>Comfort</x:v>
       </x:c>
       <x:c r="G47" s="6" t="str">
-        <x:v>UX / accessibility / assignment pending</x:v>
+        <x:v>UX / accessibility</x:v>
       </x:c>
       <x:c r="H47" s="6" t="str">
         <x:v>V41</x:v>
@@ -3107,7 +3156,7 @@
         <x:v>Presentation</x:v>
       </x:c>
       <x:c r="G48" s="6" t="str">
-        <x:v>Art / audio / assignment pending</x:v>
+        <x:v>Art / audio</x:v>
       </x:c>
       <x:c r="H48" s="6" t="str">
         <x:v>V22</x:v>
@@ -3153,7 +3202,7 @@
         <x:v>Comfort</x:v>
       </x:c>
       <x:c r="G49" s="6" t="str">
-        <x:v>UX / accessibility / assignment pending</x:v>
+        <x:v>UX / accessibility</x:v>
       </x:c>
       <x:c r="H49" s="6" t="str">
         <x:v>V43, V41</x:v>
@@ -3198,7 +3247,7 @@
         <x:v>Archery</x:v>
       </x:c>
       <x:c r="G50" s="6" t="str">
-        <x:v>Gameplay / assignment pending</x:v>
+        <x:v>Gameplay</x:v>
       </x:c>
       <x:c r="H50" s="6" t="str">
         <x:v>V02, V41</x:v>
@@ -3249,7 +3298,7 @@
         <x:v>Progression</x:v>
       </x:c>
       <x:c r="G51" s="6" t="str">
-        <x:v>Engineering / assignment pending</x:v>
+        <x:v>Engineering</x:v>
       </x:c>
       <x:c r="H51" s="6" t="str">
         <x:v>V20, V21</x:v>
@@ -3295,7 +3344,7 @@
         <x:v>Progression</x:v>
       </x:c>
       <x:c r="G52" s="6" t="str">
-        <x:v>Engineering / assignment pending</x:v>
+        <x:v>Engineering</x:v>
       </x:c>
       <x:c r="H52" s="6" t="str">
         <x:v>V15</x:v>
@@ -3322,7 +3371,7 @@
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/pilgrim-save.js</x:v>
       </x:c>
     </x:row>
-    <x:row r="53" ht="134" customHeight="1">
+    <x:row r="53" ht="190" customHeight="1">
       <x:c r="A53" s="6" t="str">
         <x:v>V48</x:v>
       </x:c>
@@ -3342,7 +3391,7 @@
         <x:v>Foundation</x:v>
       </x:c>
       <x:c r="G53" s="6" t="str">
-        <x:v>Engineering / assignment pending</x:v>
+        <x:v>Engineering</x:v>
       </x:c>
       <x:c r="H53" s="6" t="str">
         <x:v>V15</x:v>
@@ -3354,7 +3403,7 @@
         <x:v>Keep roadmap.json version aligned with release.json and core.js. Preserve V01-V76; export the six-sheet workbook with matching source digest and live summary formulas. Keep DEVELOPMENT-HANDOFF.md and CONTINUATION-AUDIT.md linked from the board and README. Verify committed files, not browser-local edits.</x:v>
       </x:c>
       <x:c r="K53" s="6" t="str">
-        <x:v>September 13 repairs both the stale plan/workbook and the core diagnostic version label, without changing mechanics or save formats. Historical acceptance had 148 model passes and one plan-version failure; fresh checks are recorded separately. Physical/human gates remain open.</x:v>
+        <x:v>Pilgrimage 0.17.0: The 76 stable task IDs and six-sheet workbook remain canonical. Pilgrimage metadata is synchronized; exact accepted source and public results belong in its separate publication receipt. Earlier implementation evidence remains in the referenced release notes. Exact accepted revisions belong in publication receipts; hardware and human gates remain separate.</x:v>
       </x:c>
       <x:c r="L53" s="6" t="str">
         <x:v>roadmap.json
@@ -3363,16 +3412,22 @@
 tests/production.test.cjs
 tests/production-browser.py
 DEVELOPMENT-HANDOFF.md
-CONTINUATION-AUDIT.md</x:v>
+CONTINUATION-AUDIT.md
+PILGRIMAGE.md
+pilgrimage-model.js
+pilgrimage-view.js
+tests/pilgrimage.test.cjs
+tests/pilgrimage-driver.cjs
+tests/pilgrimage-browser.py</x:v>
       </x:c>
       <x:c r="M53" s="6" t="str">
-        <x:v>0.9.0 foundation; 0.12.0 planning synchronization</x:v>
+        <x:v>0.17.0 Pilgrimage</x:v>
       </x:c>
       <x:c r="N53" s="6" t="str">
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
       </x:c>
     </x:row>
-    <x:row r="54" ht="195" customHeight="1">
+    <x:row r="54" ht="190" customHeight="1">
       <x:c r="A54" s="6" t="str">
         <x:v>V49</x:v>
       </x:c>
@@ -3392,7 +3447,7 @@
         <x:v>Practice</x:v>
       </x:c>
       <x:c r="G54" s="6" t="str">
-        <x:v>Gameplay / UX / assignment pending</x:v>
+        <x:v>Gameplay / UX</x:v>
       </x:c>
       <x:c r="H54" s="6" t="str">
         <x:v>V25, V41, V45</x:v>
@@ -3404,7 +3459,7 @@
         <x:v>A new player can learn nock/draw, cancel, reload, shield, Blink, shard step, pickups and quiver in either handedness, then enter a short scored encounter. Record completion, confusion and fatigue.</x:v>
       </x:c>
       <x:c r="K54" s="6" t="str">
-        <x:v>Ten playable lessons now verify actual outcomes, with device-specific hints and a spatial Quest coach. Skips are recorded separately. Software-only: first-user confusion, reversed-hand ergonomics and fatigue remain to be measured. Returning Bell replaces the default fresh opening; all guided First Bell lessons remain explicitly available. Physical onboarding and newcomer study remain open. Goldwind adds an opt-in physical bow preset; exact model, native input and publication outcomes belong in its versioned evidence receipt. Classic/crossbow and Xbox remain. Real-device ergonomics and human acceptance are not closed.</x:v>
+        <x:v>Pilgrimage 0.17.0: New expeditions enter Pilgrimage by default with an explicit two-signal objective, direct Goldwind controls and a protected arrival. First Bell lessons and the authored Returning Bell remain selectable; human first-session understanding is not established. Earlier implementation evidence remains in the referenced release notes. Exact accepted revisions belong in publication receipts; hardware and human gates remain separate.</x:v>
       </x:c>
       <x:c r="L54" s="6" t="str">
         <x:v>first-bell.js
@@ -3414,16 +3469,22 @@
 goldwind-model.js
 goldwind-xr.js
 tests/goldwind.test.cjs
-tests/goldwind-browser.py</x:v>
+tests/goldwind-browser.py
+PILGRIMAGE.md
+pilgrimage-model.js
+pilgrimage-view.js
+tests/pilgrimage.test.cjs
+tests/pilgrimage-driver.cjs
+tests/pilgrimage-browser.py</x:v>
       </x:c>
       <x:c r="M54" s="6" t="str">
-        <x:v>0.16.0 Goldwind</x:v>
+        <x:v>0.17.0 Pilgrimage</x:v>
       </x:c>
       <x:c r="N54" s="6" t="str">
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/first-bell.js</x:v>
       </x:c>
     </x:row>
-    <x:row r="55" ht="124" customHeight="1">
+    <x:row r="55" ht="190" customHeight="1">
       <x:c r="A55" s="6" t="str">
         <x:v>V50</x:v>
       </x:c>
@@ -3443,7 +3504,7 @@
         <x:v>Combat</x:v>
       </x:c>
       <x:c r="G55" s="6" t="str">
-        <x:v>Gameplay / assignment pending</x:v>
+        <x:v>Gameplay</x:v>
       </x:c>
       <x:c r="H55" s="6" t="str">
         <x:v>V13, V40, V43</x:v>
@@ -3455,15 +3516,21 @@
         <x:v>Coordinate telegraphed melee/ranged attacks, limit unavoidable overlap and offscreen attacks, preserve escape routes and add recovery beats. Replay fixed-seed stress encounters.</x:v>
       </x:c>
       <x:c r="K55" s="6" t="str">
-        <x:v>The optional Oath coordinates three staged encounters with front-hemisphere initiation, bolt/windup budgets and recovery supplies. The original Endless mode is unchanged. Broad seed/human difficulty evaluation remains open. Returning Bell deliberately places five retained defenders along different approaches; it does not claim a new global director or patrol system.</x:v>
+        <x:v>Pilgrimage 0.17.0: Six purposeful role slots per chapter place a court volley, gallery angle and ground pressure in each module. Roster selection is deterministic and independent of geometry. Navigation limits are retained honestly; no new adaptive director or enemy climbing is claimed. Earlier implementation evidence remains in the referenced release notes. Exact accepted revisions belong in publication receipts; hardware and human gates remain separate.</x:v>
       </x:c>
       <x:c r="L55" s="6" t="str">
         <x:v>oath-model.js
 tests/oath.test.cjs
-tests/first-bell-browser.py</x:v>
+tests/first-bell-browser.py
+PILGRIMAGE.md
+pilgrimage-model.js
+pilgrimage-view.js
+tests/pilgrimage.test.cjs
+tests/pilgrimage-driver.cjs
+tests/pilgrimage-browser.py</x:v>
       </x:c>
       <x:c r="M55" s="6" t="str">
-        <x:v>0.10.0 First Bell</x:v>
+        <x:v>0.17.0 Pilgrimage</x:v>
       </x:c>
       <x:c r="N55" s="6" t="str">
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/oath-model.js</x:v>
@@ -3489,7 +3556,7 @@
         <x:v>Combat</x:v>
       </x:c>
       <x:c r="G56" s="6" t="str">
-        <x:v>Gameplay / assignment pending</x:v>
+        <x:v>Gameplay</x:v>
       </x:c>
       <x:c r="H56" s="6" t="str">
         <x:v>V50, V18, V04</x:v>
@@ -3516,7 +3583,7 @@
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/oath-model.js</x:v>
       </x:c>
     </x:row>
-    <x:row r="57" ht="162" customHeight="1">
+    <x:row r="57" ht="190" customHeight="1">
       <x:c r="A57" s="6" t="str">
         <x:v>V52</x:v>
       </x:c>
@@ -3536,7 +3603,7 @@
         <x:v>World</x:v>
       </x:c>
       <x:c r="G57" s="6" t="str">
-        <x:v>Level design / assignment pending</x:v>
+        <x:v>Level design</x:v>
       </x:c>
       <x:c r="H57" s="6" t="str">
         <x:v>V39, V34</x:v>
@@ -3548,7 +3615,7 @@
         <x:v>One polished 20-30 minute target route mixes safe introduction, alternate approach, escalating encounter, discovery and boss payoff. Validate every traversal connector and recovery path. Duration is a design target, not measured content. Preserve multi-level gothic sightlines and multiple approaches. Plan selective water-adjacent discoveries with purpose; the present water layer does not create new navigable rooms.</x:v>
       </x:c>
       <x:c r="K57" s="6" t="str">
-        <x:v>Open Line refines the existing seven-place chapter instead of expanding it. A new versioned central stair shares the screen's cover/shot tradeoff with a repositioned existing watcher. Ordinary arrows can lift the brass release; the gallery still reverses it. A learned signal shot can complete without entering the tower. Model and controller-driven route comparisons record actual distance, simulation time, health and shots; human comprehension, enjoyment and the original finished-slice gate remain open.</x:v>
+        <x:v>Pilgrimage 0.17.0: Two chapter families assemble authored encounter modules with distinct direct, gallery and service routes. The reversible shutter couples movement to exposure; an ordinary shot can lift its release, and relay shots from below permit legitimate alternate completion. Body-clearance samples, actual movement, projectile and recovery tests are retained. Earlier implementation evidence remains in the referenced release notes. Exact accepted revisions belong in publication receipts; hardware and human gates remain separate.</x:v>
       </x:c>
       <x:c r="L57" s="6" t="str">
         <x:v>oath-model.js
@@ -3564,10 +3631,16 @@
 OPEN-LINE.md
 returning-bell-lanes.js
 tests/open-line.test.cjs
-tests/open-line-browser.py</x:v>
+tests/open-line-browser.py
+PILGRIMAGE.md
+pilgrimage-model.js
+pilgrimage-view.js
+tests/pilgrimage.test.cjs
+tests/pilgrimage-driver.cjs
+tests/pilgrimage-browser.py</x:v>
       </x:c>
       <x:c r="M57" s="6" t="str">
-        <x:v>0.15.0 Open Line</x:v>
+        <x:v>0.17.0 Pilgrimage</x:v>
       </x:c>
       <x:c r="N57" s="6" t="str">
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/oath-model.js</x:v>
@@ -3593,7 +3666,7 @@
         <x:v>Progression</x:v>
       </x:c>
       <x:c r="G58" s="6" t="str">
-        <x:v>Engineering / assignment pending</x:v>
+        <x:v>Engineering</x:v>
       </x:c>
       <x:c r="H58" s="6" t="str">
         <x:v>V46, V51</x:v>
@@ -3658,7 +3731,7 @@
         <x:v>0.13.0</x:v>
       </x:c>
       <x:c r="N59" s="6" t="str">
-        <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/CONTINUATION-AUDIT.md</x:v>
+        <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/dominion-art.js</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="124" customHeight="1">
@@ -3681,7 +3754,7 @@
         <x:v>Art</x:v>
       </x:c>
       <x:c r="G60" s="6" t="str">
-        <x:v>Technical art / assignment pending</x:v>
+        <x:v>Technical art</x:v>
       </x:c>
       <x:c r="H60" s="6" t="str">
         <x:v>V54</x:v>
@@ -3701,7 +3774,7 @@
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
       </x:c>
     </x:row>
-    <x:row r="61" ht="124" customHeight="1">
+    <x:row r="61" ht="190" customHeight="1">
       <x:c r="A61" s="6" t="str">
         <x:v>V56</x:v>
       </x:c>
@@ -3721,7 +3794,7 @@
         <x:v>World</x:v>
       </x:c>
       <x:c r="G61" s="6" t="str">
-        <x:v>Level design / assignment pending</x:v>
+        <x:v>Level design</x:v>
       </x:c>
       <x:c r="H61" s="6" t="str">
         <x:v>V52, V54</x:v>
@@ -3733,15 +3806,24 @@
         <x:v>Complete coherent crypt, storm roof and luminous sanctuary kits with different navigation, encounter opportunities, materials and sonic palettes. Validate seed combinations and repeated transitions.</x:v>
       </x:c>
       <x:c r="K61" s="6" t="str">
-        <x:v>Not closed; no completion credit without gate evidence.</x:v>
-      </x:c>
-      <x:c r="L61" s="6" t="str"/>
-      <x:c r="M61" s="6" t="str"/>
+        <x:v>Pilgrimage 0.17.0: Two initial graybox-first spatial identities exist, not three completed production biome kits. Causeway exposure contrasts with Archive ceilings and interrupted sightlines; polished bespoke assets, audio and a third biome remain open. Earlier implementation evidence remains in the referenced release notes. Exact accepted revisions belong in publication receipts; hardware and human gates remain separate.</x:v>
+      </x:c>
+      <x:c r="L61" s="6" t="str">
+        <x:v>PILGRIMAGE.md
+pilgrimage-model.js
+pilgrimage-view.js
+tests/pilgrimage.test.cjs
+tests/pilgrimage-driver.cjs
+tests/pilgrimage-browser.py</x:v>
+      </x:c>
+      <x:c r="M61" s="6" t="str">
+        <x:v>0.17.0 Pilgrimage</x:v>
+      </x:c>
       <x:c r="N61" s="6" t="str">
-        <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="62" ht="124" customHeight="1">
+        <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/PILGRIMAGE.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="62" ht="190" customHeight="1">
       <x:c r="A62" s="6" t="str">
         <x:v>V57</x:v>
       </x:c>
@@ -3761,7 +3843,7 @@
         <x:v>Presentation</x:v>
       </x:c>
       <x:c r="G62" s="6" t="str">
-        <x:v>Art / audio / assignment pending</x:v>
+        <x:v>Art / audio</x:v>
       </x:c>
       <x:c r="H62" s="6" t="str">
         <x:v>V52, V56</x:v>
@@ -3773,7 +3855,7 @@
         <x:v>Public-only lore, landmarks and discoveries connect the world; skippable/accessible presentation; no private story content enters this repository without permission.</x:v>
       </x:c>
       <x:c r="K62" s="6" t="str">
-        <x:v>Open Line links a visible brass release and cable to the actual moving screens, labels the exposed short stair, and preserves the recognizable refuge gate. Functional cues express speed/exposure versus observation/control. Recognition and environmental-story understanding require unfamiliar-player observation; no human narrative rating is claimed.</x:v>
+        <x:v>Pilgrimage 0.17.0: Functional signal-road and reading/service circulation explain relays, shutters and return latches. Familiar refuge markers are seen through the closed gate before its service-side opening. Narrative content is original and public-only; human recognition is not inferred from screenshots. Earlier implementation evidence remains in the referenced release notes. Exact accepted revisions belong in publication receipts; hardware and human gates remain separate.</x:v>
       </x:c>
       <x:c r="L62" s="6" t="str">
         <x:v>returning-bell-model.js
@@ -3782,13 +3864,19 @@
 OPEN-LINE.md
 returning-bell-lanes.js
 tests/open-line.test.cjs
-tests/open-line-browser.py</x:v>
+tests/open-line-browser.py
+PILGRIMAGE.md
+pilgrimage-model.js
+pilgrimage-view.js
+tests/pilgrimage.test.cjs
+tests/pilgrimage-driver.cjs
+tests/pilgrimage-browser.py</x:v>
       </x:c>
       <x:c r="M62" s="6" t="str">
-        <x:v>0.15.0 Open Line</x:v>
+        <x:v>0.17.0 Pilgrimage</x:v>
       </x:c>
       <x:c r="N62" s="6" t="str">
-        <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
+        <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/returning-bell-model.js</x:v>
       </x:c>
     </x:row>
     <x:row r="63" ht="162" customHeight="1">
@@ -3811,7 +3899,7 @@
         <x:v>Presentation</x:v>
       </x:c>
       <x:c r="G63" s="6" t="str">
-        <x:v>Art / audio / assignment pending</x:v>
+        <x:v>Art / audio</x:v>
       </x:c>
       <x:c r="H63" s="6" t="str">
         <x:v>V43, V44, V50</x:v>
@@ -3855,7 +3943,7 @@
         <x:v>Hardware</x:v>
       </x:c>
       <x:c r="G64" s="6" t="str">
-        <x:v>Device QA / assignment pending</x:v>
+        <x:v>Device QA</x:v>
       </x:c>
       <x:c r="H64" s="6" t="str">
         <x:v>V38, V54</x:v>
@@ -3895,7 +3983,7 @@
         <x:v>Foundation</x:v>
       </x:c>
       <x:c r="G65" s="6" t="str">
-        <x:v>Engineering / assignment pending</x:v>
+        <x:v>Engineering</x:v>
       </x:c>
       <x:c r="H65" s="6" t="str">
         <x:v>V59</x:v>
@@ -3956,7 +4044,7 @@
       </x:c>
       <x:c r="M66" s="6" t="str"/>
       <x:c r="N66" s="6" t="str">
-        <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/CONTINUATION-AUDIT.md</x:v>
+        <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/dominion-controls.js</x:v>
       </x:c>
     </x:row>
     <x:row r="67" ht="124" customHeight="1">
@@ -3979,7 +4067,7 @@
         <x:v>Hardware</x:v>
       </x:c>
       <x:c r="G67" s="6" t="str">
-        <x:v>Device QA / assignment pending</x:v>
+        <x:v>Device QA</x:v>
       </x:c>
       <x:c r="H67" s="6" t="str">
         <x:v>V15, V41, V61</x:v>
@@ -4019,7 +4107,7 @@
         <x:v>Comfort</x:v>
       </x:c>
       <x:c r="G68" s="6" t="str">
-        <x:v>UX / accessibility / assignment pending</x:v>
+        <x:v>UX / accessibility</x:v>
       </x:c>
       <x:c r="H68" s="6" t="str">
         <x:v>V44, V55</x:v>
@@ -4061,7 +4149,7 @@
         <x:v>Testing</x:v>
       </x:c>
       <x:c r="G69" s="6" t="str">
-        <x:v>QA / play research / assignment pending</x:v>
+        <x:v>QA / play research</x:v>
       </x:c>
       <x:c r="H69" s="6" t="str">
         <x:v>V49, V51, V52</x:v>
@@ -4081,7 +4169,7 @@
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
       </x:c>
     </x:row>
-    <x:row r="70" ht="195" customHeight="1">
+    <x:row r="70" ht="190" customHeight="1">
       <x:c r="A70" s="6" t="str">
         <x:v>V65</x:v>
       </x:c>
@@ -4101,7 +4189,7 @@
         <x:v>Progression</x:v>
       </x:c>
       <x:c r="G70" s="6" t="str">
-        <x:v>Engineering / assignment pending</x:v>
+        <x:v>Engineering</x:v>
       </x:c>
       <x:c r="H70" s="6" t="str">
         <x:v>V47</x:v>
@@ -4113,7 +4201,7 @@
         <x:v>Keep fixtures for old supported generator/schema versions, offer explicit local backup/restore and verify interrupted writes, browser quota and update migration. Never silently reset incompatible saves. Any future discrete-hit-point conversion must specify health/healing balance and tested checkpoint migration; retain current health and profiles in presentation-only releases.</x:v>
       </x:c>
       <x:c r="K70" s="6" t="str">
-        <x:v>Legacy hollow-dominions-1 and returning-bell-1 fixtures remain. Open Line adds returning-bell-2 and captures/restores the actual layout identity; mechanism geometry is rebuilt before supported-position checks, including a player saved inside the raised-screen crossing. This compatibility work does not complete export, backup, storage eviction or general migration tooling. Goldwind adds an opt-in physical bow preset; exact model, native input and publication outcomes belong in its versioned evidence receipt. Classic/crossbow and Xbox remain. Real-device ergonomics and human acceptance are not closed.</x:v>
+        <x:v>Pilgrimage 0.17.0: New layouts use lantern-causeway-1 and ashen-archive-1 without changing hollow-dominions-1 or either Returning Bell ID. Stage, tier and signature are validated; mechanism geometry is rebuilt before checkpoint collision checks. General export/backup and physical storage-failure acceptance remain open. Earlier implementation evidence remains in the referenced release notes. Exact accepted revisions belong in publication receipts; hardware and human gates remain separate.</x:v>
       </x:c>
       <x:c r="L70" s="6" t="str">
         <x:v>OPEN-LINE.md
@@ -4124,16 +4212,22 @@
 goldwind-model.js
 goldwind-xr.js
 tests/goldwind.test.cjs
-tests/goldwind-browser.py</x:v>
+tests/goldwind-browser.py
+PILGRIMAGE.md
+pilgrimage-model.js
+pilgrimage-view.js
+tests/pilgrimage.test.cjs
+tests/pilgrimage-driver.cjs
+tests/pilgrimage-browser.py</x:v>
       </x:c>
       <x:c r="M70" s="6" t="str">
-        <x:v>0.16.0 Goldwind</x:v>
+        <x:v>0.17.0 Pilgrimage</x:v>
       </x:c>
       <x:c r="N70" s="6" t="str">
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/OPEN-LINE.md</x:v>
       </x:c>
     </x:row>
-    <x:row r="71" ht="176" customHeight="1">
+    <x:row r="71" ht="190" customHeight="1">
       <x:c r="A71" s="6" t="str">
         <x:v>V66</x:v>
       </x:c>
@@ -4153,7 +4247,7 @@
         <x:v>Testing</x:v>
       </x:c>
       <x:c r="G71" s="6" t="str">
-        <x:v>QA / play research / assignment pending</x:v>
+        <x:v>QA / play research</x:v>
       </x:c>
       <x:c r="H71" s="6" t="str">
         <x:v>V50, V60, V65</x:v>
@@ -4165,12 +4259,20 @@
         <x:v>Run at least 1000 proposed seed/depth fixtures and 50 lifecycle transitions, tracking unreachable rewards, spawning collisions, NaNs, leaks and progress duplication. Publish failures and seed repros. Add dedicated Tidelight tests for pool placement across depth/seed, standing on high walks above water, actual arrow-water crossings, paused/reduced-effects motion, sector clock resets, AR return and old-save continuation.</x:v>
       </x:c>
       <x:c r="K71" s="6" t="str">
-        <x:v>Not closed; no completion credit without gate evidence.</x:v>
+        <x:v>Pilgrimage 0.17.0: The added model suite samples 96 chapter/seed combinations across three tier snapshots, both handed module orientations and all four tile families. It also exercises real movement, signal shots, upper Blink landings and saved open gates. Sampling is not a proof of every possible play experience or a complete long-session soak. Earlier implementation evidence remains in the referenced release notes. Exact accepted revisions belong in publication receipts; hardware and human gates remain separate.</x:v>
       </x:c>
       <x:c r="L71" s="6" t="str">
-        <x:v>CONTINUATION-AUDIT.md</x:v>
-      </x:c>
-      <x:c r="M71" s="6" t="str"/>
+        <x:v>CONTINUATION-AUDIT.md
+PILGRIMAGE.md
+pilgrimage-model.js
+pilgrimage-view.js
+tests/pilgrimage.test.cjs
+tests/pilgrimage-driver.cjs
+tests/pilgrimage-browser.py</x:v>
+      </x:c>
+      <x:c r="M71" s="6" t="str">
+        <x:v>0.17.0 Pilgrimage</x:v>
+      </x:c>
       <x:c r="N71" s="6" t="str">
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/CONTINUATION-AUDIT.md</x:v>
       </x:c>
@@ -4195,7 +4297,7 @@
         <x:v>Testing</x:v>
       </x:c>
       <x:c r="G72" s="6" t="str">
-        <x:v>QA / play research / assignment pending</x:v>
+        <x:v>QA / play research</x:v>
       </x:c>
       <x:c r="H72" s="6" t="str">
         <x:v>V62, V63, V66</x:v>
@@ -4215,7 +4317,7 @@
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
       </x:c>
     </x:row>
-    <x:row r="73" ht="195" customHeight="1">
+    <x:row r="73" ht="190" customHeight="1">
       <x:c r="A73" s="6" t="str">
         <x:v>V68</x:v>
       </x:c>
@@ -4235,7 +4337,7 @@
         <x:v>Foundation</x:v>
       </x:c>
       <x:c r="G73" s="6" t="str">
-        <x:v>Engineering / assignment pending</x:v>
+        <x:v>Engineering</x:v>
       </x:c>
       <x:c r="H73" s="6" t="str">
         <x:v>V48, V65</x:v>
@@ -4247,7 +4349,7 @@
         <x:v>For every finished upgrade, test the actual scoped source, commit and merge without overwriting sibling games, verify GitHub Pages deployment plus public runtime/asset/plan/workbook bytes, then launch the public game. Separate source, test, deployment, hardware and human evidence. Retry transient GitHub faults with backoff; inspect failed jobs instead of polling an unchanged failure list. Preserve explicit rollback and save-compatibility notes.</x:v>
       </x:c>
       <x:c r="K73" s="6" t="str">
-        <x:v>Open Line retains exact-source model/workbook checks, four controller-driven route comparisons, full first-person VR/AR/hand/save regression and separate public-byte/launch verification. Preserve unsuccessful receipts and separate model, rendered software, physical-device and human evidence. Public success is recorded only in the matching publication receipt. Goldwind adds an opt-in physical bow preset; exact model, native input and publication outcomes belong in its versioned evidence receipt. Classic/crossbow and Xbox remain. Real-device ergonomics and human acceptance are not closed.</x:v>
+        <x:v>Pilgrimage 0.17.0: Candidate and public acceptance distinguish exact production hashes, model checks, input-driven rendered journeys and hardware/human gates. Failed graybox and transport/test traces are recorded, not counted as successful release evidence. Earlier implementation evidence remains in the referenced release notes. Exact accepted revisions belong in publication receipts; hardware and human gates remain separate.</x:v>
       </x:c>
       <x:c r="L73" s="6" t="str">
         <x:v>tests/verify-live.py
@@ -4263,10 +4365,16 @@
 goldwind-model.js
 goldwind-xr.js
 tests/goldwind.test.cjs
-tests/goldwind-browser.py</x:v>
+tests/goldwind-browser.py
+PILGRIMAGE.md
+pilgrimage-model.js
+pilgrimage-view.js
+tests/pilgrimage.test.cjs
+tests/pilgrimage-driver.cjs
+tests/pilgrimage-browser.py</x:v>
       </x:c>
       <x:c r="M73" s="6" t="str">
-        <x:v>0.16.0 Goldwind</x:v>
+        <x:v>0.17.0 Pilgrimage</x:v>
       </x:c>
       <x:c r="N73" s="6" t="str">
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/tests/verify-live.py</x:v>
@@ -4292,7 +4400,7 @@
         <x:v>Art</x:v>
       </x:c>
       <x:c r="G74" s="6" t="str">
-        <x:v>Technical art / assignment pending</x:v>
+        <x:v>Technical art</x:v>
       </x:c>
       <x:c r="H74" s="6" t="str">
         <x:v>V54, V56, V57</x:v>
@@ -4312,7 +4420,7 @@
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
       </x:c>
     </x:row>
-    <x:row r="75" ht="124" customHeight="1">
+    <x:row r="75" ht="190" customHeight="1">
       <x:c r="A75" s="6" t="str">
         <x:v>V70</x:v>
       </x:c>
@@ -4320,7 +4428,7 @@
         <x:v>Content-complete campaign and replay challenge tuning</x:v>
       </x:c>
       <x:c r="C75" s="6" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Partial</x:v>
       </x:c>
       <x:c r="D75" s="6" t="str">
         <x:v>P1</x:v>
@@ -4332,7 +4440,7 @@
         <x:v>World</x:v>
       </x:c>
       <x:c r="G75" s="6" t="str">
-        <x:v>Level design / assignment pending</x:v>
+        <x:v>Level design</x:v>
       </x:c>
       <x:c r="H75" s="6" t="str">
         <x:v>V53, V56, V64</x:v>
@@ -4344,12 +4452,21 @@
         <x:v>Complete the agreed campaign scope, enemy/loot combinations and endgame variations with no placeholder gates. Measure real play length and review progression fatigue before promising duration.</x:v>
       </x:c>
       <x:c r="K75" s="6" t="str">
-        <x:v>Not closed; no completion credit without gate evidence.</x:v>
-      </x:c>
-      <x:c r="L75" s="6" t="str"/>
-      <x:c r="M75" s="6" t="str"/>
+        <x:v>Pilgrimage 0.17.0: The new default campaign route comprises Lantern Causeway then Ashen Archive, with an ordinary blessing between them and explicit continuation to retained Endless after the second. This is an initial two-chapter pipeline, not a content-complete final campaign or new boss suite. Earlier implementation evidence remains in the referenced release notes. Exact accepted revisions belong in publication receipts; hardware and human gates remain separate.</x:v>
+      </x:c>
+      <x:c r="L75" s="6" t="str">
+        <x:v>PILGRIMAGE.md
+pilgrimage-model.js
+pilgrimage-view.js
+tests/pilgrimage.test.cjs
+tests/pilgrimage-driver.cjs
+tests/pilgrimage-browser.py</x:v>
+      </x:c>
+      <x:c r="M75" s="6" t="str">
+        <x:v>0.17.0 Pilgrimage</x:v>
+      </x:c>
       <x:c r="N75" s="6" t="str">
-        <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
+        <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/PILGRIMAGE.md</x:v>
       </x:c>
     </x:row>
     <x:row r="76" ht="124" customHeight="1">
@@ -4372,7 +4489,7 @@
         <x:v>Testing</x:v>
       </x:c>
       <x:c r="G76" s="6" t="str">
-        <x:v>QA / play research / assignment pending</x:v>
+        <x:v>QA / play research</x:v>
       </x:c>
       <x:c r="H76" s="6" t="str">
         <x:v>V66, V67, V68, V70</x:v>
@@ -4412,7 +4529,7 @@
         <x:v>Online</x:v>
       </x:c>
       <x:c r="G77" s="6" t="str">
-        <x:v>Online engineering / assignment pending</x:v>
+        <x:v>Online engineering</x:v>
       </x:c>
       <x:c r="H77" s="6" t="str">
         <x:v>V17, V71</x:v>
@@ -4452,7 +4569,7 @@
         <x:v>Testing</x:v>
       </x:c>
       <x:c r="G78" s="6" t="str">
-        <x:v>QA / play research / assignment pending</x:v>
+        <x:v>QA / play research</x:v>
       </x:c>
       <x:c r="H78" s="6" t="str">
         <x:v>V59, V62, V64, V69, V71</x:v>
@@ -4492,7 +4609,7 @@
         <x:v>Foundation</x:v>
       </x:c>
       <x:c r="G79" s="6" t="str">
-        <x:v>Engineering / assignment pending</x:v>
+        <x:v>Engineering</x:v>
       </x:c>
       <x:c r="H79" s="6" t="str">
         <x:v>V15, V48</x:v>
@@ -4536,7 +4653,7 @@
         <x:v>Testing</x:v>
       </x:c>
       <x:c r="G80" s="6" t="str">
-        <x:v>QA / play research / assignment pending</x:v>
+        <x:v>QA / play research</x:v>
       </x:c>
       <x:c r="H80" s="6" t="str">
         <x:v>V47</x:v>
@@ -4556,7 +4673,7 @@
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/roadmap.json</x:v>
       </x:c>
     </x:row>
-    <x:row r="81" ht="124" customHeight="1">
+    <x:row r="81" ht="190" customHeight="1">
       <x:c r="A81" s="6" t="str">
         <x:v>V76</x:v>
       </x:c>
@@ -4576,7 +4693,7 @@
         <x:v>Combat</x:v>
       </x:c>
       <x:c r="G81" s="6" t="str">
-        <x:v>Gameplay / assignment pending</x:v>
+        <x:v>Gameplay</x:v>
       </x:c>
       <x:c r="H81" s="6" t="str">
         <x:v>V49, V50, V51, V52</x:v>
@@ -4588,7 +4705,7 @@
         <x:v>Publish one complete integrated slice, including onboarding, traversal, encounter pacing, boss payoff and saved continuation; collect human feedback before producing additional bosses.</x:v>
       </x:c>
       <x:c r="K81" s="6" t="str">
-        <x:v>The authored opening retains the ordinary sector reward once and explicitly continues into Endless after its blessing. Open Line strengthens route purpose and a knowledge-based signal approach without adding a new boss or second authored chapter. Existing First Bell/Oath remain. External first/replay play and physical-device acceptance remain open.</x:v>
+        <x:v>Pilgrimage 0.17.0: First Bell and Bellkeeper Oath remain separate. Pilgrimage adds two objective-driven chapter endings, not a new boss. One-time sector rewards and progression into retained Endless are tested without requiring every defender to die. Earlier implementation evidence remains in the referenced release notes. Exact accepted revisions belong in publication receipts; hardware and human gates remain separate.</x:v>
       </x:c>
       <x:c r="L81" s="6" t="str">
         <x:v>FIRST-BELL.md
@@ -4597,10 +4714,16 @@
 OPEN-LINE.md
 returning-bell-lanes.js
 tests/open-line.test.cjs
-tests/open-line-browser.py</x:v>
+tests/open-line-browser.py
+PILGRIMAGE.md
+pilgrimage-model.js
+pilgrimage-view.js
+tests/pilgrimage.test.cjs
+tests/pilgrimage-driver.cjs
+tests/pilgrimage-browser.py</x:v>
       </x:c>
       <x:c r="M81" s="6" t="str">
-        <x:v>0.15.0 Open Line</x:v>
+        <x:v>0.17.0 Pilgrimage</x:v>
       </x:c>
       <x:c r="N81" s="6" t="str">
         <x:v>https://github.com/v5ma/v5ma.github.io/blob/master/vesperfall/FIRST-BELL.md</x:v>
@@ -4659,7 +4782,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R958360007258475a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbda451baef6246fa"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4961,7 +5084,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb645a74757f84a3a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdc8934ebf5ad463e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5393,7 +5516,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R037fb1aaadb14064"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R19d41ce954a046ed"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5739,7 +5862,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R46a5c22e2a4c4f25"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0d0f6dedd2864d0c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6157,7 +6280,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R732fc0fbe20745ae"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0858fbb1c5fe45d2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>